<commit_message>
Added logo for Android
</commit_message>
<xml_diff>
--- a/data/content.xlsx
+++ b/data/content.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Markus/Documents/Arbeit/Inschriftenschluessel/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FDB85DE-9336-7C44-B2C0-2763281AA6EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD5FEAD4-54F3-3C43-9DD8-1E2DF8CDC7E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4720" yWindow="1320" windowWidth="20180" windowHeight="16240" activeTab="4" xr2:uid="{F025A444-F8B0-5C41-A37E-BEE791B22240}"/>
+    <workbookView xWindow="-21400" yWindow="500" windowWidth="20180" windowHeight="16240" activeTab="4" xr2:uid="{F025A444-F8B0-5C41-A37E-BEE791B22240}"/>
   </bookViews>
   <sheets>
     <sheet name="pages" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
Table header hyphenation fix
</commit_message>
<xml_diff>
--- a/data/content.xlsx
+++ b/data/content.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Markus/Documents/Arbeit/Inschriftenschluessel/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD5FEAD4-54F3-3C43-9DD8-1E2DF8CDC7E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FF0187C-B475-4E4F-9728-6B06706DC459}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-21400" yWindow="500" windowWidth="20180" windowHeight="16240" activeTab="4" xr2:uid="{F025A444-F8B0-5C41-A37E-BEE791B22240}"/>
+    <workbookView xWindow="-21400" yWindow="500" windowWidth="20180" windowHeight="16240" activeTab="2" xr2:uid="{F025A444-F8B0-5C41-A37E-BEE791B22240}"/>
   </bookViews>
   <sheets>
     <sheet name="pages" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
formula pages referencing fix
</commit_message>
<xml_diff>
--- a/data/content.xlsx
+++ b/data/content.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Markus/Documents/Arbeit/Inschriftenschluessel/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{572965D0-70B1-7D4C-B525-65FF37DF30BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A1FC0BD-37A7-AF45-9DAE-662FD4FCA442}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6860" yWindow="1020" windowWidth="27740" windowHeight="19300" activeTab="5" xr2:uid="{F025A444-F8B0-5C41-A37E-BEE791B22240}"/>
+    <workbookView xWindow="5940" yWindow="500" windowWidth="27740" windowHeight="19300" activeTab="1" xr2:uid="{F025A444-F8B0-5C41-A37E-BEE791B22240}"/>
   </bookViews>
   <sheets>
     <sheet name="pages" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5472" uniqueCount="1268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5475" uniqueCount="1270">
   <si>
     <t>page_id</t>
   </si>
@@ -3746,9 +3746,6 @@
     <t>Worte zu sprechen durch [Gottheit] / [König] / [Person] NN: Ich habe dir gegeben [Gaben], die bei mir sind.</t>
   </si>
   <si>
-    <t>Inschrift</t>
-  </si>
-  <si>
     <t>(AR; MR)</t>
   </si>
   <si>
@@ -3846,6 +3843,15 @@
   </si>
   <si>
     <t>(AR; Sp.)</t>
+  </si>
+  <si>
+    <t>[Szenentitel]</t>
+  </si>
+  <si>
+    <t>[Rückenschutzformel]</t>
+  </si>
+  <si>
+    <t>[Beziehung]</t>
   </si>
 </sst>
 </file>
@@ -3879,7 +3885,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3928,6 +3934,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -3941,7 +3953,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -4005,6 +4017,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -4489,20 +4502,20 @@
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+    <row r="9" spans="1:6" s="31" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A9" s="31" t="s">
         <v>67</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="31" t="s">
         <v>11</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="31" t="s">
         <v>1182</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="31" t="s">
         <v>74</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="31">
         <v>70</v>
       </c>
     </row>
@@ -4632,7 +4645,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{244ECE21-4B85-B642-91D8-6A98EB98549E}">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9.5" bestFit="1" customWidth="1"/>
@@ -4737,6 +4750,20 @@
       </c>
       <c r="D7" s="21">
         <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" s="31" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A8" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="31" t="s">
+        <v>1182</v>
+      </c>
+      <c r="C8" s="31" t="s">
+        <v>67</v>
+      </c>
+      <c r="D8" s="31">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -4751,7 +4778,7 @@
   <cols>
     <col min="1" max="1" width="14.83203125" style="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="12.1640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15" style="4" customWidth="1"/>
     <col min="4" max="4" width="26" style="4" customWidth="1"/>
     <col min="5" max="5" width="23.83203125" style="4" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="2.6640625" style="4" bestFit="1" customWidth="1"/>
@@ -5175,8 +5202,8 @@
       <c r="B31" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="C31" s="22" t="s">
-        <v>1234</v>
+      <c r="C31" s="21" t="s">
+        <v>563</v>
       </c>
       <c r="D31" s="22" t="s">
         <v>570</v>
@@ -6384,7 +6411,7 @@
         <v>45</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>1237</v>
+        <v>1236</v>
       </c>
       <c r="N14" s="9" t="s">
         <v>92</v>
@@ -6431,7 +6458,7 @@
         <v>45</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>1238</v>
+        <v>1237</v>
       </c>
       <c r="N16" s="9" t="s">
         <v>92</v>
@@ -6478,7 +6505,7 @@
         <v>45</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>1239</v>
+        <v>1238</v>
       </c>
       <c r="N18" s="9" t="s">
         <v>92</v>
@@ -6525,7 +6552,7 @@
         <v>45</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>1237</v>
+        <v>1236</v>
       </c>
       <c r="N20" s="9" t="s">
         <v>92</v>
@@ -6572,7 +6599,7 @@
         <v>45</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>1237</v>
+        <v>1236</v>
       </c>
       <c r="N22" s="9" t="s">
         <v>92</v>
@@ -6619,7 +6646,7 @@
         <v>45</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>1237</v>
+        <v>1236</v>
       </c>
       <c r="N24" s="9" t="s">
         <v>92</v>
@@ -7619,7 +7646,7 @@
         <v>45</v>
       </c>
       <c r="D68" s="12" t="s">
-        <v>1240</v>
+        <v>1239</v>
       </c>
       <c r="N68" s="12" t="s">
         <v>92</v>
@@ -7707,7 +7734,7 @@
         <v>45</v>
       </c>
       <c r="D72" s="12" t="s">
-        <v>1241</v>
+        <v>1240</v>
       </c>
       <c r="N72" s="12" t="s">
         <v>93</v>
@@ -7751,7 +7778,7 @@
         <v>45</v>
       </c>
       <c r="D74" s="12" t="s">
-        <v>1241</v>
+        <v>1240</v>
       </c>
       <c r="N74" s="12" t="s">
         <v>93</v>
@@ -7795,7 +7822,7 @@
         <v>45</v>
       </c>
       <c r="D76" s="12" t="s">
-        <v>1241</v>
+        <v>1240</v>
       </c>
       <c r="N76" s="12" t="s">
         <v>93</v>
@@ -7883,7 +7910,7 @@
         <v>45</v>
       </c>
       <c r="D80" s="12" t="s">
-        <v>1241</v>
+        <v>1240</v>
       </c>
       <c r="N80" s="12" t="s">
         <v>95</v>
@@ -8349,7 +8376,7 @@
         <v>45</v>
       </c>
       <c r="D108" s="16" t="s">
-        <v>1242</v>
+        <v>1241</v>
       </c>
       <c r="N108" s="16" t="s">
         <v>92</v>
@@ -8678,7 +8705,7 @@
         <v>45</v>
       </c>
       <c r="D123" s="18" t="s">
-        <v>1243</v>
+        <v>1242</v>
       </c>
       <c r="N123" s="18" t="s">
         <v>93</v>
@@ -8695,7 +8722,7 @@
         <v>45</v>
       </c>
       <c r="D125" s="21" t="s">
-        <v>563</v>
+        <v>1269</v>
       </c>
       <c r="N125" s="21" t="s">
         <v>90</v>
@@ -8712,7 +8739,7 @@
         <v>45</v>
       </c>
       <c r="D126" s="21" t="s">
-        <v>589</v>
+        <v>1267</v>
       </c>
       <c r="N126" s="21" t="s">
         <v>90</v>
@@ -8749,7 +8776,7 @@
         <v>45</v>
       </c>
       <c r="D128" s="21" t="s">
-        <v>569</v>
+        <v>1268</v>
       </c>
       <c r="N128" s="21" t="s">
         <v>90</v>
@@ -9290,7 +9317,7 @@
         <v>45</v>
       </c>
       <c r="D157" t="s">
-        <v>1241</v>
+        <v>1240</v>
       </c>
       <c r="N157" t="s">
         <v>92</v>
@@ -10161,13 +10188,13 @@
         <v>113</v>
       </c>
       <c r="I33" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J33" t="s">
         <v>1244</v>
       </c>
-      <c r="J33" t="s">
+      <c r="K33" t="s">
         <v>1245</v>
-      </c>
-      <c r="K33" t="s">
-        <v>1246</v>
       </c>
       <c r="L33" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D33:K33)</f>
@@ -10273,13 +10300,13 @@
         <v>113</v>
       </c>
       <c r="I39" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J39" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K39" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L39" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D39:K39)</f>
@@ -10620,13 +10647,13 @@
         <v>113</v>
       </c>
       <c r="I56" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J56" t="s">
-        <v>1248</v>
+        <v>1247</v>
       </c>
       <c r="K56" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L56" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D56:K56)</f>
@@ -10756,13 +10783,13 @@
         <v>113</v>
       </c>
       <c r="I63" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J63" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K63" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L63" t="str">
         <f t="shared" ref="L63:L65" si="10">_xlfn.TEXTJOIN("", TRUE, D63:K63)</f>
@@ -10789,13 +10816,13 @@
         <v>113</v>
       </c>
       <c r="I64" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J64" t="s">
         <v>1198</v>
       </c>
       <c r="K64" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L64" t="str">
         <f t="shared" si="10"/>
@@ -10822,13 +10849,13 @@
         <v>113</v>
       </c>
       <c r="I65" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J65" t="s">
         <v>1198</v>
       </c>
       <c r="K65" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L65" t="str">
         <f t="shared" si="10"/>
@@ -10934,13 +10961,13 @@
         <v>113</v>
       </c>
       <c r="I71" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J71" t="s">
-        <v>1235</v>
+        <v>1234</v>
       </c>
       <c r="K71" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L71" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D71:K71)</f>
@@ -10991,13 +11018,13 @@
         <v>113</v>
       </c>
       <c r="I73" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J73" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K73" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L73" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D73:K73)</f>
@@ -11103,13 +11130,13 @@
         <v>113</v>
       </c>
       <c r="I79" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J79" t="s">
         <v>1198</v>
       </c>
       <c r="K79" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L79" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D79:K79)</f>
@@ -11160,13 +11187,13 @@
         <v>113</v>
       </c>
       <c r="I81" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J81" t="s">
         <v>1198</v>
       </c>
       <c r="K81" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L81" t="str">
         <f t="shared" ref="L81:L83" si="14">_xlfn.TEXTJOIN("", TRUE, D81:K81)</f>
@@ -11193,13 +11220,13 @@
         <v>113</v>
       </c>
       <c r="I82" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J82" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K82" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L82" t="str">
         <f t="shared" si="14"/>
@@ -11226,13 +11253,13 @@
         <v>113</v>
       </c>
       <c r="I83" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J83" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K83" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L83" t="str">
         <f t="shared" si="14"/>
@@ -11316,13 +11343,13 @@
         <v>113</v>
       </c>
       <c r="I86" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J86" t="s">
         <v>1198</v>
       </c>
       <c r="K86" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L86" t="str">
         <f t="shared" ref="L86:L87" si="16">_xlfn.TEXTJOIN("", TRUE, D86:K86)</f>
@@ -11352,13 +11379,13 @@
         <v>113</v>
       </c>
       <c r="I87" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J87" t="s">
         <v>1198</v>
       </c>
       <c r="K87" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L87" t="str">
         <f t="shared" si="16"/>
@@ -11618,13 +11645,13 @@
         <v>113</v>
       </c>
       <c r="I101" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J101" t="s">
         <v>1244</v>
       </c>
-      <c r="J101" t="s">
+      <c r="K101" t="s">
         <v>1245</v>
-      </c>
-      <c r="K101" t="s">
-        <v>1246</v>
       </c>
       <c r="L101" t="str">
         <f t="shared" ref="L101:L109" si="21">_xlfn.TEXTJOIN("", TRUE, D101:K101)</f>
@@ -11651,13 +11678,13 @@
         <v>113</v>
       </c>
       <c r="I102" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J102" t="s">
         <v>1244</v>
       </c>
-      <c r="J102" t="s">
+      <c r="K102" t="s">
         <v>1245</v>
-      </c>
-      <c r="K102" t="s">
-        <v>1246</v>
       </c>
       <c r="L102" t="str">
         <f t="shared" si="21"/>
@@ -11684,13 +11711,13 @@
         <v>113</v>
       </c>
       <c r="I103" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J103" t="s">
         <v>1244</v>
       </c>
-      <c r="J103" t="s">
+      <c r="K103" t="s">
         <v>1245</v>
-      </c>
-      <c r="K103" t="s">
-        <v>1246</v>
       </c>
       <c r="L103" t="str">
         <f t="shared" si="21"/>
@@ -11717,13 +11744,13 @@
         <v>113</v>
       </c>
       <c r="I104" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J104" t="s">
-        <v>1259</v>
+        <v>1258</v>
       </c>
       <c r="K104" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L104" t="str">
         <f t="shared" si="21"/>
@@ -11750,13 +11777,13 @@
         <v>113</v>
       </c>
       <c r="I105" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J105" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K105" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L105" t="str">
         <f t="shared" si="21"/>
@@ -11783,13 +11810,13 @@
         <v>113</v>
       </c>
       <c r="I106" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J106" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K106" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L106" t="str">
         <f t="shared" si="21"/>
@@ -11816,13 +11843,13 @@
         <v>113</v>
       </c>
       <c r="I107" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J107" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K107" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L107" t="str">
         <f t="shared" si="21"/>
@@ -11849,13 +11876,13 @@
         <v>113</v>
       </c>
       <c r="I108" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J108" t="s">
-        <v>1250</v>
+        <v>1249</v>
       </c>
       <c r="K108" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L108" t="str">
         <f t="shared" si="21"/>
@@ -11882,13 +11909,13 @@
         <v>113</v>
       </c>
       <c r="I109" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J109" t="s">
-        <v>1251</v>
+        <v>1250</v>
       </c>
       <c r="K109" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L109" t="str">
         <f t="shared" si="21"/>
@@ -12071,13 +12098,13 @@
         <v>113</v>
       </c>
       <c r="I116" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J116" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K116" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L116" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D116:K116)</f>
@@ -12204,13 +12231,13 @@
         <v>113</v>
       </c>
       <c r="I123" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J123" t="s">
         <v>1198</v>
       </c>
       <c r="K123" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L123" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D123:K123)</f>
@@ -12267,13 +12294,13 @@
         <v>113</v>
       </c>
       <c r="I125" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J125" t="s">
         <v>1244</v>
       </c>
-      <c r="J125" t="s">
+      <c r="K125" t="s">
         <v>1245</v>
-      </c>
-      <c r="K125" t="s">
-        <v>1246</v>
       </c>
       <c r="L125" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D125:K125)</f>
@@ -12864,13 +12891,13 @@
         <v>113</v>
       </c>
       <c r="I166" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J166" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K166" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L166" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D166:K166)</f>
@@ -13045,13 +13072,13 @@
         <v>113</v>
       </c>
       <c r="I175" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J175" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K175" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L175" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D175:K175)</f>
@@ -13316,13 +13343,13 @@
         <v>113</v>
       </c>
       <c r="I193" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J193" t="s">
         <v>1244</v>
       </c>
-      <c r="J193" t="s">
+      <c r="K193" t="s">
         <v>1245</v>
-      </c>
-      <c r="K193" t="s">
-        <v>1246</v>
       </c>
       <c r="L193" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D193:K193)</f>
@@ -13380,13 +13407,13 @@
         <v>113</v>
       </c>
       <c r="I197" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J197" t="s">
-        <v>1252</v>
+        <v>1251</v>
       </c>
       <c r="K197" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L197" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D197:K197)</f>
@@ -13444,13 +13471,13 @@
         <v>113</v>
       </c>
       <c r="I201" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J201" t="s">
-        <v>1260</v>
+        <v>1259</v>
       </c>
       <c r="K201" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L201" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D201:K201)</f>
@@ -13712,13 +13739,13 @@
         <v>113</v>
       </c>
       <c r="I226" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J226" t="s">
         <v>1198</v>
       </c>
       <c r="K226" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L226" t="str">
         <f t="shared" ref="L226:L228" si="48">_xlfn.TEXTJOIN("", TRUE, D226:K226)</f>
@@ -13745,13 +13772,13 @@
         <v>113</v>
       </c>
       <c r="I227" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J227" t="s">
-        <v>1236</v>
+        <v>1235</v>
       </c>
       <c r="K227" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L227" t="str">
         <f t="shared" si="48"/>
@@ -13778,13 +13805,13 @@
         <v>113</v>
       </c>
       <c r="I228" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J228" t="s">
-        <v>1236</v>
+        <v>1235</v>
       </c>
       <c r="K228" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L228" t="str">
         <f t="shared" si="48"/>
@@ -14837,13 +14864,13 @@
         <v>113</v>
       </c>
       <c r="I290" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J290" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K290" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L290" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D290:K290)</f>
@@ -15764,13 +15791,13 @@
         <v>113</v>
       </c>
       <c r="I348" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J348" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K348" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L348" t="str">
         <f t="shared" ref="L348:L349" si="75">_xlfn.TEXTJOIN("", TRUE, D348:K348)</f>
@@ -15797,13 +15824,13 @@
         <v>113</v>
       </c>
       <c r="I349" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J349" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K349" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L349" t="str">
         <f t="shared" si="75"/>
@@ -16167,13 +16194,13 @@
         <v>113</v>
       </c>
       <c r="I374" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J374" t="s">
         <v>1244</v>
       </c>
-      <c r="J374" t="s">
+      <c r="K374" t="s">
         <v>1245</v>
-      </c>
-      <c r="K374" t="s">
-        <v>1246</v>
       </c>
       <c r="L374" t="str">
         <f t="shared" ref="L374:L377" si="77">_xlfn.TEXTJOIN("", TRUE, D374:K374)</f>
@@ -16200,13 +16227,13 @@
         <v>113</v>
       </c>
       <c r="I375" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J375" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K375" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L375" t="str">
         <f t="shared" si="77"/>
@@ -16233,13 +16260,13 @@
         <v>113</v>
       </c>
       <c r="I376" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J376" t="s">
         <v>1198</v>
       </c>
       <c r="K376" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L376" t="str">
         <f t="shared" si="77"/>
@@ -16266,13 +16293,13 @@
         <v>113</v>
       </c>
       <c r="I377" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J377" t="s">
         <v>1198</v>
       </c>
       <c r="K377" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L377" t="str">
         <f t="shared" si="77"/>
@@ -16478,13 +16505,13 @@
         <v>113</v>
       </c>
       <c r="I390" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J390" t="s">
         <v>1198</v>
       </c>
       <c r="K390" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L390" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D390:K390)</f>
@@ -16663,13 +16690,13 @@
         <v>113</v>
       </c>
       <c r="I401" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J401" t="s">
-        <v>1236</v>
+        <v>1235</v>
       </c>
       <c r="K401" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L401" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D401:K401)</f>
@@ -16822,13 +16849,13 @@
         <v>113</v>
       </c>
       <c r="I409" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J409" t="s">
         <v>1244</v>
       </c>
-      <c r="J409" t="s">
+      <c r="K409" t="s">
         <v>1245</v>
-      </c>
-      <c r="K409" t="s">
-        <v>1246</v>
       </c>
       <c r="L409" t="str">
         <f t="shared" ref="L409:L410" si="80">_xlfn.TEXTJOIN("", TRUE, D409:K409)</f>
@@ -16858,13 +16885,13 @@
         <v>113</v>
       </c>
       <c r="I410" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J410" t="s">
         <v>1244</v>
       </c>
-      <c r="J410" t="s">
+      <c r="K410" t="s">
         <v>1245</v>
-      </c>
-      <c r="K410" t="s">
-        <v>1246</v>
       </c>
       <c r="L410" t="str">
         <f t="shared" si="80"/>
@@ -17058,13 +17085,13 @@
         <v>113</v>
       </c>
       <c r="I421" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J421" t="s">
         <v>1198</v>
       </c>
       <c r="K421" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L421" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D421:K421)</f>
@@ -17122,13 +17149,13 @@
         <v>113</v>
       </c>
       <c r="I425" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J425" t="s">
         <v>1244</v>
       </c>
-      <c r="J425" t="s">
+      <c r="K425" t="s">
         <v>1245</v>
-      </c>
-      <c r="K425" t="s">
-        <v>1246</v>
       </c>
       <c r="L425" t="str">
         <f t="shared" ref="L425:L433" si="81">_xlfn.TEXTJOIN("", TRUE, D425:K425)</f>
@@ -17158,13 +17185,13 @@
         <v>113</v>
       </c>
       <c r="I426" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J426" t="s">
         <v>1244</v>
       </c>
-      <c r="J426" t="s">
+      <c r="K426" t="s">
         <v>1245</v>
-      </c>
-      <c r="K426" t="s">
-        <v>1246</v>
       </c>
       <c r="L426" t="str">
         <f t="shared" si="81"/>
@@ -17194,13 +17221,13 @@
         <v>113</v>
       </c>
       <c r="I427" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J427" t="s">
         <v>1244</v>
       </c>
-      <c r="J427" t="s">
+      <c r="K427" t="s">
         <v>1245</v>
-      </c>
-      <c r="K427" t="s">
-        <v>1246</v>
       </c>
       <c r="L427" t="str">
         <f t="shared" si="81"/>
@@ -17230,13 +17257,13 @@
         <v>113</v>
       </c>
       <c r="I428" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J428" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K428" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L428" t="str">
         <f t="shared" si="81"/>
@@ -17266,13 +17293,13 @@
         <v>113</v>
       </c>
       <c r="I429" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J429" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K429" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L429" t="str">
         <f t="shared" si="81"/>
@@ -17302,13 +17329,13 @@
         <v>113</v>
       </c>
       <c r="I430" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J430" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="K430" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L430" t="str">
         <f t="shared" si="81"/>
@@ -17338,13 +17365,13 @@
         <v>113</v>
       </c>
       <c r="I431" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J431" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K431" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L431" t="str">
         <f t="shared" si="81"/>
@@ -17374,13 +17401,13 @@
         <v>113</v>
       </c>
       <c r="I432" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J432" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K432" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L432" t="str">
         <f t="shared" si="81"/>
@@ -17410,13 +17437,13 @@
         <v>113</v>
       </c>
       <c r="I433" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J433" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K433" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L433" t="str">
         <f t="shared" si="81"/>
@@ -17543,13 +17570,13 @@
         <v>113</v>
       </c>
       <c r="I444" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J444" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K444" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L444" t="str">
         <f t="shared" ref="L444:L447" si="83">_xlfn.TEXTJOIN("", TRUE, D444:K444)</f>
@@ -17576,13 +17603,13 @@
         <v>113</v>
       </c>
       <c r="I445" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J445" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K445" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L445" t="str">
         <f t="shared" si="83"/>
@@ -17609,13 +17636,13 @@
         <v>113</v>
       </c>
       <c r="I446" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J446" t="s">
         <v>1198</v>
       </c>
       <c r="K446" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L446" t="str">
         <f t="shared" si="83"/>
@@ -17642,13 +17669,13 @@
         <v>113</v>
       </c>
       <c r="I447" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J447" t="s">
-        <v>1254</v>
+        <v>1253</v>
       </c>
       <c r="K447" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L447" t="str">
         <f t="shared" si="83"/>
@@ -17858,13 +17885,13 @@
         <v>113</v>
       </c>
       <c r="I461" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J461" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="K461" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L461" t="str">
         <f t="shared" ref="L461:L463" si="84">_xlfn.TEXTJOIN("", TRUE, D461:K461)</f>
@@ -17891,13 +17918,13 @@
         <v>113</v>
       </c>
       <c r="I462" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J462" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K462" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L462" t="str">
         <f t="shared" si="84"/>
@@ -17924,13 +17951,13 @@
         <v>113</v>
       </c>
       <c r="I463" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J463" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K463" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L463" t="str">
         <f t="shared" si="84"/>
@@ -18233,13 +18260,13 @@
         <v>113</v>
       </c>
       <c r="I485" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J485" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="K485" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L485" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D485:K485)</f>
@@ -18297,13 +18324,13 @@
         <v>113</v>
       </c>
       <c r="I489" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J489" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="K489" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L489" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D489:K489)</f>
@@ -18361,13 +18388,13 @@
         <v>113</v>
       </c>
       <c r="I493" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J493" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="K493" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L493" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D493:K493)</f>
@@ -18701,13 +18728,13 @@
         <v>113</v>
       </c>
       <c r="I516" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J516" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K516" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L516" t="str">
         <f t="shared" ref="L516:L522" si="86">_xlfn.TEXTJOIN("", TRUE, D516:K516)</f>
@@ -18734,13 +18761,13 @@
         <v>113</v>
       </c>
       <c r="I517" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J517" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K517" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L517" t="str">
         <f t="shared" si="86"/>
@@ -18767,13 +18794,13 @@
         <v>113</v>
       </c>
       <c r="I518" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J518" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K518" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L518" t="str">
         <f t="shared" si="86"/>
@@ -18800,13 +18827,13 @@
         <v>113</v>
       </c>
       <c r="I519" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J519" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K519" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L519" t="str">
         <f t="shared" si="86"/>
@@ -18833,13 +18860,13 @@
         <v>113</v>
       </c>
       <c r="I520" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J520" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K520" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L520" t="str">
         <f t="shared" si="86"/>
@@ -18866,13 +18893,13 @@
         <v>113</v>
       </c>
       <c r="I521" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J521" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K521" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L521" t="str">
         <f t="shared" si="86"/>
@@ -18899,13 +18926,13 @@
         <v>113</v>
       </c>
       <c r="I522" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J522" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K522" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L522" t="str">
         <f t="shared" si="86"/>
@@ -19085,13 +19112,13 @@
         <v>113</v>
       </c>
       <c r="I531" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J531" t="s">
         <v>1198</v>
       </c>
       <c r="K531" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L531" t="str">
         <f t="shared" ref="L531:L532" si="87">_xlfn.TEXTJOIN("", TRUE, D531:K531)</f>
@@ -19121,13 +19148,13 @@
         <v>113</v>
       </c>
       <c r="I532" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J532" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K532" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L532" t="str">
         <f t="shared" si="87"/>
@@ -19377,13 +19404,13 @@
         <v>787</v>
       </c>
       <c r="I544" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J544" t="s">
-        <v>1255</v>
+        <v>1254</v>
       </c>
       <c r="K544" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L544" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D544:K544)</f>
@@ -19593,13 +19620,13 @@
         <v>792</v>
       </c>
       <c r="I558" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J558" t="s">
         <v>1244</v>
       </c>
-      <c r="J558" t="s">
+      <c r="K558" t="s">
         <v>1245</v>
-      </c>
-      <c r="K558" t="s">
-        <v>1246</v>
       </c>
       <c r="L558" t="str">
         <f t="shared" ref="L558:L562" si="90">_xlfn.TEXTJOIN("", TRUE, D558:K558)</f>
@@ -19626,13 +19653,13 @@
         <v>793</v>
       </c>
       <c r="I559" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J559" t="s">
         <v>1244</v>
       </c>
-      <c r="J559" t="s">
+      <c r="K559" t="s">
         <v>1245</v>
-      </c>
-      <c r="K559" t="s">
-        <v>1246</v>
       </c>
       <c r="L559" t="str">
         <f t="shared" si="90"/>
@@ -19659,13 +19686,13 @@
         <v>794</v>
       </c>
       <c r="I560" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J560" t="s">
-        <v>1255</v>
+        <v>1254</v>
       </c>
       <c r="K560" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L560" t="str">
         <f t="shared" si="90"/>
@@ -19692,13 +19719,13 @@
         <v>795</v>
       </c>
       <c r="I561" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J561" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K561" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L561" t="str">
         <f t="shared" si="90"/>
@@ -19725,13 +19752,13 @@
         <v>796</v>
       </c>
       <c r="I562" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J562" t="s">
-        <v>1265</v>
+        <v>1264</v>
       </c>
       <c r="K562" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L562" t="str">
         <f t="shared" si="90"/>
@@ -19935,13 +19962,13 @@
         <v>801</v>
       </c>
       <c r="I581" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J581" t="s">
         <v>1244</v>
       </c>
-      <c r="J581" t="s">
+      <c r="K581" t="s">
         <v>1245</v>
-      </c>
-      <c r="K581" t="s">
-        <v>1246</v>
       </c>
       <c r="L581" t="str">
         <f t="shared" ref="L581:L582" si="91">_xlfn.TEXTJOIN("", TRUE, D581:K581)</f>
@@ -19965,13 +19992,13 @@
         <v>802</v>
       </c>
       <c r="I582" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J582" t="s">
         <v>1198</v>
       </c>
       <c r="K582" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L582" t="str">
         <f t="shared" si="91"/>
@@ -20087,13 +20114,13 @@
         <v>805</v>
       </c>
       <c r="I591" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J591" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K591" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L591" t="str">
         <f t="shared" ref="L591:L592" si="92">_xlfn.TEXTJOIN("", TRUE, D591:K591)</f>
@@ -20117,13 +20144,13 @@
         <v>806</v>
       </c>
       <c r="I592" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J592" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K592" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L592" t="str">
         <f t="shared" si="92"/>
@@ -20368,13 +20395,13 @@
         <v>820</v>
       </c>
       <c r="I609" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J609" t="s">
         <v>1244</v>
       </c>
-      <c r="J609" t="s">
+      <c r="K609" t="s">
         <v>1245</v>
-      </c>
-      <c r="K609" t="s">
-        <v>1246</v>
       </c>
       <c r="L609" t="str">
         <f t="shared" ref="L609:L619" si="94">_xlfn.TEXTJOIN("", TRUE, D609:K609)</f>
@@ -20398,13 +20425,13 @@
         <v>821</v>
       </c>
       <c r="I610" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J610" t="s">
         <v>1244</v>
       </c>
-      <c r="J610" t="s">
+      <c r="K610" t="s">
         <v>1245</v>
-      </c>
-      <c r="K610" t="s">
-        <v>1246</v>
       </c>
       <c r="L610" t="str">
         <f t="shared" si="94"/>
@@ -20428,13 +20455,13 @@
         <v>822</v>
       </c>
       <c r="I611" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J611" t="s">
         <v>1244</v>
       </c>
-      <c r="J611" t="s">
+      <c r="K611" t="s">
         <v>1245</v>
-      </c>
-      <c r="K611" t="s">
-        <v>1246</v>
       </c>
       <c r="L611" t="str">
         <f t="shared" si="94"/>
@@ -20458,13 +20485,13 @@
         <v>823</v>
       </c>
       <c r="I612" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J612" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K612" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L612" t="str">
         <f t="shared" si="94"/>
@@ -20488,13 +20515,13 @@
         <v>824</v>
       </c>
       <c r="I613" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J613" t="s">
-        <v>1254</v>
+        <v>1253</v>
       </c>
       <c r="K613" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L613" t="str">
         <f t="shared" si="94"/>
@@ -20518,13 +20545,13 @@
         <v>825</v>
       </c>
       <c r="I614" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J614" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K614" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L614" t="str">
         <f t="shared" si="94"/>
@@ -20548,13 +20575,13 @@
         <v>818</v>
       </c>
       <c r="I615" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J615" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K615" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L615" t="str">
         <f t="shared" si="94"/>
@@ -20581,13 +20608,13 @@
         <v>859</v>
       </c>
       <c r="I616" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J616" t="s">
         <v>1244</v>
       </c>
-      <c r="J616" t="s">
+      <c r="K616" t="s">
         <v>1245</v>
-      </c>
-      <c r="K616" t="s">
-        <v>1246</v>
       </c>
       <c r="L616" t="str">
         <f t="shared" si="94"/>
@@ -20614,13 +20641,13 @@
         <v>860</v>
       </c>
       <c r="I617" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J617" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K617" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L617" t="str">
         <f t="shared" si="94"/>
@@ -20647,13 +20674,13 @@
         <v>861</v>
       </c>
       <c r="I618" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J618" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K618" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L618" t="str">
         <f t="shared" si="94"/>
@@ -20680,13 +20707,13 @@
         <v>862</v>
       </c>
       <c r="I619" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J619" t="s">
-        <v>1254</v>
+        <v>1253</v>
       </c>
       <c r="K619" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L619" t="str">
         <f t="shared" si="94"/>
@@ -20803,13 +20830,13 @@
         <v>872</v>
       </c>
       <c r="I626" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J626" t="s">
         <v>1244</v>
       </c>
-      <c r="J626" t="s">
+      <c r="K626" t="s">
         <v>1245</v>
-      </c>
-      <c r="K626" t="s">
-        <v>1246</v>
       </c>
       <c r="L626" t="str">
         <f t="shared" ref="L626:L629" si="96">_xlfn.TEXTJOIN("", TRUE, D626:K626)</f>
@@ -20836,13 +20863,13 @@
         <v>873</v>
       </c>
       <c r="I627" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J627" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K627" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L627" t="str">
         <f t="shared" si="96"/>
@@ -20869,13 +20896,13 @@
         <v>874</v>
       </c>
       <c r="I628" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J628" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K628" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L628" t="str">
         <f t="shared" si="96"/>
@@ -20902,13 +20929,13 @@
         <v>875</v>
       </c>
       <c r="I629" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J629" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K629" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L629" t="str">
         <f t="shared" si="96"/>
@@ -20987,13 +21014,13 @@
         <v>877</v>
       </c>
       <c r="I634" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J634" t="s">
         <v>1244</v>
       </c>
-      <c r="J634" t="s">
+      <c r="K634" t="s">
         <v>1245</v>
-      </c>
-      <c r="K634" t="s">
-        <v>1246</v>
       </c>
       <c r="L634" t="str">
         <f t="shared" ref="L634:L637" si="97">_xlfn.TEXTJOIN("", TRUE, D634:K634)</f>
@@ -21020,13 +21047,13 @@
         <v>878</v>
       </c>
       <c r="I635" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J635" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K635" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L635" t="str">
         <f t="shared" si="97"/>
@@ -21053,13 +21080,13 @@
         <v>879</v>
       </c>
       <c r="I636" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J636" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K636" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L636" t="str">
         <f t="shared" si="97"/>
@@ -21086,13 +21113,13 @@
         <v>880</v>
       </c>
       <c r="I637" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J637" t="s">
-        <v>1254</v>
+        <v>1253</v>
       </c>
       <c r="K637" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L637" t="str">
         <f t="shared" si="97"/>
@@ -21297,13 +21324,13 @@
         <v>887</v>
       </c>
       <c r="I651" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J651" t="s">
         <v>1244</v>
       </c>
-      <c r="J651" t="s">
+      <c r="K651" t="s">
         <v>1245</v>
-      </c>
-      <c r="K651" t="s">
-        <v>1246</v>
       </c>
       <c r="L651" t="str">
         <f t="shared" ref="L651:L660" si="99">_xlfn.TEXTJOIN("", TRUE, D651:K651)</f>
@@ -21327,13 +21354,13 @@
         <v>888</v>
       </c>
       <c r="I652" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J652" t="s">
         <v>1244</v>
       </c>
-      <c r="J652" t="s">
+      <c r="K652" t="s">
         <v>1245</v>
-      </c>
-      <c r="K652" t="s">
-        <v>1246</v>
       </c>
       <c r="L652" t="str">
         <f t="shared" si="99"/>
@@ -21357,13 +21384,13 @@
         <v>889</v>
       </c>
       <c r="I653" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J653" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K653" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L653" t="str">
         <f t="shared" si="99"/>
@@ -21387,13 +21414,13 @@
         <v>890</v>
       </c>
       <c r="I654" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J654" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K654" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L654" t="str">
         <f t="shared" si="99"/>
@@ -21417,13 +21444,13 @@
         <v>891</v>
       </c>
       <c r="I655" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J655" t="s">
         <v>1198</v>
       </c>
       <c r="K655" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L655" t="str">
         <f t="shared" si="99"/>
@@ -21447,13 +21474,13 @@
         <v>892</v>
       </c>
       <c r="I656" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J656" t="s">
         <v>1198</v>
       </c>
       <c r="K656" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L656" t="str">
         <f t="shared" si="99"/>
@@ -21477,13 +21504,13 @@
         <v>893</v>
       </c>
       <c r="I657" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J657" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K657" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L657" t="str">
         <f t="shared" si="99"/>
@@ -21507,13 +21534,13 @@
         <v>884</v>
       </c>
       <c r="I658" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J658" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K658" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L658" t="str">
         <f t="shared" si="99"/>
@@ -21540,13 +21567,13 @@
         <v>894</v>
       </c>
       <c r="I659" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J659" t="s">
         <v>1244</v>
       </c>
-      <c r="J659" t="s">
+      <c r="K659" t="s">
         <v>1245</v>
-      </c>
-      <c r="K659" t="s">
-        <v>1246</v>
       </c>
       <c r="L659" t="str">
         <f t="shared" si="99"/>
@@ -21573,13 +21600,13 @@
         <v>895</v>
       </c>
       <c r="I660" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J660" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K660" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L660" t="str">
         <f t="shared" si="99"/>
@@ -22012,13 +22039,13 @@
         <v>911</v>
       </c>
       <c r="I693" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J693" t="s">
         <v>1198</v>
       </c>
       <c r="K693" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L693" t="str">
         <f t="shared" ref="L693:L696" si="101">_xlfn.TEXTJOIN("", TRUE, D693:K693)</f>
@@ -22042,13 +22069,13 @@
         <v>912</v>
       </c>
       <c r="I694" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J694" t="s">
         <v>1198</v>
       </c>
       <c r="K694" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L694" t="str">
         <f t="shared" si="101"/>
@@ -22072,13 +22099,13 @@
         <v>913</v>
       </c>
       <c r="I695" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J695" t="s">
         <v>1198</v>
       </c>
       <c r="K695" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L695" t="str">
         <f t="shared" si="101"/>
@@ -22102,13 +22129,13 @@
         <v>914</v>
       </c>
       <c r="I696" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J696" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K696" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L696" t="str">
         <f t="shared" si="101"/>
@@ -22454,13 +22481,13 @@
         <v>930</v>
       </c>
       <c r="I717" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J717" t="s">
         <v>1198</v>
       </c>
       <c r="K717" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L717" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D717:K717)</f>
@@ -22559,13 +22586,13 @@
         <v>932</v>
       </c>
       <c r="I725" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J725" t="s">
         <v>1244</v>
       </c>
-      <c r="J725" t="s">
+      <c r="K725" t="s">
         <v>1245</v>
-      </c>
-      <c r="K725" t="s">
-        <v>1246</v>
       </c>
       <c r="L725" t="str">
         <f t="shared" ref="L725:L729" si="104">_xlfn.TEXTJOIN("", TRUE, D725:K725)</f>
@@ -22589,13 +22616,13 @@
         <v>933</v>
       </c>
       <c r="I726" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J726" t="s">
         <v>1244</v>
       </c>
-      <c r="J726" t="s">
+      <c r="K726" t="s">
         <v>1245</v>
-      </c>
-      <c r="K726" t="s">
-        <v>1246</v>
       </c>
       <c r="L726" t="str">
         <f t="shared" si="104"/>
@@ -22619,13 +22646,13 @@
         <v>934</v>
       </c>
       <c r="I727" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J727" t="s">
         <v>1244</v>
       </c>
-      <c r="J727" t="s">
+      <c r="K727" t="s">
         <v>1245</v>
-      </c>
-      <c r="K727" t="s">
-        <v>1246</v>
       </c>
       <c r="L727" t="str">
         <f t="shared" si="104"/>
@@ -22649,13 +22676,13 @@
         <v>935</v>
       </c>
       <c r="I728" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J728" t="s">
         <v>1198</v>
       </c>
       <c r="K728" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L728" t="str">
         <f t="shared" si="104"/>
@@ -22679,13 +22706,13 @@
         <v>936</v>
       </c>
       <c r="I729" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J729" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K729" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L729" t="str">
         <f t="shared" si="104"/>
@@ -22784,13 +22811,13 @@
         <v>938</v>
       </c>
       <c r="I737" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J737" t="s">
         <v>1244</v>
       </c>
-      <c r="J737" t="s">
+      <c r="K737" t="s">
         <v>1245</v>
-      </c>
-      <c r="K737" t="s">
-        <v>1246</v>
       </c>
       <c r="L737" t="str">
         <f t="shared" ref="L737:L742" si="106">_xlfn.TEXTJOIN("", TRUE, D737:K737)</f>
@@ -22814,13 +22841,13 @@
         <v>939</v>
       </c>
       <c r="I738" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J738" t="s">
         <v>1198</v>
       </c>
       <c r="K738" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L738" t="str">
         <f t="shared" si="106"/>
@@ -22844,13 +22871,13 @@
         <v>940</v>
       </c>
       <c r="I739" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J739" t="s">
         <v>1198</v>
       </c>
       <c r="K739" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L739" t="str">
         <f t="shared" si="106"/>
@@ -22874,13 +22901,13 @@
         <v>941</v>
       </c>
       <c r="I740" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J740" t="s">
-        <v>1254</v>
+        <v>1253</v>
       </c>
       <c r="K740" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L740" t="str">
         <f t="shared" si="106"/>
@@ -22904,13 +22931,13 @@
         <v>942</v>
       </c>
       <c r="I741" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J741" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K741" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L741" t="str">
         <f t="shared" si="106"/>
@@ -22934,13 +22961,13 @@
         <v>943</v>
       </c>
       <c r="I742" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J742" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K742" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L742" t="str">
         <f t="shared" si="106"/>
@@ -23060,13 +23087,13 @@
         <v>946</v>
       </c>
       <c r="I751" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J751" t="s">
         <v>1198</v>
       </c>
       <c r="K751" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L751" t="str">
         <f t="shared" ref="L751:L755" si="108">_xlfn.TEXTJOIN("", TRUE, D751:K751)</f>
@@ -23090,13 +23117,13 @@
         <v>947</v>
       </c>
       <c r="I752" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J752" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K752" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L752" t="str">
         <f t="shared" si="108"/>
@@ -23120,13 +23147,13 @@
         <v>948</v>
       </c>
       <c r="I753" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J753" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K753" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L753" t="str">
         <f t="shared" si="108"/>
@@ -23153,13 +23180,13 @@
         <v>949</v>
       </c>
       <c r="I754" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J754" t="s">
         <v>1198</v>
       </c>
       <c r="K754" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L754" t="str">
         <f t="shared" si="108"/>
@@ -23186,13 +23213,13 @@
         <v>950</v>
       </c>
       <c r="I755" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J755" t="s">
         <v>1198</v>
       </c>
       <c r="K755" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L755" t="str">
         <f t="shared" si="108"/>
@@ -23297,13 +23324,13 @@
         <v>953</v>
       </c>
       <c r="I763" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J763" t="s">
         <v>1198</v>
       </c>
       <c r="K763" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L763" t="str">
         <f t="shared" ref="L763:L765" si="109">_xlfn.TEXTJOIN("", TRUE, D763:K763)</f>
@@ -23327,13 +23354,13 @@
         <v>954</v>
       </c>
       <c r="I764" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J764" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K764" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L764" t="str">
         <f t="shared" si="109"/>
@@ -23363,13 +23390,13 @@
         <v>113</v>
       </c>
       <c r="I765" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J765" t="s">
         <v>1244</v>
       </c>
-      <c r="J765" t="s">
+      <c r="K765" t="s">
         <v>1245</v>
-      </c>
-      <c r="K765" t="s">
-        <v>1246</v>
       </c>
       <c r="L765" t="str">
         <f t="shared" si="109"/>
@@ -23453,13 +23480,13 @@
         <v>957</v>
       </c>
       <c r="I772" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J772" t="s">
-        <v>1254</v>
+        <v>1253</v>
       </c>
       <c r="K772" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L772" t="str">
         <f t="shared" ref="L772:L778" si="111">_xlfn.TEXTJOIN("", TRUE, D772:K772)</f>
@@ -23483,13 +23510,13 @@
         <v>958</v>
       </c>
       <c r="I773" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J773" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K773" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L773" t="str">
         <f t="shared" si="111"/>
@@ -23513,13 +23540,13 @@
         <v>959</v>
       </c>
       <c r="I774" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J774" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K774" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L774" t="str">
         <f t="shared" si="111"/>
@@ -23546,13 +23573,13 @@
         <v>960</v>
       </c>
       <c r="I775" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J775" t="s">
         <v>1244</v>
       </c>
-      <c r="J775" t="s">
+      <c r="K775" t="s">
         <v>1245</v>
-      </c>
-      <c r="K775" t="s">
-        <v>1246</v>
       </c>
       <c r="L775" t="str">
         <f t="shared" si="111"/>
@@ -23579,13 +23606,13 @@
         <v>961</v>
       </c>
       <c r="I776" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J776" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K776" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L776" t="str">
         <f t="shared" si="111"/>
@@ -23612,13 +23639,13 @@
         <v>962</v>
       </c>
       <c r="I777" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J777" t="s">
         <v>1198</v>
       </c>
       <c r="K777" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L777" t="str">
         <f t="shared" si="111"/>
@@ -23645,13 +23672,13 @@
         <v>963</v>
       </c>
       <c r="I778" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J778" t="s">
         <v>1198</v>
       </c>
       <c r="K778" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L778" t="str">
         <f t="shared" si="111"/>
@@ -23807,13 +23834,13 @@
         <v>965</v>
       </c>
       <c r="I792" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J792" t="s">
         <v>1244</v>
       </c>
-      <c r="J792" t="s">
+      <c r="K792" t="s">
         <v>1245</v>
-      </c>
-      <c r="K792" t="s">
-        <v>1246</v>
       </c>
       <c r="L792" t="str">
         <f t="shared" ref="L792:L796" si="113">_xlfn.TEXTJOIN("", TRUE, D792:K792)</f>
@@ -23837,13 +23864,13 @@
         <v>966</v>
       </c>
       <c r="I793" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J793" t="s">
         <v>1244</v>
       </c>
-      <c r="J793" t="s">
+      <c r="K793" t="s">
         <v>1245</v>
-      </c>
-      <c r="K793" t="s">
-        <v>1246</v>
       </c>
       <c r="L793" t="str">
         <f t="shared" si="113"/>
@@ -23867,13 +23894,13 @@
         <v>967</v>
       </c>
       <c r="I794" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J794" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="K794" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L794" t="str">
         <f t="shared" si="113"/>
@@ -23897,13 +23924,13 @@
         <v>968</v>
       </c>
       <c r="I795" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J795" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="K795" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L795" t="str">
         <f t="shared" si="113"/>
@@ -23927,13 +23954,13 @@
         <v>969</v>
       </c>
       <c r="I796" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J796" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="K796" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L796" t="str">
         <f t="shared" si="113"/>
@@ -24011,13 +24038,13 @@
         <v>970</v>
       </c>
       <c r="I803" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J803" t="s">
         <v>1244</v>
       </c>
-      <c r="J803" t="s">
+      <c r="K803" t="s">
         <v>1245</v>
-      </c>
-      <c r="K803" t="s">
-        <v>1246</v>
       </c>
       <c r="L803" t="str">
         <f t="shared" ref="L803:L814" si="114">_xlfn.TEXTJOIN("", TRUE, D803:K803)</f>
@@ -24041,13 +24068,13 @@
         <v>971</v>
       </c>
       <c r="I804" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J804" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K804" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L804" t="str">
         <f t="shared" si="114"/>
@@ -24071,13 +24098,13 @@
         <v>972</v>
       </c>
       <c r="I805" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J805" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K805" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L805" t="str">
         <f t="shared" si="114"/>
@@ -24101,13 +24128,13 @@
         <v>973</v>
       </c>
       <c r="I806" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J806" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K806" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L806" t="str">
         <f t="shared" si="114"/>
@@ -24131,13 +24158,13 @@
         <v>974</v>
       </c>
       <c r="I807" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J807" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K807" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L807" t="str">
         <f t="shared" si="114"/>
@@ -24161,13 +24188,13 @@
         <v>975</v>
       </c>
       <c r="I808" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J808" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K808" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L808" t="str">
         <f t="shared" si="114"/>
@@ -24191,13 +24218,13 @@
         <v>976</v>
       </c>
       <c r="I809" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J809" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K809" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L809" t="str">
         <f t="shared" si="114"/>
@@ -24221,13 +24248,13 @@
         <v>977</v>
       </c>
       <c r="I810" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J810" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
       <c r="K810" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L810" t="str">
         <f t="shared" si="114"/>
@@ -24251,13 +24278,13 @@
         <v>978</v>
       </c>
       <c r="I811" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J811" t="s">
-        <v>1256</v>
+        <v>1255</v>
       </c>
       <c r="K811" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L811" t="str">
         <f t="shared" si="114"/>
@@ -24281,13 +24308,13 @@
         <v>981</v>
       </c>
       <c r="I812" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J812" t="s">
-        <v>1257</v>
+        <v>1256</v>
       </c>
       <c r="K812" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L812" t="str">
         <f t="shared" si="114"/>
@@ -24311,13 +24338,13 @@
         <v>982</v>
       </c>
       <c r="I813" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J813" t="s">
-        <v>1257</v>
+        <v>1256</v>
       </c>
       <c r="K813" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L813" t="str">
         <f t="shared" si="114"/>
@@ -24341,13 +24368,13 @@
         <v>983</v>
       </c>
       <c r="I814" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J814" t="s">
-        <v>1257</v>
+        <v>1256</v>
       </c>
       <c r="K814" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L814" t="str">
         <f t="shared" si="114"/>
@@ -24479,13 +24506,13 @@
         <v>985</v>
       </c>
       <c r="I823" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J823" t="s">
         <v>1244</v>
       </c>
-      <c r="J823" t="s">
+      <c r="K823" t="s">
         <v>1245</v>
-      </c>
-      <c r="K823" t="s">
-        <v>1246</v>
       </c>
       <c r="L823" t="str">
         <f t="shared" ref="L823:L824" si="116">_xlfn.TEXTJOIN("", TRUE, D823:K823)</f>
@@ -24509,13 +24536,13 @@
         <v>986</v>
       </c>
       <c r="I824" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J824" t="s">
         <v>1244</v>
       </c>
-      <c r="J824" t="s">
+      <c r="K824" t="s">
         <v>1245</v>
-      </c>
-      <c r="K824" t="s">
-        <v>1246</v>
       </c>
       <c r="L824" t="str">
         <f t="shared" si="116"/>
@@ -24635,13 +24662,13 @@
         <v>989</v>
       </c>
       <c r="I833" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J833" t="s">
         <v>1244</v>
       </c>
-      <c r="J833" t="s">
+      <c r="K833" t="s">
         <v>1245</v>
-      </c>
-      <c r="K833" t="s">
-        <v>1246</v>
       </c>
       <c r="L833" t="str">
         <f t="shared" ref="L833:L834" si="118">_xlfn.TEXTJOIN("", TRUE, D833:K833)</f>
@@ -24665,13 +24692,13 @@
         <v>990</v>
       </c>
       <c r="I834" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J834" t="s">
         <v>1198</v>
       </c>
       <c r="K834" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L834" t="str">
         <f t="shared" si="118"/>
@@ -24746,13 +24773,13 @@
         <v>993</v>
       </c>
       <c r="I837" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J837" t="s">
-        <v>1267</v>
+        <v>1266</v>
       </c>
       <c r="K837" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L837" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D837:K837)</f>
@@ -24824,13 +24851,13 @@
         <v>113</v>
       </c>
       <c r="I842" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J842" t="s">
-        <v>1266</v>
+        <v>1265</v>
       </c>
       <c r="K842" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L842" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D842:K842)</f>
@@ -24966,13 +24993,13 @@
         <v>1001</v>
       </c>
       <c r="I854" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J854" t="s">
         <v>1244</v>
       </c>
-      <c r="J854" t="s">
+      <c r="K854" t="s">
         <v>1245</v>
-      </c>
-      <c r="K854" t="s">
-        <v>1246</v>
       </c>
       <c r="L854" t="str">
         <f t="shared" ref="L854:L856" si="120">_xlfn.TEXTJOIN("", TRUE, D854:K854)</f>
@@ -24996,13 +25023,13 @@
         <v>1002</v>
       </c>
       <c r="I855" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J855" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K855" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L855" t="str">
         <f t="shared" si="120"/>
@@ -25026,13 +25053,13 @@
         <v>1003</v>
       </c>
       <c r="I856" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J856" t="s">
-        <v>1261</v>
+        <v>1260</v>
       </c>
       <c r="K856" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L856" t="str">
         <f t="shared" si="120"/>
@@ -25185,13 +25212,13 @@
         <v>1008</v>
       </c>
       <c r="I866" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J866" t="s">
         <v>1244</v>
       </c>
-      <c r="J866" t="s">
+      <c r="K866" t="s">
         <v>1245</v>
-      </c>
-      <c r="K866" t="s">
-        <v>1246</v>
       </c>
       <c r="L866" t="str">
         <f t="shared" ref="L866:L867" si="121">_xlfn.TEXTJOIN("", TRUE, D866:K866)</f>
@@ -25215,13 +25242,13 @@
         <v>1009</v>
       </c>
       <c r="I867" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J867" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K867" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L867" t="str">
         <f t="shared" si="121"/>
@@ -25418,13 +25445,13 @@
         <v>113</v>
       </c>
       <c r="I881" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J881" t="s">
-        <v>1236</v>
+        <v>1235</v>
       </c>
       <c r="K881" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L881" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D881:K881)</f>
@@ -25779,13 +25806,13 @@
         <v>1034</v>
       </c>
       <c r="I907" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J907" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="K907" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L907" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D907:K907)</f>
@@ -25980,13 +26007,13 @@
         <v>1041</v>
       </c>
       <c r="I919" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J919" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K919" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L919" t="str">
         <f t="shared" ref="L919:L920" si="123">_xlfn.TEXTJOIN("", TRUE, D919:K919)</f>
@@ -26010,13 +26037,13 @@
         <v>1042</v>
       </c>
       <c r="I920" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J920" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K920" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L920" t="str">
         <f t="shared" si="123"/>
@@ -26169,13 +26196,13 @@
         <v>1047</v>
       </c>
       <c r="I930" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J930" t="s">
         <v>1198</v>
       </c>
       <c r="K930" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L930" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D930:K930)</f>
@@ -26316,13 +26343,13 @@
         <v>1051</v>
       </c>
       <c r="I940" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J940" t="s">
         <v>1198</v>
       </c>
       <c r="K940" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L940" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D940:K940)</f>
@@ -26472,13 +26499,13 @@
         <v>1056</v>
       </c>
       <c r="I950" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J950" t="s">
-        <v>1262</v>
+        <v>1261</v>
       </c>
       <c r="K950" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L950" t="str">
         <f t="shared" ref="L950:L953" si="125">_xlfn.TEXTJOIN("", TRUE, D950:K950)</f>
@@ -26502,13 +26529,13 @@
         <v>1057</v>
       </c>
       <c r="I951" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J951" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K951" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L951" t="str">
         <f t="shared" si="125"/>
@@ -26532,13 +26559,13 @@
         <v>1058</v>
       </c>
       <c r="I952" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J952" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K952" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L952" t="str">
         <f t="shared" si="125"/>
@@ -26562,13 +26589,13 @@
         <v>1059</v>
       </c>
       <c r="I953" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J953" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K953" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L953" t="str">
         <f t="shared" si="125"/>
@@ -26700,13 +26727,13 @@
         <v>1063</v>
       </c>
       <c r="I962" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J962" t="s">
         <v>1244</v>
       </c>
-      <c r="J962" t="s">
+      <c r="K962" t="s">
         <v>1245</v>
-      </c>
-      <c r="K962" t="s">
-        <v>1246</v>
       </c>
       <c r="L962" t="str">
         <f t="shared" ref="L962:L966" si="127">_xlfn.TEXTJOIN("", TRUE, D962:K962)</f>
@@ -26730,13 +26757,13 @@
         <v>1064</v>
       </c>
       <c r="I963" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J963" t="s">
         <v>1244</v>
       </c>
-      <c r="J963" t="s">
+      <c r="K963" t="s">
         <v>1245</v>
-      </c>
-      <c r="K963" t="s">
-        <v>1246</v>
       </c>
       <c r="L963" t="str">
         <f t="shared" si="127"/>
@@ -26760,13 +26787,13 @@
         <v>1065</v>
       </c>
       <c r="I964" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J964" t="s">
         <v>1198</v>
       </c>
       <c r="K964" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L964" t="str">
         <f t="shared" si="127"/>
@@ -26790,13 +26817,13 @@
         <v>1066</v>
       </c>
       <c r="I965" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J965" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K965" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L965" t="str">
         <f t="shared" si="127"/>
@@ -26820,13 +26847,13 @@
         <v>1067</v>
       </c>
       <c r="I966" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J966" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K966" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L966" t="str">
         <f t="shared" si="127"/>
@@ -27009,13 +27036,13 @@
         <v>1071</v>
       </c>
       <c r="I981" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J981" t="s">
         <v>1244</v>
       </c>
-      <c r="J981" t="s">
+      <c r="K981" t="s">
         <v>1245</v>
-      </c>
-      <c r="K981" t="s">
-        <v>1246</v>
       </c>
       <c r="L981" t="str">
         <f t="shared" ref="L981:L984" si="129">_xlfn.TEXTJOIN("", TRUE, D981:K981)</f>
@@ -27039,13 +27066,13 @@
         <v>1072</v>
       </c>
       <c r="I982" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J982" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K982" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L982" t="str">
         <f t="shared" si="129"/>
@@ -27069,13 +27096,13 @@
         <v>1073</v>
       </c>
       <c r="I983" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J983" t="s">
         <v>1198</v>
       </c>
       <c r="K983" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L983" t="str">
         <f t="shared" si="129"/>
@@ -27099,13 +27126,13 @@
         <v>1074</v>
       </c>
       <c r="I984" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J984" t="s">
-        <v>1254</v>
+        <v>1253</v>
       </c>
       <c r="K984" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L984" t="str">
         <f t="shared" si="129"/>
@@ -27237,13 +27264,13 @@
         <v>1081</v>
       </c>
       <c r="I992" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J992" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K992" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L992" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D992:K992)</f>
@@ -27322,13 +27349,13 @@
         <v>1084</v>
       </c>
       <c r="I997" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J997" t="s">
-        <v>1254</v>
+        <v>1253</v>
       </c>
       <c r="K997" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L997" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D997:K997)</f>
@@ -27401,13 +27428,13 @@
         <v>1087</v>
       </c>
       <c r="I1003" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J1003" t="s">
         <v>1244</v>
       </c>
-      <c r="J1003" t="s">
+      <c r="K1003" t="s">
         <v>1245</v>
-      </c>
-      <c r="K1003" t="s">
-        <v>1246</v>
       </c>
       <c r="L1003" t="str">
         <f t="shared" ref="L1003:L1013" si="131">_xlfn.TEXTJOIN("", TRUE, D1003:K1003)</f>
@@ -27431,13 +27458,13 @@
         <v>1088</v>
       </c>
       <c r="I1004" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1004" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K1004" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1004" t="str">
         <f t="shared" si="131"/>
@@ -27461,13 +27488,13 @@
         <v>1089</v>
       </c>
       <c r="I1005" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1005" t="s">
-        <v>1263</v>
+        <v>1262</v>
       </c>
       <c r="K1005" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1005" t="str">
         <f t="shared" si="131"/>
@@ -27491,13 +27518,13 @@
         <v>1090</v>
       </c>
       <c r="I1006" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1006" t="s">
         <v>1198</v>
       </c>
       <c r="K1006" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1006" t="str">
         <f t="shared" si="131"/>
@@ -27521,13 +27548,13 @@
         <v>1091</v>
       </c>
       <c r="I1007" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1007" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="K1007" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1007" t="str">
         <f t="shared" si="131"/>
@@ -27551,13 +27578,13 @@
         <v>1092</v>
       </c>
       <c r="I1008" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1008" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="K1008" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1008" t="str">
         <f t="shared" si="131"/>
@@ -27581,13 +27608,13 @@
         <v>1093</v>
       </c>
       <c r="I1009" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1009" t="s">
-        <v>1253</v>
+        <v>1252</v>
       </c>
       <c r="K1009" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1009" t="str">
         <f t="shared" si="131"/>
@@ -27611,13 +27638,13 @@
         <v>1094</v>
       </c>
       <c r="I1010" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1010" t="s">
-        <v>1258</v>
+        <v>1257</v>
       </c>
       <c r="K1010" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1010" t="str">
         <f t="shared" si="131"/>
@@ -27641,13 +27668,13 @@
         <v>1095</v>
       </c>
       <c r="I1011" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1011" t="s">
-        <v>1258</v>
+        <v>1257</v>
       </c>
       <c r="K1011" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1011" t="str">
         <f t="shared" si="131"/>
@@ -27671,13 +27698,13 @@
         <v>1096</v>
       </c>
       <c r="I1012" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1012" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K1012" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1012" t="str">
         <f t="shared" si="131"/>
@@ -27701,13 +27728,13 @@
         <v>1085</v>
       </c>
       <c r="I1013" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1013" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K1013" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1013" t="str">
         <f t="shared" si="131"/>
@@ -27782,13 +27809,13 @@
         <v>1099</v>
       </c>
       <c r="I1016" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1016" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K1016" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1016" t="str">
         <f>_xlfn.TEXTJOIN("", TRUE, D1016:K1016)</f>
@@ -27872,13 +27899,13 @@
         <v>1101</v>
       </c>
       <c r="I1023" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J1023" t="s">
         <v>1244</v>
       </c>
-      <c r="J1023" t="s">
+      <c r="K1023" t="s">
         <v>1245</v>
-      </c>
-      <c r="K1023" t="s">
-        <v>1246</v>
       </c>
       <c r="L1023" t="str">
         <f t="shared" ref="L1023:L1026" si="133">_xlfn.TEXTJOIN("", TRUE, D1023:K1023)</f>
@@ -27902,13 +27929,13 @@
         <v>1102</v>
       </c>
       <c r="I1024" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1024" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K1024" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1024" t="str">
         <f t="shared" si="133"/>
@@ -27932,13 +27959,13 @@
         <v>1103</v>
       </c>
       <c r="I1025" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1025" t="s">
         <v>1198</v>
       </c>
       <c r="K1025" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1025" t="str">
         <f t="shared" si="133"/>
@@ -27962,13 +27989,13 @@
         <v>1104</v>
       </c>
       <c r="I1026" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1026" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K1026" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1026" t="str">
         <f t="shared" si="133"/>
@@ -28109,13 +28136,13 @@
         <v>1109</v>
       </c>
       <c r="I1036" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1036" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K1036" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1036" t="str">
         <f t="shared" ref="L1036:L1043" si="135">_xlfn.TEXTJOIN("", TRUE, D1036:K1036)</f>
@@ -28139,13 +28166,13 @@
         <v>1110</v>
       </c>
       <c r="I1037" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1037" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K1037" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1037" t="str">
         <f t="shared" si="135"/>
@@ -28169,13 +28196,13 @@
         <v>1111</v>
       </c>
       <c r="I1038" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1038" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K1038" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1038" t="str">
         <f t="shared" si="135"/>
@@ -28199,13 +28226,13 @@
         <v>1112</v>
       </c>
       <c r="I1039" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1039" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K1039" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1039" t="str">
         <f t="shared" si="135"/>
@@ -28229,13 +28256,13 @@
         <v>1113</v>
       </c>
       <c r="I1040" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1040" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K1040" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1040" t="str">
         <f t="shared" si="135"/>
@@ -28259,13 +28286,13 @@
         <v>1105</v>
       </c>
       <c r="I1041" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1041" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K1041" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1041" t="str">
         <f t="shared" si="135"/>
@@ -28292,13 +28319,13 @@
         <v>1114</v>
       </c>
       <c r="I1042" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1042" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K1042" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1042" t="str">
         <f t="shared" si="135"/>
@@ -28325,13 +28352,13 @@
         <v>1115</v>
       </c>
       <c r="I1043" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1043" t="s">
-        <v>1247</v>
+        <v>1246</v>
       </c>
       <c r="K1043" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1043" t="str">
         <f t="shared" si="135"/>
@@ -28394,13 +28421,13 @@
         <v>1116</v>
       </c>
       <c r="I1049" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J1049" t="s">
         <v>1244</v>
       </c>
-      <c r="J1049" t="s">
+      <c r="K1049" t="s">
         <v>1245</v>
-      </c>
-      <c r="K1049" t="s">
-        <v>1246</v>
       </c>
       <c r="L1049" t="str">
         <f t="shared" ref="L1049:L1053" si="136">_xlfn.TEXTJOIN("", TRUE, D1049:K1049)</f>
@@ -28424,13 +28451,13 @@
         <v>1117</v>
       </c>
       <c r="I1050" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J1050" t="s">
         <v>1244</v>
       </c>
-      <c r="J1050" t="s">
+      <c r="K1050" t="s">
         <v>1245</v>
-      </c>
-      <c r="K1050" t="s">
-        <v>1246</v>
       </c>
       <c r="L1050" t="str">
         <f t="shared" si="136"/>
@@ -28454,13 +28481,13 @@
         <v>1118</v>
       </c>
       <c r="I1051" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1051" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K1051" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1051" t="str">
         <f t="shared" si="136"/>
@@ -28484,13 +28511,13 @@
         <v>1119</v>
       </c>
       <c r="I1052" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1052" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K1052" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1052" t="str">
         <f t="shared" si="136"/>
@@ -28514,13 +28541,13 @@
         <v>1120</v>
       </c>
       <c r="I1053" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1053" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K1053" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1053" t="str">
         <f t="shared" si="136"/>
@@ -28598,13 +28625,13 @@
         <v>1121</v>
       </c>
       <c r="I1060" t="s">
+        <v>1243</v>
+      </c>
+      <c r="J1060" t="s">
         <v>1244</v>
       </c>
-      <c r="J1060" t="s">
+      <c r="K1060" t="s">
         <v>1245</v>
-      </c>
-      <c r="K1060" t="s">
-        <v>1246</v>
       </c>
       <c r="L1060" t="str">
         <f t="shared" ref="L1060:L1070" si="138">_xlfn.TEXTJOIN("", TRUE, D1060:K1060)</f>
@@ -28628,13 +28655,13 @@
         <v>1122</v>
       </c>
       <c r="I1061" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1061" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K1061" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1061" t="str">
         <f t="shared" si="138"/>
@@ -28658,13 +28685,13 @@
         <v>1123</v>
       </c>
       <c r="I1062" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1062" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K1062" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1062" t="str">
         <f t="shared" si="138"/>
@@ -28688,13 +28715,13 @@
         <v>1124</v>
       </c>
       <c r="I1063" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1063" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K1063" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1063" t="str">
         <f t="shared" si="138"/>
@@ -28718,13 +28745,13 @@
         <v>1125</v>
       </c>
       <c r="I1064" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1064" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K1064" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1064" t="str">
         <f t="shared" si="138"/>
@@ -28748,13 +28775,13 @@
         <v>1126</v>
       </c>
       <c r="I1065" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1065" t="s">
-        <v>1249</v>
+        <v>1248</v>
       </c>
       <c r="K1065" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1065" t="str">
         <f t="shared" si="138"/>
@@ -28778,13 +28805,13 @@
         <v>1127</v>
       </c>
       <c r="I1066" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1066" t="s">
-        <v>1254</v>
+        <v>1253</v>
       </c>
       <c r="K1066" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1066" t="str">
         <f t="shared" si="138"/>
@@ -28808,13 +28835,13 @@
         <v>1128</v>
       </c>
       <c r="I1067" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1067" t="s">
-        <v>1254</v>
+        <v>1253</v>
       </c>
       <c r="K1067" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1067" t="str">
         <f t="shared" si="138"/>
@@ -28838,13 +28865,13 @@
         <v>1129</v>
       </c>
       <c r="I1068" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1068" t="s">
-        <v>1264</v>
+        <v>1263</v>
       </c>
       <c r="K1068" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1068" t="str">
         <f t="shared" si="138"/>
@@ -28868,13 +28895,13 @@
         <v>1130</v>
       </c>
       <c r="I1069" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1069" t="s">
-        <v>1264</v>
+        <v>1263</v>
       </c>
       <c r="K1069" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1069" t="str">
         <f t="shared" si="138"/>
@@ -28901,13 +28928,13 @@
         <v>1131</v>
       </c>
       <c r="I1070" t="s">
-        <v>1244</v>
+        <v>1243</v>
       </c>
       <c r="J1070" t="s">
-        <v>1254</v>
+        <v>1253</v>
       </c>
       <c r="K1070" t="s">
-        <v>1246</v>
+        <v>1245</v>
       </c>
       <c r="L1070" t="str">
         <f t="shared" si="138"/>

</xml_diff>

<commit_message>
added Seltene Hieroglyphen and Projekt pages
</commit_message>
<xml_diff>
--- a/data/content.xlsx
+++ b/data/content.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Markus/Documents/Arbeit/Inschriftenschluessel/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21DC3380-A992-124B-82C5-3098548C4EEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D33B314-41E0-BC4B-A3AD-B9FAFA5F237B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1240" yWindow="500" windowWidth="21640" windowHeight="19440" activeTab="3" xr2:uid="{F025A444-F8B0-5C41-A37E-BEE791B22240}"/>
+    <workbookView xWindow="2640" yWindow="500" windowWidth="21640" windowHeight="19440" activeTab="3" xr2:uid="{F025A444-F8B0-5C41-A37E-BEE791B22240}"/>
   </bookViews>
   <sheets>
     <sheet name="pages" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5600" uniqueCount="1283">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5889" uniqueCount="1366">
   <si>
     <t>page_id</t>
   </si>
@@ -3891,6 +3891,255 @@
   </si>
   <si>
     <t>bei Müttern im AR: *sꜣ⸗s*</t>
+  </si>
+  <si>
+    <t>seltenHierogl</t>
+  </si>
+  <si>
+    <t>Seltene Hieroglphen</t>
+  </si>
+  <si>
+    <t>pages/seltenHierogl</t>
+  </si>
+  <si>
+    <t>Hieroglyphe</t>
+  </si>
+  <si>
+    <t>tb_seltenHierogl_GardF</t>
+  </si>
+  <si>
+    <t>A – Der Mann und seine Tätigkeiten</t>
+  </si>
+  <si>
+    <t>B – Die Frau und ihre Tätigkeiten</t>
+  </si>
+  <si>
+    <t>C – Gottheiten in Menschengestalt</t>
+  </si>
+  <si>
+    <t>D – Teile des menschlichen Körpers</t>
+  </si>
+  <si>
+    <t>E – Säugetiere</t>
+  </si>
+  <si>
+    <t>F – Teile von Säugetieren</t>
+  </si>
+  <si>
+    <t>G – Vögel</t>
+  </si>
+  <si>
+    <t>H – Teile von Vögeln</t>
+  </si>
+  <si>
+    <t>I – Amphibien und Reptilien</t>
+  </si>
+  <si>
+    <t>K – Fische und Teile von Fischen</t>
+  </si>
+  <si>
+    <t>L – Wirbellose und andere Tiere</t>
+  </si>
+  <si>
+    <t>M – Bäume und andere Pflanzen</t>
+  </si>
+  <si>
+    <t>N – Himmel, Erde und Wasser</t>
+  </si>
+  <si>
+    <t>O – Gebäude und Teile von Gebäuden</t>
+  </si>
+  <si>
+    <t>P – Schiffe und Teile von Schiffen</t>
+  </si>
+  <si>
+    <t>Q – Möbel</t>
+  </si>
+  <si>
+    <t>R – Tempel</t>
+  </si>
+  <si>
+    <t>S – Kronen</t>
+  </si>
+  <si>
+    <t>T – Krieg, Jagd und Schlachterei</t>
+  </si>
+  <si>
+    <t>U – Landwirtschaft und Handwerk</t>
+  </si>
+  <si>
+    <t>V – Seil, Faser, Korb usw.</t>
+  </si>
+  <si>
+    <t>W – Stein- und Tongefäße</t>
+  </si>
+  <si>
+    <t>X – Laibe und Kuchen</t>
+  </si>
+  <si>
+    <t>Y – Schreiben, Spiele und Musik</t>
+  </si>
+  <si>
+    <t>Z – Geometrische Figuren</t>
+  </si>
+  <si>
+    <t>Aa – unklassifizierte Hieroglyphen</t>
+  </si>
+  <si>
+    <t>tb_seltenHierogl_GardA</t>
+  </si>
+  <si>
+    <t>tb_seltenHierogl_GardB</t>
+  </si>
+  <si>
+    <t>tb_seltenHierogl_GardC</t>
+  </si>
+  <si>
+    <t>tb_seltenHierogl_GardD</t>
+  </si>
+  <si>
+    <t>tb_seltenHierogl_GardE</t>
+  </si>
+  <si>
+    <t>tb_seltenHierogl_GardG</t>
+  </si>
+  <si>
+    <t>tb_seltenHierogl_GardH</t>
+  </si>
+  <si>
+    <t>tb_seltenHierogl_GardI</t>
+  </si>
+  <si>
+    <t>tb_seltenHierogl_GardK</t>
+  </si>
+  <si>
+    <t>tb_seltenHierogl_GardL</t>
+  </si>
+  <si>
+    <t>tb_seltenHierogl_GardM</t>
+  </si>
+  <si>
+    <t>tb_seltenHierogl_GardN</t>
+  </si>
+  <si>
+    <t>tb_seltenHierogl_GardO</t>
+  </si>
+  <si>
+    <t>tb_seltenHierogl_GardP</t>
+  </si>
+  <si>
+    <t>tb_seltenHierogl_GardQ</t>
+  </si>
+  <si>
+    <t>tb_seltenHierogl_GardR</t>
+  </si>
+  <si>
+    <t>tb_seltenHierogl_GardS</t>
+  </si>
+  <si>
+    <t>tb_seltenHierogl_GardT</t>
+  </si>
+  <si>
+    <t>tb_seltenHierogl_GardU</t>
+  </si>
+  <si>
+    <t>tb_seltenHierogl_GardV</t>
+  </si>
+  <si>
+    <t>tb_seltenHierogl_GardW</t>
+  </si>
+  <si>
+    <t>tb_seltenHierogl_GardX</t>
+  </si>
+  <si>
+    <t>tb_seltenHierogl_GardY</t>
+  </si>
+  <si>
+    <t>tb_seltenHierogl_GardZ</t>
+  </si>
+  <si>
+    <t>tb_seltenHierogl_GardAa</t>
+  </si>
+  <si>
+    <t>F63_xnty_01</t>
+  </si>
+  <si>
+    <t>03_Hieroglyphen-selten/</t>
+  </si>
+  <si>
+    <t>*ḫnty*</t>
+  </si>
+  <si>
+    <t>vorn befindlich</t>
+  </si>
+  <si>
+    <t>Gardiner-Nr.</t>
+  </si>
+  <si>
+    <t>F63</t>
+  </si>
+  <si>
+    <t>N6B</t>
+  </si>
+  <si>
+    <t>N6B_nsw-bjt_01</t>
+  </si>
+  <si>
+    <t>König von Ober- und Unterägypten</t>
+  </si>
+  <si>
+    <t>N102_jmn_01</t>
+  </si>
+  <si>
+    <t>N102</t>
+  </si>
+  <si>
+    <t>projekt</t>
+  </si>
+  <si>
+    <t>Projekt</t>
+  </si>
+  <si>
+    <t>pages/projekt</t>
+  </si>
+  <si>
+    <t>Version:</t>
+  </si>
+  <si>
+    <t>RStudio 2025.09.1+401 "Cucumberleaf Sunflower" Release (20de356561bd58a6d88927cce948bd076d06e4ca, 2025-09-23) for macOS</t>
+  </si>
+  <si>
+    <t>Mozilla/5.0 (Macintosh; Intel Mac OS X 10_15_7)</t>
+  </si>
+  <si>
+    <t>AppleWebKit/537.36 (KHTML, like Gecko)</t>
+  </si>
+  <si>
+    <t>RStudio/2025.09.1+401</t>
+  </si>
+  <si>
+    <t>Chrome/138.0.7204.185</t>
+  </si>
+  <si>
+    <t>Github:</t>
+  </si>
+  <si>
+    <t>&lt;https://github.com/MarkusKut/Inschriftenschluessel.git&gt;</t>
+  </si>
+  <si>
+    <t>Mitarbeiter:</t>
+  </si>
+  <si>
+    <t>- **Projektleitung:** Prof. Friedhelm Hoffmann</t>
+  </si>
+  <si>
+    <t>- **Recherche, Datengrundlage:** Iulia Comșa</t>
+  </si>
+  <si>
+    <t>- **Programmierung, Hieroglyphensetzung:** Markus Kutschka</t>
+  </si>
+  <si>
+    <t>Diese Website wurde mit Quarto unter R erstellt:</t>
   </si>
 </sst>
 </file>
@@ -3900,7 +4149,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0000"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -3921,6 +4170,14 @@
       <sz val="12"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -3989,10 +4246,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -4061,8 +4319,13 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Link" xfId="1" builtinId="8"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -4395,7 +4658,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E50E2D7D-6A15-A747-8ABA-0F1F90941768}">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="7.5" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.83203125" bestFit="1" customWidth="1"/>
@@ -4679,6 +4942,40 @@
       </c>
       <c r="F16">
         <v>150</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B17" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" t="s">
+        <v>1284</v>
+      </c>
+      <c r="D17" t="s">
+        <v>1285</v>
+      </c>
+      <c r="F17">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>1350</v>
+      </c>
+      <c r="B18" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" t="s">
+        <v>1351</v>
+      </c>
+      <c r="D18" t="s">
+        <v>1352</v>
+      </c>
+      <c r="F18">
+        <v>170</v>
       </c>
     </row>
   </sheetData>
@@ -5313,13 +5610,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AEDD5969-C8E3-C04D-AF17-FDEFB8218719}">
-  <dimension ref="A1:K55"/>
+  <dimension ref="A1:K98"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="7.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12" style="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="11.1640625" style="4" customWidth="1"/>
     <col min="3" max="3" width="7.33203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.33203125" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.1640625" style="4" customWidth="1"/>
     <col min="5" max="5" width="36.1640625" style="2" customWidth="1"/>
     <col min="6" max="6" width="21.1640625" style="4" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.1640625" style="4" bestFit="1" customWidth="1"/>
@@ -6309,7 +6606,912 @@
         <v>4</v>
       </c>
     </row>
+    <row r="59" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A59" s="4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C59" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>1288</v>
+      </c>
+      <c r="F59" s="4" t="s">
+        <v>1314</v>
+      </c>
+      <c r="G59" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J59" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="K59" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A60" s="4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B60" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C60" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D60" s="4" t="s">
+        <v>1289</v>
+      </c>
+      <c r="F60" s="4" t="s">
+        <v>1315</v>
+      </c>
+      <c r="G60" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J60" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="K60" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A61" s="4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B61" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C61" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D61" s="4" t="s">
+        <v>1290</v>
+      </c>
+      <c r="F61" s="4" t="s">
+        <v>1316</v>
+      </c>
+      <c r="G61" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J61" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="K61" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A62" s="4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C62" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D62" s="4" t="s">
+        <v>1291</v>
+      </c>
+      <c r="F62" s="4" t="s">
+        <v>1317</v>
+      </c>
+      <c r="G62" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J62" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="K62" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A63" s="4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B63" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C63" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D63" s="4" t="s">
+        <v>1292</v>
+      </c>
+      <c r="F63" s="4" t="s">
+        <v>1318</v>
+      </c>
+      <c r="G63" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J63" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="K63" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A64" s="4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B64" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C64" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D64" s="4" t="s">
+        <v>1293</v>
+      </c>
+      <c r="F64" s="4" t="s">
+        <v>1287</v>
+      </c>
+      <c r="G64" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J64" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="K64" s="4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A65" s="4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B65" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C65" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D65" s="4" t="s">
+        <v>1294</v>
+      </c>
+      <c r="F65" s="4" t="s">
+        <v>1319</v>
+      </c>
+      <c r="G65" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J65" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="K65" s="4">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A66" s="4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B66" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C66" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D66" s="4" t="s">
+        <v>1295</v>
+      </c>
+      <c r="F66" s="4" t="s">
+        <v>1320</v>
+      </c>
+      <c r="G66" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J66" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="K66" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A67" s="4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B67" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C67" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D67" s="4" t="s">
+        <v>1296</v>
+      </c>
+      <c r="F67" s="4" t="s">
+        <v>1321</v>
+      </c>
+      <c r="G67" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J67" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="K67" s="4">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A68" s="4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D68" s="4" t="s">
+        <v>1297</v>
+      </c>
+      <c r="F68" s="4" t="s">
+        <v>1322</v>
+      </c>
+      <c r="G68" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J68" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="K68" s="4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A69" s="4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B69" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C69" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D69" s="4" t="s">
+        <v>1298</v>
+      </c>
+      <c r="F69" s="4" t="s">
+        <v>1323</v>
+      </c>
+      <c r="G69" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J69" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="K69" s="4">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A70" s="4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C70" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D70" s="4" t="s">
+        <v>1299</v>
+      </c>
+      <c r="F70" s="4" t="s">
+        <v>1324</v>
+      </c>
+      <c r="G70" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J70" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="K70" s="4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A71" s="4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B71" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C71" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D71" s="4" t="s">
+        <v>1300</v>
+      </c>
+      <c r="F71" s="4" t="s">
+        <v>1325</v>
+      </c>
+      <c r="G71" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J71" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="K71" s="4">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A72" s="4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C72" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D72" s="4" t="s">
+        <v>1301</v>
+      </c>
+      <c r="F72" s="4" t="s">
+        <v>1326</v>
+      </c>
+      <c r="G72" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J72" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="K72" s="4">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A73" s="4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D73" s="4" t="s">
+        <v>1302</v>
+      </c>
+      <c r="F73" s="4" t="s">
+        <v>1327</v>
+      </c>
+      <c r="G73" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J73" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="K73" s="4">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A74" s="4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B74" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D74" s="4" t="s">
+        <v>1303</v>
+      </c>
+      <c r="F74" s="4" t="s">
+        <v>1328</v>
+      </c>
+      <c r="G74" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J74" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="K74" s="4">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A75" s="4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D75" s="4" t="s">
+        <v>1304</v>
+      </c>
+      <c r="F75" s="4" t="s">
+        <v>1329</v>
+      </c>
+      <c r="G75" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J75" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="K75" s="4">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A76" s="4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B76" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D76" s="4" t="s">
+        <v>1305</v>
+      </c>
+      <c r="F76" s="4" t="s">
+        <v>1330</v>
+      </c>
+      <c r="G76" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J76" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="K76" s="4">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A77" s="4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B77" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D77" s="4" t="s">
+        <v>1306</v>
+      </c>
+      <c r="F77" s="4" t="s">
+        <v>1331</v>
+      </c>
+      <c r="G77" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J77" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="K77" s="4">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A78" s="4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B78" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C78" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D78" s="4" t="s">
+        <v>1307</v>
+      </c>
+      <c r="F78" s="4" t="s">
+        <v>1332</v>
+      </c>
+      <c r="G78" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J78" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="K78" s="4">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A79" s="4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C79" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D79" s="4" t="s">
+        <v>1308</v>
+      </c>
+      <c r="F79" s="4" t="s">
+        <v>1333</v>
+      </c>
+      <c r="G79" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J79" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="K79" s="4">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A80" s="4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B80" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C80" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D80" s="4" t="s">
+        <v>1309</v>
+      </c>
+      <c r="F80" s="4" t="s">
+        <v>1334</v>
+      </c>
+      <c r="G80" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J80" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="K80" s="4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A81" s="4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B81" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C81" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D81" s="4" t="s">
+        <v>1310</v>
+      </c>
+      <c r="F81" s="4" t="s">
+        <v>1335</v>
+      </c>
+      <c r="G81" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J81" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="K81" s="4">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A82" s="4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B82" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C82" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D82" s="4" t="s">
+        <v>1311</v>
+      </c>
+      <c r="F82" s="4" t="s">
+        <v>1336</v>
+      </c>
+      <c r="G82" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J82" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="K82" s="4">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A83" s="4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B83" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C83" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D83" s="4" t="s">
+        <v>1312</v>
+      </c>
+      <c r="F83" s="4" t="s">
+        <v>1337</v>
+      </c>
+      <c r="G83" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J83" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="K83" s="4">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" ht="51" x14ac:dyDescent="0.2">
+      <c r="A84" s="4" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B84" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="C84" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D84" s="4" t="s">
+        <v>1313</v>
+      </c>
+      <c r="F84" s="4" t="s">
+        <v>1338</v>
+      </c>
+      <c r="G84" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J84" s="2" t="s">
+        <v>1099</v>
+      </c>
+      <c r="K84" s="4">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>1350</v>
+      </c>
+      <c r="B88" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C88" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D88" s="4" t="s">
+        <v>1361</v>
+      </c>
+      <c r="G88" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="K88" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>1350</v>
+      </c>
+      <c r="B89" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C89" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E89" s="37" t="s">
+        <v>1362</v>
+      </c>
+      <c r="G89" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="K89" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
+        <v>1350</v>
+      </c>
+      <c r="B90" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C90" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E90" s="37" t="s">
+        <v>1363</v>
+      </c>
+      <c r="G90" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="K90" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="91" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>1350</v>
+      </c>
+      <c r="B91" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C91" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="E91" s="37" t="s">
+        <v>1364</v>
+      </c>
+      <c r="G91" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="K91" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="92" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+      <c r="A92" t="s">
+        <v>1350</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C92" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D92" s="4" t="s">
+        <v>1353</v>
+      </c>
+      <c r="E92" s="2" t="s">
+        <v>1365</v>
+      </c>
+      <c r="G92" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="K92" s="4">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="93" spans="1:11" ht="68" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
+        <v>1350</v>
+      </c>
+      <c r="B93" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C93" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="E93" s="2" t="s">
+        <v>1354</v>
+      </c>
+      <c r="G93" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="K93" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="94" spans="1:11" ht="34" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
+        <v>1350</v>
+      </c>
+      <c r="B94" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C94" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="E94" s="2" t="s">
+        <v>1355</v>
+      </c>
+      <c r="G94" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="K94" s="4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="95" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
+        <v>1350</v>
+      </c>
+      <c r="B95" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C95" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="E95" s="2" t="s">
+        <v>1356</v>
+      </c>
+      <c r="G95" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="K95" s="4">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="96" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+      <c r="A96" t="s">
+        <v>1350</v>
+      </c>
+      <c r="B96" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C96" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="E96" s="2" t="s">
+        <v>1357</v>
+      </c>
+      <c r="G96" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="K96" s="4">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="97" spans="1:11" ht="17" x14ac:dyDescent="0.2">
+      <c r="A97" t="s">
+        <v>1350</v>
+      </c>
+      <c r="B97" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C97" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="E97" s="2" t="s">
+        <v>1358</v>
+      </c>
+      <c r="G97" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="K97" s="4">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A98" t="s">
+        <v>1350</v>
+      </c>
+      <c r="B98" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C98" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="D98" s="4" t="s">
+        <v>1359</v>
+      </c>
+      <c r="E98" s="36" t="s">
+        <v>1360</v>
+      </c>
+      <c r="G98" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="K98" s="4">
+        <v>10</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E98" r:id="rId1" xr:uid="{0ACED111-27C4-D24A-8D2D-292F7EF8BCCB}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -10311,15 +11513,15 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C62D4F70-2351-5545-A291-11D662F747FD}">
-  <dimension ref="A1:L1072"/>
+  <dimension ref="A1:L1093"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="16.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="25.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6.6640625" style="27" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="3.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="54.33203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="35.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="24.33203125" customWidth="1"/>
+    <col min="6" max="6" width="7.6640625" customWidth="1"/>
     <col min="7" max="7" width="32.5" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="4.5" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6.33203125" bestFit="1" customWidth="1"/>
@@ -29615,6 +30817,204 @@
         <v>108</v>
       </c>
     </row>
+    <row r="1078" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1078" s="4" t="s">
+        <v>1287</v>
+      </c>
+      <c r="B1078" s="27">
+        <v>1</v>
+      </c>
+      <c r="C1078" t="s">
+        <v>1343</v>
+      </c>
+      <c r="L1078" t="s">
+        <v>1344</v>
+      </c>
+    </row>
+    <row r="1079" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1079" s="4" t="s">
+        <v>1287</v>
+      </c>
+      <c r="B1079" s="27">
+        <v>1</v>
+      </c>
+      <c r="C1079" t="s">
+        <v>1286</v>
+      </c>
+      <c r="E1079" t="s">
+        <v>1340</v>
+      </c>
+      <c r="G1079" t="s">
+        <v>1339</v>
+      </c>
+      <c r="H1079" t="s">
+        <v>113</v>
+      </c>
+      <c r="L1079" t="str">
+        <f t="shared" ref="L1079" si="140">_xlfn.TEXTJOIN("", TRUE, D1079:K1079)</f>
+        <v>03_Hieroglyphen-selten/F63_xnty_01.png</v>
+      </c>
+    </row>
+    <row r="1080" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1080" s="4" t="s">
+        <v>1287</v>
+      </c>
+      <c r="B1080" s="27">
+        <v>1</v>
+      </c>
+      <c r="C1080" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1080" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="1081" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1081" s="4" t="s">
+        <v>1287</v>
+      </c>
+      <c r="B1081" s="27">
+        <v>1</v>
+      </c>
+      <c r="C1081" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1081" t="s">
+        <v>1342</v>
+      </c>
+    </row>
+    <row r="1086" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1086" s="4" t="s">
+        <v>1325</v>
+      </c>
+      <c r="B1086" s="27">
+        <v>1</v>
+      </c>
+      <c r="C1086" t="s">
+        <v>1343</v>
+      </c>
+      <c r="L1086" t="s">
+        <v>1345</v>
+      </c>
+    </row>
+    <row r="1087" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1087" s="4" t="s">
+        <v>1325</v>
+      </c>
+      <c r="B1087" s="27">
+        <v>1</v>
+      </c>
+      <c r="C1087" t="s">
+        <v>1286</v>
+      </c>
+      <c r="E1087" t="s">
+        <v>1340</v>
+      </c>
+      <c r="G1087" t="s">
+        <v>1346</v>
+      </c>
+      <c r="H1087" t="s">
+        <v>113</v>
+      </c>
+      <c r="L1087" t="str">
+        <f t="shared" ref="L1087" si="141">_xlfn.TEXTJOIN("", TRUE, D1087:K1087)</f>
+        <v>03_Hieroglyphen-selten/N6B_nsw-bjt_01.png</v>
+      </c>
+    </row>
+    <row r="1088" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1088" s="4" t="s">
+        <v>1325</v>
+      </c>
+      <c r="B1088" s="27">
+        <v>1</v>
+      </c>
+      <c r="C1088" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1088" t="s">
+        <v>528</v>
+      </c>
+    </row>
+    <row r="1089" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1089" s="4" t="s">
+        <v>1325</v>
+      </c>
+      <c r="B1089" s="27">
+        <v>1</v>
+      </c>
+      <c r="C1089" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1089" t="s">
+        <v>1347</v>
+      </c>
+    </row>
+    <row r="1090" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1090" s="4" t="s">
+        <v>1325</v>
+      </c>
+      <c r="B1090" s="27">
+        <v>2</v>
+      </c>
+      <c r="C1090" t="s">
+        <v>1343</v>
+      </c>
+      <c r="L1090" t="s">
+        <v>1349</v>
+      </c>
+    </row>
+    <row r="1091" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1091" s="4" t="s">
+        <v>1325</v>
+      </c>
+      <c r="B1091" s="27">
+        <v>2</v>
+      </c>
+      <c r="C1091" t="s">
+        <v>1286</v>
+      </c>
+      <c r="E1091" t="s">
+        <v>1340</v>
+      </c>
+      <c r="G1091" t="s">
+        <v>1348</v>
+      </c>
+      <c r="H1091" t="s">
+        <v>113</v>
+      </c>
+      <c r="L1091" t="str">
+        <f t="shared" ref="L1091" si="142">_xlfn.TEXTJOIN("", TRUE, D1091:K1091)</f>
+        <v>03_Hieroglyphen-selten/N102_jmn_01.png</v>
+      </c>
+    </row>
+    <row r="1092" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1092" s="4" t="s">
+        <v>1325</v>
+      </c>
+      <c r="B1092" s="27">
+        <v>2</v>
+      </c>
+      <c r="C1092" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1092" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="1093" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1093" s="4" t="s">
+        <v>1325</v>
+      </c>
+      <c r="B1093" s="27">
+        <v>2</v>
+      </c>
+      <c r="C1093" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1093" t="s">
+        <v>112</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <ignoredErrors>

</xml_diff>

<commit_message>
more spacing between hieroglyphs in table and variants
</commit_message>
<xml_diff>
--- a/data/content.xlsx
+++ b/data/content.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Markus/Documents/Arbeit/Inschriftenschluessel/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D33B314-41E0-BC4B-A3AD-B9FAFA5F237B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{130B32DD-00A9-154D-B757-5DC8FD20783D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2640" yWindow="500" windowWidth="21640" windowHeight="19440" activeTab="3" xr2:uid="{F025A444-F8B0-5C41-A37E-BEE791B22240}"/>
   </bookViews>
@@ -4130,9 +4130,6 @@
     <t>Mitarbeiter:</t>
   </si>
   <si>
-    <t>- **Projektleitung:** Prof. Friedhelm Hoffmann</t>
-  </si>
-  <si>
     <t>- **Recherche, Datengrundlage:** Iulia Comșa</t>
   </si>
   <si>
@@ -4140,6 +4137,9 @@
   </si>
   <si>
     <t>Diese Website wurde mit Quarto unter R erstellt:</t>
+  </si>
+  <si>
+    <t>- **Projektleitung:** Prof. Dr. Friedhelm Hoffmann</t>
   </si>
 </sst>
 </file>
@@ -4250,7 +4250,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -4315,10 +4315,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -7312,8 +7308,8 @@
       <c r="C89" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="E89" s="37" t="s">
-        <v>1362</v>
+      <c r="E89" s="33" t="s">
+        <v>1365</v>
       </c>
       <c r="G89" s="4" t="s">
         <v>54</v>
@@ -7332,8 +7328,8 @@
       <c r="C90" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="E90" s="37" t="s">
-        <v>1363</v>
+      <c r="E90" s="33" t="s">
+        <v>1362</v>
       </c>
       <c r="G90" s="4" t="s">
         <v>54</v>
@@ -7352,8 +7348,8 @@
       <c r="C91" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="E91" s="37" t="s">
-        <v>1364</v>
+      <c r="E91" s="33" t="s">
+        <v>1363</v>
       </c>
       <c r="G91" s="4" t="s">
         <v>54</v>
@@ -7376,7 +7372,7 @@
         <v>1353</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>1365</v>
+        <v>1364</v>
       </c>
       <c r="G92" s="4" t="s">
         <v>54</v>
@@ -7498,7 +7494,7 @@
       <c r="D98" s="4" t="s">
         <v>1359</v>
       </c>
-      <c r="E98" s="36" t="s">
+      <c r="E98" s="32" t="s">
         <v>1360</v>
       </c>
       <c r="G98" s="4" t="s">
@@ -12422,7 +12418,7 @@
         <v>113</v>
       </c>
       <c r="L57" t="str">
-        <f t="shared" ref="L55:L58" si="8">_xlfn.TEXTJOIN("", TRUE, D57:J57)</f>
+        <f t="shared" ref="L57:L58" si="8">_xlfn.TEXTJOIN("", TRUE, D57:J57)</f>
         <v>02_Slots/Gaben/0030_Gefluegel/0020_Apd_Abk_02.png</v>
       </c>
     </row>
@@ -17821,16 +17817,15 @@
       </c>
     </row>
     <row r="361" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A361" s="32" t="s">
+      <c r="A361" t="s">
         <v>1030</v>
       </c>
-      <c r="B361" s="35">
+      <c r="B361" s="27">
         <v>2</v>
       </c>
-      <c r="C361" s="32" t="s">
-        <v>105</v>
-      </c>
-      <c r="D361" s="32"/>
+      <c r="C361" t="s">
+        <v>105</v>
+      </c>
       <c r="E361" t="s">
         <v>1223</v>
       </c>
@@ -17855,76 +17850,43 @@
       </c>
     </row>
     <row r="362" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A362" s="32" t="s">
+      <c r="A362" t="s">
         <v>1030</v>
       </c>
-      <c r="B362" s="35">
+      <c r="B362" s="27">
         <v>2</v>
       </c>
-      <c r="C362" s="32" t="s">
+      <c r="C362" t="s">
         <v>27</v>
       </c>
-      <c r="D362" s="32"/>
       <c r="L362" t="s">
         <v>1093</v>
       </c>
     </row>
-    <row r="363" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A363" s="32"/>
-      <c r="B363" s="35"/>
-      <c r="C363" s="32"/>
-      <c r="D363" s="32"/>
-    </row>
-    <row r="364" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A364" s="32"/>
-      <c r="B364" s="35"/>
-      <c r="C364" s="32"/>
-      <c r="D364" s="32"/>
-    </row>
-    <row r="365" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A365" s="32"/>
-      <c r="B365" s="35"/>
-      <c r="C365" s="32"/>
-      <c r="D365" s="32"/>
-    </row>
-    <row r="366" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A366" s="32"/>
-      <c r="B366" s="35"/>
-      <c r="C366" s="32"/>
-      <c r="D366" s="32"/>
-    </row>
-    <row r="367" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A367" s="32"/>
-      <c r="B367" s="35"/>
-      <c r="C367" s="32"/>
-      <c r="D367" s="32"/>
-    </row>
     <row r="368" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A368" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B368" s="33">
+      <c r="A368" t="s">
+        <v>60</v>
+      </c>
+      <c r="B368" s="28">
         <v>20</v>
       </c>
-      <c r="C368" s="32" t="s">
+      <c r="C368" t="s">
         <v>39</v>
       </c>
-      <c r="D368" s="32"/>
       <c r="L368" t="s">
         <v>177</v>
       </c>
     </row>
     <row r="369" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A369" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B369" s="33">
+      <c r="A369" t="s">
+        <v>60</v>
+      </c>
+      <c r="B369" s="28">
         <v>20</v>
       </c>
-      <c r="C369" s="32" t="s">
-        <v>105</v>
-      </c>
-      <c r="D369" s="32"/>
+      <c r="C369" t="s">
+        <v>105</v>
+      </c>
       <c r="E369" t="s">
         <v>1224</v>
       </c>
@@ -17940,16 +17902,15 @@
       </c>
     </row>
     <row r="370" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A370" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B370" s="33">
+      <c r="A370" t="s">
+        <v>60</v>
+      </c>
+      <c r="B370" s="28">
         <v>20</v>
       </c>
-      <c r="C370" s="32" t="s">
-        <v>105</v>
-      </c>
-      <c r="D370" s="32"/>
+      <c r="C370" t="s">
+        <v>105</v>
+      </c>
       <c r="E370" t="s">
         <v>1224</v>
       </c>
@@ -17974,16 +17935,15 @@
       </c>
     </row>
     <row r="371" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A371" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B371" s="33">
+      <c r="A371" t="s">
+        <v>60</v>
+      </c>
+      <c r="B371" s="28">
         <v>20</v>
       </c>
-      <c r="C371" s="32" t="s">
-        <v>105</v>
-      </c>
-      <c r="D371" s="32"/>
+      <c r="C371" t="s">
+        <v>105</v>
+      </c>
       <c r="E371" t="s">
         <v>1224</v>
       </c>
@@ -18008,16 +17968,15 @@
       </c>
     </row>
     <row r="372" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A372" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B372" s="33">
+      <c r="A372" t="s">
+        <v>60</v>
+      </c>
+      <c r="B372" s="28">
         <v>20</v>
       </c>
-      <c r="C372" s="32" t="s">
+      <c r="C372" t="s">
         <v>106</v>
       </c>
-      <c r="D372" s="32"/>
       <c r="E372" t="s">
         <v>1224</v>
       </c>
@@ -18036,67 +17995,57 @@
       </c>
     </row>
     <row r="373" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A373" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B373" s="33">
+      <c r="A373" t="s">
+        <v>60</v>
+      </c>
+      <c r="B373" s="28">
         <v>20</v>
       </c>
-      <c r="C373" s="32" t="s">
+      <c r="C373" t="s">
         <v>107</v>
       </c>
-      <c r="D373" s="32"/>
       <c r="L373" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="374" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A374" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B374" s="33">
+      <c r="A374" t="s">
+        <v>60</v>
+      </c>
+      <c r="B374" s="28">
         <v>20</v>
       </c>
-      <c r="C374" s="32" t="s">
+      <c r="C374" t="s">
         <v>108</v>
       </c>
-      <c r="D374" s="32"/>
       <c r="L374" t="s">
         <v>1170</v>
       </c>
     </row>
-    <row r="375" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A375" s="32"/>
-      <c r="B375" s="35"/>
-      <c r="C375" s="32"/>
-      <c r="D375" s="32"/>
-    </row>
     <row r="376" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A376" s="32" t="s">
+      <c r="A376" t="s">
         <v>610</v>
       </c>
-      <c r="B376" s="35">
+      <c r="B376" s="27">
         <v>1</v>
       </c>
-      <c r="C376" s="32" t="s">
+      <c r="C376" t="s">
         <v>39</v>
       </c>
-      <c r="D376" s="32"/>
       <c r="L376" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="377" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A377" s="32" t="s">
+      <c r="A377" t="s">
         <v>610</v>
       </c>
-      <c r="B377" s="35">
+      <c r="B377" s="27">
         <v>1</v>
       </c>
-      <c r="C377" s="32" t="s">
-        <v>105</v>
-      </c>
-      <c r="D377" s="32"/>
+      <c r="C377" t="s">
+        <v>105</v>
+      </c>
       <c r="E377" t="s">
         <v>110</v>
       </c>
@@ -18115,38 +18064,29 @@
       </c>
     </row>
     <row r="378" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A378" s="32" t="s">
+      <c r="A378" t="s">
         <v>610</v>
       </c>
-      <c r="B378" s="35">
+      <c r="B378" s="27">
         <v>1</v>
       </c>
-      <c r="C378" s="32" t="s">
+      <c r="C378" t="s">
         <v>27</v>
       </c>
-      <c r="D378" s="32"/>
       <c r="L378" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="379" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A379" s="32"/>
-      <c r="B379" s="35"/>
-      <c r="C379" s="32"/>
-      <c r="D379" s="32"/>
-    </row>
     <row r="380" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A380" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B380" s="34">
+      <c r="A380" t="s">
+        <v>60</v>
+      </c>
+      <c r="B380" s="28">
         <v>30</v>
       </c>
-      <c r="C380" s="32" t="s">
+      <c r="C380" t="s">
         <v>39</v>
       </c>
-      <c r="D380" s="32"/>
-      <c r="E380" s="32"/>
       <c r="G380" t="s">
         <v>127</v>
       </c>
@@ -18155,17 +18095,16 @@
       </c>
     </row>
     <row r="381" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A381" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B381" s="34">
+      <c r="A381" t="s">
+        <v>60</v>
+      </c>
+      <c r="B381" s="28">
         <v>30</v>
       </c>
-      <c r="C381" s="32" t="s">
-        <v>105</v>
-      </c>
-      <c r="D381" s="32"/>
-      <c r="E381" s="32" t="s">
+      <c r="C381" t="s">
+        <v>105</v>
+      </c>
+      <c r="E381" t="s">
         <v>1225</v>
       </c>
       <c r="G381" t="s">
@@ -18180,82 +18119,69 @@
       </c>
     </row>
     <row r="382" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A382" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B382" s="34">
+      <c r="A382" t="s">
+        <v>60</v>
+      </c>
+      <c r="B382" s="28">
         <v>30</v>
       </c>
-      <c r="C382" s="32" t="s">
+      <c r="C382" t="s">
         <v>106</v>
       </c>
-      <c r="D382" s="32"/>
-      <c r="E382" s="32"/>
     </row>
     <row r="383" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A383" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B383" s="34">
+      <c r="A383" t="s">
+        <v>60</v>
+      </c>
+      <c r="B383" s="28">
         <v>30</v>
       </c>
-      <c r="C383" s="32" t="s">
+      <c r="C383" t="s">
         <v>107</v>
       </c>
-      <c r="D383" s="32"/>
-      <c r="E383" s="32"/>
       <c r="L383" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="384" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A384" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B384" s="34">
+      <c r="A384" t="s">
+        <v>60</v>
+      </c>
+      <c r="B384" s="28">
         <v>30</v>
       </c>
-      <c r="C384" s="32" t="s">
+      <c r="C384" t="s">
         <v>108</v>
       </c>
-      <c r="D384" s="32"/>
-      <c r="E384" s="32"/>
     </row>
     <row r="385" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A385" s="32"/>
-      <c r="B385" s="33"/>
-      <c r="C385" s="32"/>
-      <c r="D385" s="32"/>
-      <c r="E385" s="32"/>
+      <c r="B385" s="28"/>
     </row>
     <row r="386" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A386" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B386" s="33">
+      <c r="A386" t="s">
+        <v>60</v>
+      </c>
+      <c r="B386" s="28">
         <v>40</v>
       </c>
-      <c r="C386" s="32" t="s">
+      <c r="C386" t="s">
         <v>39</v>
       </c>
-      <c r="D386" s="32"/>
-      <c r="E386" s="32"/>
       <c r="L386" t="s">
         <v>1228</v>
       </c>
     </row>
     <row r="387" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A387" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B387" s="33">
+      <c r="A387" t="s">
+        <v>60</v>
+      </c>
+      <c r="B387" s="28">
         <v>40</v>
       </c>
-      <c r="C387" s="32" t="s">
-        <v>105</v>
-      </c>
-      <c r="D387" s="32"/>
-      <c r="E387" s="32" t="s">
+      <c r="C387" t="s">
+        <v>105</v>
+      </c>
+      <c r="E387" t="s">
         <v>1226</v>
       </c>
       <c r="G387" t="s">
@@ -18270,82 +18196,69 @@
       </c>
     </row>
     <row r="388" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A388" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B388" s="33">
+      <c r="A388" t="s">
+        <v>60</v>
+      </c>
+      <c r="B388" s="28">
         <v>40</v>
       </c>
-      <c r="C388" s="32" t="s">
+      <c r="C388" t="s">
         <v>106</v>
       </c>
-      <c r="D388" s="32"/>
-      <c r="E388" s="32"/>
     </row>
     <row r="389" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A389" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B389" s="33">
+      <c r="A389" t="s">
+        <v>60</v>
+      </c>
+      <c r="B389" s="28">
         <v>40</v>
       </c>
-      <c r="C389" s="32" t="s">
+      <c r="C389" t="s">
         <v>107</v>
       </c>
-      <c r="D389" s="32"/>
-      <c r="E389" s="32"/>
       <c r="L389" t="s">
         <v>129</v>
       </c>
     </row>
     <row r="390" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A390" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B390" s="33">
+      <c r="A390" t="s">
+        <v>60</v>
+      </c>
+      <c r="B390" s="28">
         <v>40</v>
       </c>
-      <c r="C390" s="32" t="s">
+      <c r="C390" t="s">
         <v>108</v>
       </c>
-      <c r="D390" s="32"/>
-      <c r="E390" s="32"/>
     </row>
     <row r="391" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A391" s="32"/>
-      <c r="B391" s="33"/>
-      <c r="C391" s="32"/>
-      <c r="D391" s="32"/>
-      <c r="E391" s="32"/>
+      <c r="B391" s="28"/>
     </row>
     <row r="392" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A392" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B392" s="33">
+      <c r="A392" t="s">
+        <v>60</v>
+      </c>
+      <c r="B392" s="28">
         <v>50</v>
       </c>
-      <c r="C392" s="32" t="s">
+      <c r="C392" t="s">
         <v>39</v>
       </c>
-      <c r="D392" s="32"/>
-      <c r="E392" s="32"/>
       <c r="L392" t="s">
         <v>588</v>
       </c>
     </row>
     <row r="393" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A393" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B393" s="33">
+      <c r="A393" t="s">
+        <v>60</v>
+      </c>
+      <c r="B393" s="28">
         <v>50</v>
       </c>
-      <c r="C393" s="32" t="s">
-        <v>105</v>
-      </c>
-      <c r="D393" s="32"/>
-      <c r="E393" s="32" t="s">
+      <c r="C393" t="s">
+        <v>105</v>
+      </c>
+      <c r="E393" t="s">
         <v>1229</v>
       </c>
       <c r="G393" t="s">
@@ -18360,17 +18273,16 @@
       </c>
     </row>
     <row r="394" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A394" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B394" s="33">
+      <c r="A394" t="s">
+        <v>60</v>
+      </c>
+      <c r="B394" s="28">
         <v>50</v>
       </c>
-      <c r="C394" s="32" t="s">
-        <v>105</v>
-      </c>
-      <c r="D394" s="32"/>
-      <c r="E394" s="32" t="s">
+      <c r="C394" t="s">
+        <v>105</v>
+      </c>
+      <c r="E394" t="s">
         <v>1229</v>
       </c>
       <c r="G394" t="s">
@@ -18385,17 +18297,16 @@
       </c>
     </row>
     <row r="395" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A395" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B395" s="33">
+      <c r="A395" t="s">
+        <v>60</v>
+      </c>
+      <c r="B395" s="28">
         <v>50</v>
       </c>
-      <c r="C395" s="32" t="s">
-        <v>105</v>
-      </c>
-      <c r="D395" s="32"/>
-      <c r="E395" s="32" t="s">
+      <c r="C395" t="s">
+        <v>105</v>
+      </c>
+      <c r="E395" t="s">
         <v>1229</v>
       </c>
       <c r="G395" t="s">
@@ -18410,17 +18321,16 @@
       </c>
     </row>
     <row r="396" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A396" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B396" s="33">
+      <c r="A396" t="s">
+        <v>60</v>
+      </c>
+      <c r="B396" s="28">
         <v>50</v>
       </c>
-      <c r="C396" s="32" t="s">
-        <v>105</v>
-      </c>
-      <c r="D396" s="32"/>
-      <c r="E396" s="32" t="s">
+      <c r="C396" t="s">
+        <v>105</v>
+      </c>
+      <c r="E396" t="s">
         <v>1229</v>
       </c>
       <c r="G396" t="s">
@@ -18444,17 +18354,16 @@
       </c>
     </row>
     <row r="397" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A397" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B397" s="33">
+      <c r="A397" t="s">
+        <v>60</v>
+      </c>
+      <c r="B397" s="28">
         <v>50</v>
       </c>
-      <c r="C397" s="32" t="s">
-        <v>105</v>
-      </c>
-      <c r="D397" s="32"/>
-      <c r="E397" s="32" t="s">
+      <c r="C397" t="s">
+        <v>105</v>
+      </c>
+      <c r="E397" t="s">
         <v>1229</v>
       </c>
       <c r="G397" t="s">
@@ -18478,17 +18387,16 @@
       </c>
     </row>
     <row r="398" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A398" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B398" s="33">
+      <c r="A398" t="s">
+        <v>60</v>
+      </c>
+      <c r="B398" s="28">
         <v>50</v>
       </c>
-      <c r="C398" s="32" t="s">
-        <v>105</v>
-      </c>
-      <c r="D398" s="32"/>
-      <c r="E398" s="32" t="s">
+      <c r="C398" t="s">
+        <v>105</v>
+      </c>
+      <c r="E398" t="s">
         <v>1229</v>
       </c>
       <c r="G398" t="s">
@@ -18512,17 +18420,16 @@
       </c>
     </row>
     <row r="399" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A399" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B399" s="33">
+      <c r="A399" t="s">
+        <v>60</v>
+      </c>
+      <c r="B399" s="28">
         <v>50</v>
       </c>
-      <c r="C399" s="32" t="s">
-        <v>105</v>
-      </c>
-      <c r="D399" s="32"/>
-      <c r="E399" s="32" t="s">
+      <c r="C399" t="s">
+        <v>105</v>
+      </c>
+      <c r="E399" t="s">
         <v>1229</v>
       </c>
       <c r="G399" t="s">
@@ -18546,30 +18453,26 @@
       </c>
     </row>
     <row r="400" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A400" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B400" s="33">
+      <c r="A400" t="s">
+        <v>60</v>
+      </c>
+      <c r="B400" s="28">
         <v>50</v>
       </c>
-      <c r="C400" s="32" t="s">
+      <c r="C400" t="s">
         <v>106</v>
       </c>
-      <c r="D400" s="32"/>
-      <c r="E400" s="32"/>
     </row>
     <row r="401" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A401" s="32" t="s">
-        <v>60</v>
-      </c>
-      <c r="B401" s="33">
+      <c r="A401" t="s">
+        <v>60</v>
+      </c>
+      <c r="B401" s="28">
         <v>50</v>
       </c>
-      <c r="C401" s="32" t="s">
+      <c r="C401" t="s">
         <v>107</v>
       </c>
-      <c r="D401" s="32"/>
-      <c r="E401" s="32"/>
       <c r="L401" t="s">
         <v>130</v>
       </c>

</xml_diff>

<commit_message>
fixed column width of wide tables
</commit_message>
<xml_diff>
--- a/data/content.xlsx
+++ b/data/content.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Markus/Documents/Arbeit/Inschriftenschluessel/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{130B32DD-00A9-154D-B757-5DC8FD20783D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB992A9E-A7CD-8D47-8644-ABE40EEF4031}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2640" yWindow="500" windowWidth="21640" windowHeight="19440" activeTab="3" xr2:uid="{F025A444-F8B0-5C41-A37E-BEE791B22240}"/>
+    <workbookView xWindow="-23400" yWindow="500" windowWidth="21640" windowHeight="17500" activeTab="3" xr2:uid="{F025A444-F8B0-5C41-A37E-BEE791B22240}"/>
   </bookViews>
   <sheets>
     <sheet name="pages" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
added Beischrift slot variant to jn
</commit_message>
<xml_diff>
--- a/data/content.xlsx
+++ b/data/content.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Markus/Documents/Arbeit/Inschriftenschluessel/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9791674-86FC-9044-9746-58D43CD73EB0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37BCE710-6790-D84E-9B89-45738A059ACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16200" activeTab="4" xr2:uid="{F025A444-F8B0-5C41-A37E-BEE791B22240}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="18380" windowHeight="16200" activeTab="4" xr2:uid="{F025A444-F8B0-5C41-A37E-BEE791B22240}"/>
   </bookViews>
   <sheets>
     <sheet name="pages" sheetId="1" r:id="rId1"/>

</xml_diff>

<commit_message>
added Khonsu epithet m wAs.t and pA jrj sxr.w m wAs.t
</commit_message>
<xml_diff>
--- a/data/content.xlsx
+++ b/data/content.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Markus/Documents/Arbeit/Inschriftenschluessel/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57E2934E-3A32-3D4B-9D3E-E27ED654FC13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2A65100-16B1-4D45-93E5-4AADA291EF01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="19840" activeTab="4" xr2:uid="{F025A444-F8B0-5C41-A37E-BEE791B22240}"/>
+    <workbookView xWindow="-28800" yWindow="500" windowWidth="28800" windowHeight="17500" activeTab="5" xr2:uid="{F025A444-F8B0-5C41-A37E-BEE791B22240}"/>
   </bookViews>
   <sheets>
     <sheet name="pages" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6721" uniqueCount="1502">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6758" uniqueCount="1513">
   <si>
     <t>page_id</t>
   </si>
@@ -4572,6 +4572,39 @@
   <si>
     <t>0070_mw.t_Sp_01.png</t>
   </si>
+  <si>
+    <t>[[table:tb_epith_chons_001|Öffne]]</t>
+  </si>
+  <si>
+    <t>tb_epith_chons_001</t>
+  </si>
+  <si>
+    <t>0001_m-WAs.t_NR_01.png</t>
+  </si>
+  <si>
+    <t>0010_m-WAs.t_NR_02.png</t>
+  </si>
+  <si>
+    <t>epitheta/01-m-wAs.t/</t>
+  </si>
+  <si>
+    <t>*m wꜣs.t*</t>
+  </si>
+  <si>
+    <t>in Theben</t>
+  </si>
+  <si>
+    <t>*pꜣ iri sḫr.w m wꜣs.t*</t>
+  </si>
+  <si>
+    <t>der die Pläne in Theben macht</t>
+  </si>
+  <si>
+    <t>0001_pA-jrj-sxr.w-m-WAs.t_Sp_01.png</t>
+  </si>
+  <si>
+    <t>epitheta/02-pA-jrj-sxr.w-m-WAs.t/</t>
+  </si>
 </sst>
 </file>
 
@@ -4580,7 +4613,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0000"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -4621,6 +4654,13 @@
       <i/>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -4695,7 +4735,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -4781,6 +4821,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
@@ -5740,7 +5781,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:6" s="7" customFormat="1" ht="136" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" s="7" customFormat="1" ht="119" x14ac:dyDescent="0.2">
       <c r="A10" s="7" t="s">
         <v>62</v>
       </c>
@@ -10221,7 +10262,7 @@
         <v>1501</v>
       </c>
       <c r="L76" s="6" t="str">
-        <f t="shared" ref="L76:L77" si="12">_xlfn.TEXTJOIN("", TRUE, E76:K76)</f>
+        <f t="shared" ref="L76" si="12">_xlfn.TEXTJOIN("", TRUE, E76:K76)</f>
         <v>01_Textgattung/02_Denkmaelerformel/03-1_mw.t/0070_mw.t_Sp_01.png</v>
       </c>
       <c r="N76" s="6" t="s">
@@ -14493,16 +14534,16 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C62D4F70-2351-5545-A291-11D662F747FD}">
-  <dimension ref="A1:L1135"/>
+  <dimension ref="A1:L1148"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="16.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="25.83203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6.6640625" style="27" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="22.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="3.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="26.1640625" customWidth="1"/>
-    <col min="6" max="6" width="24.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24" customWidth="1"/>
+    <col min="5" max="5" width="46.5" customWidth="1"/>
+    <col min="6" max="6" width="20.5" customWidth="1"/>
+    <col min="7" max="7" width="30" customWidth="1"/>
     <col min="8" max="8" width="4.5" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="6.33203125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12.33203125" bestFit="1" customWidth="1"/>
@@ -32370,7 +32411,7 @@
         <v>955</v>
       </c>
       <c r="L992" t="str">
-        <f>_xlfn.TEXTJOIN("", TRUE, D992:J992)</f>
+        <f t="shared" ref="L992:L993" si="129">_xlfn.TEXTJOIN("", TRUE, D992:K992)</f>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0360_Chons/0001_Xnsw_01.png</v>
       </c>
     </row>
@@ -32391,7 +32432,7 @@
         <v>956</v>
       </c>
       <c r="L993" t="str">
-        <f>_xlfn.TEXTJOIN("", TRUE, D993:J993)</f>
+        <f t="shared" si="129"/>
         <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0360_Chons/0010_Xnsw_02.png</v>
       </c>
     </row>
@@ -32464,238 +32505,195 @@
       <c r="C997" t="s">
         <v>108</v>
       </c>
+      <c r="L997" s="39" t="s">
+        <v>1502</v>
+      </c>
+    </row>
+    <row r="998" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="L998" s="39"/>
+    </row>
+    <row r="999" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A999" t="s">
+        <v>1503</v>
+      </c>
+      <c r="B999" s="27">
+        <v>1</v>
+      </c>
+      <c r="C999" t="s">
+        <v>39</v>
+      </c>
+      <c r="L999" s="39" t="s">
+        <v>1507</v>
+      </c>
     </row>
     <row r="1000" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1000" t="s">
-        <v>60</v>
+        <v>1503</v>
       </c>
       <c r="B1000" s="27">
-        <v>370</v>
+        <v>1</v>
       </c>
       <c r="C1000" t="s">
-        <v>39</v>
-      </c>
-      <c r="L1000" t="s">
-        <v>678</v>
+        <v>105</v>
+      </c>
+      <c r="E1000" t="s">
+        <v>1209</v>
+      </c>
+      <c r="F1000" t="s">
+        <v>1506</v>
+      </c>
+      <c r="G1000" t="s">
+        <v>1504</v>
+      </c>
+      <c r="I1000" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1000" t="s">
+        <v>1103</v>
+      </c>
+      <c r="K1000" t="s">
+        <v>1149</v>
+      </c>
+      <c r="L1000" t="str">
+        <f t="shared" ref="L1000:L1001" si="130">_xlfn.TEXTJOIN("", TRUE, D1000:K1000)</f>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0360_Chons/epitheta/01-m-wAs.t/0001_m-WAs.t_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1001" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1001" t="s">
-        <v>60</v>
+        <v>1503</v>
       </c>
       <c r="B1001" s="27">
-        <v>370</v>
+        <v>1</v>
       </c>
       <c r="C1001" t="s">
         <v>105</v>
       </c>
       <c r="E1001" t="s">
-        <v>1210</v>
+        <v>1209</v>
+      </c>
+      <c r="F1001" t="s">
+        <v>1506</v>
       </c>
       <c r="G1001" t="s">
-        <v>958</v>
+        <v>1505</v>
+      </c>
+      <c r="I1001" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1001" t="s">
+        <v>1103</v>
+      </c>
+      <c r="K1001" t="s">
+        <v>1149</v>
       </c>
       <c r="L1001" t="str">
-        <f>_xlfn.TEXTJOIN("", TRUE, D1001:J1001)</f>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0370_Sobek/0001_sbk_01.png</v>
+        <f t="shared" si="130"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0360_Chons/epitheta/01-m-wAs.t/0010_m-WAs.t_NR_02.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1002" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1002" t="s">
-        <v>60</v>
+        <v>1503</v>
       </c>
       <c r="B1002" s="27">
-        <v>370</v>
+        <v>1</v>
       </c>
       <c r="C1002" t="s">
-        <v>105</v>
-      </c>
-      <c r="E1002" t="s">
-        <v>1210</v>
-      </c>
-      <c r="G1002" t="s">
-        <v>959</v>
-      </c>
-      <c r="L1002" t="str">
-        <f>_xlfn.TEXTJOIN("", TRUE, D1002:J1002)</f>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0370_Sobek/0010_sbk_02.png</v>
+        <v>27</v>
+      </c>
+      <c r="L1002" s="39" t="s">
+        <v>1508</v>
       </c>
     </row>
     <row r="1003" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1003" t="s">
-        <v>60</v>
-      </c>
-      <c r="B1003" s="27">
-        <v>370</v>
-      </c>
-      <c r="C1003" t="s">
-        <v>105</v>
-      </c>
-      <c r="E1003" t="s">
-        <v>1210</v>
-      </c>
-      <c r="G1003" t="s">
-        <v>960</v>
-      </c>
-      <c r="L1003" t="str">
-        <f>_xlfn.TEXTJOIN("", TRUE, D1003:J1003)</f>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0370_Sobek/0020_sbk_03.png</v>
-      </c>
+      <c r="L1003" s="39"/>
     </row>
     <row r="1004" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1004" t="s">
-        <v>60</v>
+        <v>1503</v>
       </c>
       <c r="B1004" s="27">
-        <v>370</v>
+        <v>2</v>
       </c>
       <c r="C1004" t="s">
-        <v>105</v>
-      </c>
-      <c r="E1004" t="s">
-        <v>1210</v>
-      </c>
-      <c r="G1004" t="s">
-        <v>961</v>
-      </c>
-      <c r="I1004" t="s">
-        <v>1147</v>
-      </c>
-      <c r="J1004" t="s">
-        <v>1103</v>
-      </c>
-      <c r="K1004" t="s">
-        <v>1149</v>
-      </c>
-      <c r="L1004" t="str">
-        <f>_xlfn.TEXTJOIN("", TRUE, D1004:K1004)</f>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0370_Sobek/0030_sbk_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
+        <v>39</v>
+      </c>
+      <c r="L1004" s="39" t="s">
+        <v>1509</v>
       </c>
     </row>
     <row r="1005" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1005" t="s">
-        <v>60</v>
+        <v>1503</v>
       </c>
       <c r="B1005" s="27">
-        <v>370</v>
+        <v>2</v>
       </c>
       <c r="C1005" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E1005" t="s">
-        <v>1210</v>
+        <v>1209</v>
       </c>
       <c r="F1005" t="s">
-        <v>110</v>
+        <v>1512</v>
       </c>
       <c r="G1005" t="s">
-        <v>962</v>
+        <v>1511</v>
+      </c>
+      <c r="I1005" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1005" t="s">
+        <v>1156</v>
+      </c>
+      <c r="K1005" t="s">
+        <v>1149</v>
       </c>
       <c r="L1005" t="str">
-        <f>_xlfn.TEXTJOIN("", TRUE, D1005:J1005)</f>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0370_Sobek/det/0001_sbk_det_01.png</v>
+        <f t="shared" ref="L1005" si="131">_xlfn.TEXTJOIN("", TRUE, D1005:K1005)</f>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0360_Chons/epitheta/02-pA-jrj-sxr.w-m-WAs.t/0001_pA-jrj-sxr.w-m-WAs.t_Sp_01.png &lt;sup&gt;(Sp.)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1006" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1006" t="s">
-        <v>60</v>
+        <v>1503</v>
       </c>
       <c r="B1006" s="27">
-        <v>370</v>
+        <v>2</v>
       </c>
       <c r="C1006" t="s">
-        <v>107</v>
-      </c>
-      <c r="L1006" t="s">
-        <v>160</v>
+        <v>27</v>
+      </c>
+      <c r="L1006" s="39" t="s">
+        <v>1510</v>
       </c>
     </row>
     <row r="1007" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1007" t="s">
-        <v>60</v>
-      </c>
-      <c r="B1007" s="27">
-        <v>370</v>
-      </c>
-      <c r="C1007" t="s">
-        <v>108</v>
-      </c>
+      <c r="L1007" s="39"/>
+    </row>
+    <row r="1008" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="L1008" s="39"/>
+    </row>
+    <row r="1009" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="L1009" s="39"/>
     </row>
     <row r="1010" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1010" t="s">
-        <v>60</v>
-      </c>
-      <c r="B1010" s="27">
-        <v>380</v>
-      </c>
-      <c r="C1010" t="s">
-        <v>39</v>
-      </c>
-      <c r="L1010" t="s">
-        <v>679</v>
-      </c>
-    </row>
-    <row r="1011" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1011" t="s">
-        <v>60</v>
-      </c>
-      <c r="B1011" s="27">
-        <v>380</v>
-      </c>
-      <c r="C1011" t="s">
-        <v>105</v>
-      </c>
-      <c r="E1011" t="s">
-        <v>1211</v>
-      </c>
-      <c r="G1011" t="s">
-        <v>963</v>
-      </c>
-      <c r="L1011" t="str">
-        <f t="shared" ref="L1011:L1019" si="129">_xlfn.TEXTJOIN("", TRUE, D1011:J1011)</f>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0380_Selkis/0001_srq.t_01.png</v>
-      </c>
-    </row>
-    <row r="1012" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1012" t="s">
-        <v>60</v>
-      </c>
-      <c r="B1012" s="27">
-        <v>380</v>
-      </c>
-      <c r="C1012" t="s">
-        <v>105</v>
-      </c>
-      <c r="E1012" t="s">
-        <v>1211</v>
-      </c>
-      <c r="G1012" t="s">
-        <v>964</v>
-      </c>
-      <c r="L1012" t="str">
-        <f t="shared" si="129"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0380_Selkis/0010_srq.t_02.png</v>
-      </c>
+      <c r="L1010" s="39"/>
     </row>
     <row r="1013" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1013" t="s">
         <v>60</v>
       </c>
       <c r="B1013" s="27">
-        <v>380</v>
+        <v>370</v>
       </c>
       <c r="C1013" t="s">
-        <v>105</v>
-      </c>
-      <c r="E1013" t="s">
-        <v>1211</v>
-      </c>
-      <c r="G1013" t="s">
-        <v>965</v>
-      </c>
-      <c r="L1013" t="str">
-        <f t="shared" si="129"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0380_Selkis/0020_srq.t_03.png</v>
+        <v>39</v>
+      </c>
+      <c r="L1013" t="s">
+        <v>678</v>
       </c>
     </row>
     <row r="1014" spans="1:12" x14ac:dyDescent="0.2">
@@ -32703,29 +32701,20 @@
         <v>60</v>
       </c>
       <c r="B1014" s="27">
-        <v>380</v>
+        <v>370</v>
       </c>
       <c r="C1014" t="s">
         <v>105</v>
       </c>
       <c r="E1014" t="s">
-        <v>1211</v>
+        <v>1210</v>
       </c>
       <c r="G1014" t="s">
-        <v>966</v>
-      </c>
-      <c r="I1014" t="s">
-        <v>1147</v>
-      </c>
-      <c r="J1014" t="s">
-        <v>1164</v>
-      </c>
-      <c r="K1014" t="s">
-        <v>1149</v>
+        <v>958</v>
       </c>
       <c r="L1014" t="str">
-        <f t="shared" ref="L1014:L1017" si="130">_xlfn.TEXTJOIN("", TRUE, D1014:K1014)</f>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0380_Selkis/0030_srq.t_Pyr.-MR_01.png &lt;sup&gt;(Pyr.; NR)&lt;/sup&gt;</v>
+        <f>_xlfn.TEXTJOIN("", TRUE, D1014:J1014)</f>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0370_Sobek/0001_sbk_01.png</v>
       </c>
     </row>
     <row r="1015" spans="1:12" x14ac:dyDescent="0.2">
@@ -32733,29 +32722,20 @@
         <v>60</v>
       </c>
       <c r="B1015" s="27">
-        <v>380</v>
+        <v>370</v>
       </c>
       <c r="C1015" t="s">
         <v>105</v>
       </c>
       <c r="E1015" t="s">
-        <v>1211</v>
+        <v>1210</v>
       </c>
       <c r="G1015" t="s">
-        <v>967</v>
-      </c>
-      <c r="I1015" t="s">
-        <v>1147</v>
-      </c>
-      <c r="J1015" t="s">
-        <v>1150</v>
-      </c>
-      <c r="K1015" t="s">
-        <v>1149</v>
+        <v>959</v>
       </c>
       <c r="L1015" t="str">
-        <f t="shared" si="130"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0380_Selkis/0040_srq.t_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
+        <f>_xlfn.TEXTJOIN("", TRUE, D1015:J1015)</f>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0370_Sobek/0010_sbk_02.png</v>
       </c>
     </row>
     <row r="1016" spans="1:12" x14ac:dyDescent="0.2">
@@ -32763,29 +32743,20 @@
         <v>60</v>
       </c>
       <c r="B1016" s="27">
-        <v>380</v>
+        <v>370</v>
       </c>
       <c r="C1016" t="s">
         <v>105</v>
       </c>
       <c r="E1016" t="s">
-        <v>1211</v>
+        <v>1210</v>
       </c>
       <c r="G1016" t="s">
-        <v>968</v>
-      </c>
-      <c r="I1016" t="s">
-        <v>1147</v>
-      </c>
-      <c r="J1016" t="s">
-        <v>1150</v>
-      </c>
-      <c r="K1016" t="s">
-        <v>1149</v>
+        <v>960</v>
       </c>
       <c r="L1016" t="str">
-        <f t="shared" si="130"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0380_Selkis/0050_srq.t_GR_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
+        <f>_xlfn.TEXTJOIN("", TRUE, D1016:J1016)</f>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0370_Sobek/0020_sbk_03.png</v>
       </c>
     </row>
     <row r="1017" spans="1:12" x14ac:dyDescent="0.2">
@@ -32793,29 +32764,29 @@
         <v>60</v>
       </c>
       <c r="B1017" s="27">
-        <v>380</v>
+        <v>370</v>
       </c>
       <c r="C1017" t="s">
         <v>105</v>
       </c>
       <c r="E1017" t="s">
-        <v>1211</v>
+        <v>1210</v>
       </c>
       <c r="G1017" t="s">
-        <v>969</v>
+        <v>961</v>
       </c>
       <c r="I1017" t="s">
         <v>1147</v>
       </c>
       <c r="J1017" t="s">
-        <v>1150</v>
+        <v>1103</v>
       </c>
       <c r="K1017" t="s">
         <v>1149</v>
       </c>
       <c r="L1017" t="str">
-        <f t="shared" si="130"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0380_Selkis/0060_srq.t_GR_03.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
+        <f>_xlfn.TEXTJOIN("", TRUE, D1017:K1017)</f>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0370_Sobek/0030_sbk_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1018" spans="1:12" x14ac:dyDescent="0.2">
@@ -32823,23 +32794,23 @@
         <v>60</v>
       </c>
       <c r="B1018" s="27">
-        <v>380</v>
+        <v>370</v>
       </c>
       <c r="C1018" t="s">
         <v>106</v>
       </c>
       <c r="E1018" t="s">
-        <v>1211</v>
+        <v>1210</v>
       </c>
       <c r="F1018" t="s">
         <v>110</v>
       </c>
       <c r="G1018" t="s">
-        <v>970</v>
+        <v>962</v>
       </c>
       <c r="L1018" t="str">
-        <f t="shared" si="129"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0380_Selkis/det/0001_srq.t_det_01.png</v>
+        <f>_xlfn.TEXTJOIN("", TRUE, D1018:J1018)</f>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0370_Sobek/det/0001_sbk_det_01.png</v>
       </c>
     </row>
     <row r="1019" spans="1:12" x14ac:dyDescent="0.2">
@@ -32847,23 +32818,13 @@
         <v>60</v>
       </c>
       <c r="B1019" s="27">
-        <v>380</v>
+        <v>370</v>
       </c>
       <c r="C1019" t="s">
-        <v>106</v>
-      </c>
-      <c r="E1019" t="s">
-        <v>1211</v>
-      </c>
-      <c r="F1019" t="s">
-        <v>110</v>
-      </c>
-      <c r="G1019" t="s">
-        <v>971</v>
-      </c>
-      <c r="L1019" t="str">
-        <f t="shared" si="129"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0380_Selkis/det/0010_srq.t_det_02.png</v>
+        <v>107</v>
+      </c>
+      <c r="L1019" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="1020" spans="1:12" x14ac:dyDescent="0.2">
@@ -32871,24 +32832,24 @@
         <v>60</v>
       </c>
       <c r="B1020" s="27">
+        <v>370</v>
+      </c>
+      <c r="C1020" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="1023" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1023" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1023" s="27">
         <v>380</v>
       </c>
-      <c r="C1020" t="s">
-        <v>107</v>
-      </c>
-      <c r="L1020" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="1021" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1021" t="s">
-        <v>60</v>
-      </c>
-      <c r="B1021" s="27">
-        <v>380</v>
-      </c>
-      <c r="C1021" t="s">
-        <v>108</v>
+      <c r="C1023" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1023" t="s">
+        <v>679</v>
       </c>
     </row>
     <row r="1024" spans="1:12" x14ac:dyDescent="0.2">
@@ -32896,13 +32857,20 @@
         <v>60</v>
       </c>
       <c r="B1024" s="27">
-        <v>390</v>
+        <v>380</v>
       </c>
       <c r="C1024" t="s">
-        <v>39</v>
-      </c>
-      <c r="L1024" t="s">
-        <v>680</v>
+        <v>105</v>
+      </c>
+      <c r="E1024" t="s">
+        <v>1211</v>
+      </c>
+      <c r="G1024" t="s">
+        <v>963</v>
+      </c>
+      <c r="L1024" t="str">
+        <f t="shared" ref="L1024:L1032" si="132">_xlfn.TEXTJOIN("", TRUE, D1024:J1024)</f>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0380_Selkis/0001_srq.t_01.png</v>
       </c>
     </row>
     <row r="1025" spans="1:12" x14ac:dyDescent="0.2">
@@ -32910,20 +32878,20 @@
         <v>60</v>
       </c>
       <c r="B1025" s="27">
-        <v>390</v>
+        <v>380</v>
       </c>
       <c r="C1025" t="s">
         <v>105</v>
       </c>
       <c r="E1025" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
       <c r="G1025" t="s">
-        <v>972</v>
+        <v>964</v>
       </c>
       <c r="L1025" t="str">
-        <f t="shared" ref="L1025:L1031" si="131">_xlfn.TEXTJOIN("", TRUE, D1025:J1025)</f>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0390_Sachmet/0001_sxm.t_01.png</v>
+        <f t="shared" si="132"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0380_Selkis/0010_srq.t_02.png</v>
       </c>
     </row>
     <row r="1026" spans="1:12" x14ac:dyDescent="0.2">
@@ -32931,29 +32899,20 @@
         <v>60</v>
       </c>
       <c r="B1026" s="27">
-        <v>390</v>
+        <v>380</v>
       </c>
       <c r="C1026" t="s">
         <v>105</v>
       </c>
       <c r="E1026" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
       <c r="G1026" t="s">
-        <v>973</v>
-      </c>
-      <c r="I1026" t="s">
-        <v>1147</v>
-      </c>
-      <c r="J1026" t="s">
-        <v>1148</v>
-      </c>
-      <c r="K1026" t="s">
-        <v>1149</v>
+        <v>965</v>
       </c>
       <c r="L1026" t="str">
-        <f t="shared" ref="L1026:L1030" si="132">_xlfn.TEXTJOIN("", TRUE, D1026:K1026)</f>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0390_Sachmet/0010_sxm.t_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
+        <f t="shared" si="132"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0380_Selkis/0020_srq.t_03.png</v>
       </c>
     </row>
     <row r="1027" spans="1:12" x14ac:dyDescent="0.2">
@@ -32961,29 +32920,29 @@
         <v>60</v>
       </c>
       <c r="B1027" s="27">
-        <v>390</v>
+        <v>380</v>
       </c>
       <c r="C1027" t="s">
         <v>105</v>
       </c>
       <c r="E1027" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
       <c r="G1027" t="s">
-        <v>974</v>
+        <v>966</v>
       </c>
       <c r="I1027" t="s">
         <v>1147</v>
       </c>
       <c r="J1027" t="s">
-        <v>1148</v>
+        <v>1164</v>
       </c>
       <c r="K1027" t="s">
         <v>1149</v>
       </c>
       <c r="L1027" t="str">
-        <f t="shared" si="132"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0390_Sachmet/0020_sxm.t_AR_02.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
+        <f t="shared" ref="L1027:L1030" si="133">_xlfn.TEXTJOIN("", TRUE, D1027:K1027)</f>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0380_Selkis/0030_srq.t_Pyr.-MR_01.png &lt;sup&gt;(Pyr.; NR)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1028" spans="1:12" x14ac:dyDescent="0.2">
@@ -32991,29 +32950,29 @@
         <v>60</v>
       </c>
       <c r="B1028" s="27">
-        <v>390</v>
+        <v>380</v>
       </c>
       <c r="C1028" t="s">
         <v>105</v>
       </c>
       <c r="E1028" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
       <c r="G1028" t="s">
-        <v>975</v>
+        <v>967</v>
       </c>
       <c r="I1028" t="s">
         <v>1147</v>
       </c>
       <c r="J1028" t="s">
-        <v>1103</v>
+        <v>1150</v>
       </c>
       <c r="K1028" t="s">
         <v>1149</v>
       </c>
       <c r="L1028" t="str">
-        <f t="shared" si="132"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0390_Sachmet/0030_sxm.t_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
+        <f t="shared" si="133"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0380_Selkis/0040_srq.t_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1029" spans="1:12" x14ac:dyDescent="0.2">
@@ -33021,16 +32980,16 @@
         <v>60</v>
       </c>
       <c r="B1029" s="27">
-        <v>390</v>
+        <v>380</v>
       </c>
       <c r="C1029" t="s">
         <v>105</v>
       </c>
       <c r="E1029" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
       <c r="G1029" t="s">
-        <v>976</v>
+        <v>968</v>
       </c>
       <c r="I1029" t="s">
         <v>1147</v>
@@ -33042,8 +33001,8 @@
         <v>1149</v>
       </c>
       <c r="L1029" t="str">
-        <f t="shared" si="132"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0390_Sachmet/0040_sxm.t_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
+        <f t="shared" si="133"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0380_Selkis/0050_srq.t_GR_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1030" spans="1:12" x14ac:dyDescent="0.2">
@@ -33051,16 +33010,16 @@
         <v>60</v>
       </c>
       <c r="B1030" s="27">
-        <v>390</v>
+        <v>380</v>
       </c>
       <c r="C1030" t="s">
         <v>105</v>
       </c>
       <c r="E1030" t="s">
-        <v>1212</v>
+        <v>1211</v>
       </c>
       <c r="G1030" t="s">
-        <v>977</v>
+        <v>969</v>
       </c>
       <c r="I1030" t="s">
         <v>1147</v>
@@ -33072,8 +33031,8 @@
         <v>1149</v>
       </c>
       <c r="L1030" t="str">
-        <f t="shared" si="132"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0390_Sachmet/0050_sxm.t_GR_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
+        <f t="shared" si="133"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0380_Selkis/0060_srq.t_GR_03.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1031" spans="1:12" x14ac:dyDescent="0.2">
@@ -33081,14 +33040,23 @@
         <v>60</v>
       </c>
       <c r="B1031" s="27">
-        <v>390</v>
+        <v>380</v>
       </c>
       <c r="C1031" t="s">
         <v>106</v>
       </c>
+      <c r="E1031" t="s">
+        <v>1211</v>
+      </c>
+      <c r="F1031" t="s">
+        <v>110</v>
+      </c>
+      <c r="G1031" t="s">
+        <v>970</v>
+      </c>
       <c r="L1031" t="str">
-        <f t="shared" si="131"/>
-        <v/>
+        <f t="shared" si="132"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0380_Selkis/det/0001_srq.t_det_01.png</v>
       </c>
     </row>
     <row r="1032" spans="1:12" x14ac:dyDescent="0.2">
@@ -33096,13 +33064,23 @@
         <v>60</v>
       </c>
       <c r="B1032" s="27">
-        <v>390</v>
+        <v>380</v>
       </c>
       <c r="C1032" t="s">
-        <v>107</v>
-      </c>
-      <c r="L1032" t="s">
-        <v>162</v>
+        <v>106</v>
+      </c>
+      <c r="E1032" t="s">
+        <v>1211</v>
+      </c>
+      <c r="F1032" t="s">
+        <v>110</v>
+      </c>
+      <c r="G1032" t="s">
+        <v>971</v>
+      </c>
+      <c r="L1032" t="str">
+        <f t="shared" si="132"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0380_Selkis/det/0010_srq.t_det_02.png</v>
       </c>
     </row>
     <row r="1033" spans="1:12" x14ac:dyDescent="0.2">
@@ -33110,24 +33088,24 @@
         <v>60</v>
       </c>
       <c r="B1033" s="27">
-        <v>390</v>
+        <v>380</v>
       </c>
       <c r="C1033" t="s">
+        <v>107</v>
+      </c>
+      <c r="L1033" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="1034" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1034" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1034" s="27">
+        <v>380</v>
+      </c>
+      <c r="C1034" t="s">
         <v>108</v>
-      </c>
-    </row>
-    <row r="1036" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1036" t="s">
-        <v>60</v>
-      </c>
-      <c r="B1036" s="27">
-        <v>400</v>
-      </c>
-      <c r="C1036" t="s">
-        <v>39</v>
-      </c>
-      <c r="L1036" t="s">
-        <v>681</v>
       </c>
     </row>
     <row r="1037" spans="1:12" x14ac:dyDescent="0.2">
@@ -33135,20 +33113,13 @@
         <v>60</v>
       </c>
       <c r="B1037" s="27">
-        <v>400</v>
+        <v>390</v>
       </c>
       <c r="C1037" t="s">
-        <v>105</v>
-      </c>
-      <c r="E1037" t="s">
-        <v>1213</v>
-      </c>
-      <c r="G1037" t="s">
-        <v>978</v>
-      </c>
-      <c r="L1037" t="str">
-        <f>_xlfn.TEXTJOIN("", TRUE, D1037:J1037)</f>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0400_Sokar/0001_skr_01.png</v>
+        <v>39</v>
+      </c>
+      <c r="L1037" t="s">
+        <v>680</v>
       </c>
     </row>
     <row r="1038" spans="1:12" x14ac:dyDescent="0.2">
@@ -33156,23 +33127,20 @@
         <v>60</v>
       </c>
       <c r="B1038" s="27">
-        <v>400</v>
+        <v>390</v>
       </c>
       <c r="C1038" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E1038" t="s">
-        <v>1213</v>
-      </c>
-      <c r="F1038" t="s">
-        <v>110</v>
+        <v>1212</v>
       </c>
       <c r="G1038" t="s">
-        <v>979</v>
+        <v>972</v>
       </c>
       <c r="L1038" t="str">
-        <f>_xlfn.TEXTJOIN("", TRUE, D1038:J1038)</f>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0400_Sokar/det/0001_skr_det_01.png</v>
+        <f t="shared" ref="L1038:L1044" si="134">_xlfn.TEXTJOIN("", TRUE, D1038:J1038)</f>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0390_Sachmet/0001_sxm.t_01.png</v>
       </c>
     </row>
     <row r="1039" spans="1:12" x14ac:dyDescent="0.2">
@@ -33180,13 +33148,29 @@
         <v>60</v>
       </c>
       <c r="B1039" s="27">
-        <v>400</v>
+        <v>390</v>
       </c>
       <c r="C1039" t="s">
-        <v>107</v>
-      </c>
-      <c r="L1039" t="s">
-        <v>163</v>
+        <v>105</v>
+      </c>
+      <c r="E1039" t="s">
+        <v>1212</v>
+      </c>
+      <c r="G1039" t="s">
+        <v>973</v>
+      </c>
+      <c r="I1039" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1039" t="s">
+        <v>1148</v>
+      </c>
+      <c r="K1039" t="s">
+        <v>1149</v>
+      </c>
+      <c r="L1039" t="str">
+        <f t="shared" ref="L1039:L1043" si="135">_xlfn.TEXTJOIN("", TRUE, D1039:K1039)</f>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0390_Sachmet/0010_sxm.t_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1040" spans="1:12" x14ac:dyDescent="0.2">
@@ -33194,10 +33178,89 @@
         <v>60</v>
       </c>
       <c r="B1040" s="27">
-        <v>400</v>
+        <v>390</v>
       </c>
       <c r="C1040" t="s">
-        <v>108</v>
+        <v>105</v>
+      </c>
+      <c r="E1040" t="s">
+        <v>1212</v>
+      </c>
+      <c r="G1040" t="s">
+        <v>974</v>
+      </c>
+      <c r="I1040" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1040" t="s">
+        <v>1148</v>
+      </c>
+      <c r="K1040" t="s">
+        <v>1149</v>
+      </c>
+      <c r="L1040" t="str">
+        <f t="shared" si="135"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0390_Sachmet/0020_sxm.t_AR_02.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
+      </c>
+    </row>
+    <row r="1041" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1041" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1041" s="27">
+        <v>390</v>
+      </c>
+      <c r="C1041" t="s">
+        <v>105</v>
+      </c>
+      <c r="E1041" t="s">
+        <v>1212</v>
+      </c>
+      <c r="G1041" t="s">
+        <v>975</v>
+      </c>
+      <c r="I1041" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1041" t="s">
+        <v>1103</v>
+      </c>
+      <c r="K1041" t="s">
+        <v>1149</v>
+      </c>
+      <c r="L1041" t="str">
+        <f t="shared" si="135"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0390_Sachmet/0030_sxm.t_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
+      </c>
+    </row>
+    <row r="1042" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1042" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1042" s="27">
+        <v>390</v>
+      </c>
+      <c r="C1042" t="s">
+        <v>105</v>
+      </c>
+      <c r="E1042" t="s">
+        <v>1212</v>
+      </c>
+      <c r="G1042" t="s">
+        <v>976</v>
+      </c>
+      <c r="I1042" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1042" t="s">
+        <v>1150</v>
+      </c>
+      <c r="K1042" t="s">
+        <v>1149</v>
+      </c>
+      <c r="L1042" t="str">
+        <f t="shared" si="135"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0390_Sachmet/0040_sxm.t_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1043" spans="1:12" x14ac:dyDescent="0.2">
@@ -33205,13 +33268,29 @@
         <v>60</v>
       </c>
       <c r="B1043" s="27">
-        <v>410</v>
+        <v>390</v>
       </c>
       <c r="C1043" t="s">
-        <v>39</v>
-      </c>
-      <c r="L1043" t="s">
-        <v>682</v>
+        <v>105</v>
+      </c>
+      <c r="E1043" t="s">
+        <v>1212</v>
+      </c>
+      <c r="G1043" t="s">
+        <v>977</v>
+      </c>
+      <c r="I1043" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1043" t="s">
+        <v>1150</v>
+      </c>
+      <c r="K1043" t="s">
+        <v>1149</v>
+      </c>
+      <c r="L1043" t="str">
+        <f t="shared" si="135"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0390_Sachmet/0050_sxm.t_GR_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1044" spans="1:12" x14ac:dyDescent="0.2">
@@ -33219,20 +33298,14 @@
         <v>60</v>
       </c>
       <c r="B1044" s="27">
-        <v>410</v>
+        <v>390</v>
       </c>
       <c r="C1044" t="s">
-        <v>105</v>
-      </c>
-      <c r="E1044" t="s">
-        <v>1214</v>
-      </c>
-      <c r="G1044" t="s">
-        <v>996</v>
+        <v>106</v>
       </c>
       <c r="L1044" t="str">
-        <f t="shared" ref="L1044:L1057" si="133">_xlfn.TEXTJOIN("", TRUE, D1044:J1044)</f>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0001_stX_01.png</v>
+        <f t="shared" si="134"/>
+        <v/>
       </c>
     </row>
     <row r="1045" spans="1:12" x14ac:dyDescent="0.2">
@@ -33240,29 +33313,13 @@
         <v>60</v>
       </c>
       <c r="B1045" s="27">
-        <v>410</v>
+        <v>390</v>
       </c>
       <c r="C1045" t="s">
-        <v>105</v>
-      </c>
-      <c r="E1045" t="s">
-        <v>1214</v>
-      </c>
-      <c r="G1045" t="s">
-        <v>997</v>
-      </c>
-      <c r="I1045" t="s">
-        <v>1147</v>
-      </c>
-      <c r="J1045" t="s">
-        <v>1148</v>
-      </c>
-      <c r="K1045" t="s">
-        <v>1149</v>
-      </c>
-      <c r="L1045" t="str">
-        <f t="shared" ref="L1045:L1055" si="134">_xlfn.TEXTJOIN("", TRUE, D1045:K1045)</f>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0010_stX_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
+        <v>107</v>
+      </c>
+      <c r="L1045" t="s">
+        <v>162</v>
       </c>
     </row>
     <row r="1046" spans="1:12" x14ac:dyDescent="0.2">
@@ -33270,89 +33327,10 @@
         <v>60</v>
       </c>
       <c r="B1046" s="27">
-        <v>410</v>
+        <v>390</v>
       </c>
       <c r="C1046" t="s">
-        <v>105</v>
-      </c>
-      <c r="E1046" t="s">
-        <v>1214</v>
-      </c>
-      <c r="G1046" t="s">
-        <v>998</v>
-      </c>
-      <c r="I1046" t="s">
-        <v>1147</v>
-      </c>
-      <c r="J1046" t="s">
-        <v>1151</v>
-      </c>
-      <c r="K1046" t="s">
-        <v>1149</v>
-      </c>
-      <c r="L1046" t="str">
-        <f t="shared" si="134"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0020_stX_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
-      </c>
-    </row>
-    <row r="1047" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1047" t="s">
-        <v>60</v>
-      </c>
-      <c r="B1047" s="27">
-        <v>410</v>
-      </c>
-      <c r="C1047" t="s">
-        <v>105</v>
-      </c>
-      <c r="E1047" t="s">
-        <v>1214</v>
-      </c>
-      <c r="G1047" t="s">
-        <v>999</v>
-      </c>
-      <c r="I1047" t="s">
-        <v>1147</v>
-      </c>
-      <c r="J1047" t="s">
-        <v>1165</v>
-      </c>
-      <c r="K1047" t="s">
-        <v>1149</v>
-      </c>
-      <c r="L1047" t="str">
-        <f t="shared" si="134"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0030_stX_MR-SP_01.png &lt;sup&gt;(MR; Sp.)&lt;/sup&gt;</v>
-      </c>
-    </row>
-    <row r="1048" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1048" t="s">
-        <v>60</v>
-      </c>
-      <c r="B1048" s="27">
-        <v>410</v>
-      </c>
-      <c r="C1048" t="s">
-        <v>105</v>
-      </c>
-      <c r="E1048" t="s">
-        <v>1214</v>
-      </c>
-      <c r="G1048" t="s">
-        <v>1000</v>
-      </c>
-      <c r="I1048" t="s">
-        <v>1147</v>
-      </c>
-      <c r="J1048" t="s">
-        <v>1103</v>
-      </c>
-      <c r="K1048" t="s">
-        <v>1149</v>
-      </c>
-      <c r="L1048" t="str">
-        <f t="shared" si="134"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0040_stX_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
+        <v>108</v>
       </c>
     </row>
     <row r="1049" spans="1:12" x14ac:dyDescent="0.2">
@@ -33360,29 +33338,13 @@
         <v>60</v>
       </c>
       <c r="B1049" s="27">
-        <v>410</v>
+        <v>400</v>
       </c>
       <c r="C1049" t="s">
-        <v>105</v>
-      </c>
-      <c r="E1049" t="s">
-        <v>1214</v>
-      </c>
-      <c r="G1049" t="s">
-        <v>1001</v>
-      </c>
-      <c r="I1049" t="s">
-        <v>1147</v>
-      </c>
-      <c r="J1049" t="s">
-        <v>1155</v>
-      </c>
-      <c r="K1049" t="s">
-        <v>1149</v>
-      </c>
-      <c r="L1049" t="str">
-        <f t="shared" si="134"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0050_stX_D.18_01.png &lt;sup&gt;(D.18)&lt;/sup&gt;</v>
+        <v>39</v>
+      </c>
+      <c r="L1049" t="s">
+        <v>681</v>
       </c>
     </row>
     <row r="1050" spans="1:12" x14ac:dyDescent="0.2">
@@ -33390,29 +33352,20 @@
         <v>60</v>
       </c>
       <c r="B1050" s="27">
-        <v>410</v>
+        <v>400</v>
       </c>
       <c r="C1050" t="s">
         <v>105</v>
       </c>
       <c r="E1050" t="s">
-        <v>1214</v>
+        <v>1213</v>
       </c>
       <c r="G1050" t="s">
-        <v>1002</v>
-      </c>
-      <c r="I1050" t="s">
-        <v>1147</v>
-      </c>
-      <c r="J1050" t="s">
-        <v>1155</v>
-      </c>
-      <c r="K1050" t="s">
-        <v>1149</v>
+        <v>978</v>
       </c>
       <c r="L1050" t="str">
-        <f t="shared" si="134"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0060_stX_D.18_02.png &lt;sup&gt;(D.18)&lt;/sup&gt;</v>
+        <f>_xlfn.TEXTJOIN("", TRUE, D1050:J1050)</f>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0400_Sokar/0001_skr_01.png</v>
       </c>
     </row>
     <row r="1051" spans="1:12" x14ac:dyDescent="0.2">
@@ -33420,29 +33373,23 @@
         <v>60</v>
       </c>
       <c r="B1051" s="27">
-        <v>410</v>
+        <v>400</v>
       </c>
       <c r="C1051" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E1051" t="s">
-        <v>1214</v>
+        <v>1213</v>
+      </c>
+      <c r="F1051" t="s">
+        <v>110</v>
       </c>
       <c r="G1051" t="s">
-        <v>1003</v>
-      </c>
-      <c r="I1051" t="s">
-        <v>1147</v>
-      </c>
-      <c r="J1051" t="s">
-        <v>1155</v>
-      </c>
-      <c r="K1051" t="s">
-        <v>1149</v>
+        <v>979</v>
       </c>
       <c r="L1051" t="str">
-        <f t="shared" si="134"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0070_stX_D.18_03.png &lt;sup&gt;(D.18)&lt;/sup&gt;</v>
+        <f>_xlfn.TEXTJOIN("", TRUE, D1051:J1051)</f>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0400_Sokar/det/0001_skr_det_01.png</v>
       </c>
     </row>
     <row r="1052" spans="1:12" x14ac:dyDescent="0.2">
@@ -33450,29 +33397,13 @@
         <v>60</v>
       </c>
       <c r="B1052" s="27">
-        <v>410</v>
+        <v>400</v>
       </c>
       <c r="C1052" t="s">
-        <v>105</v>
-      </c>
-      <c r="E1052" t="s">
-        <v>1214</v>
-      </c>
-      <c r="G1052" t="s">
-        <v>1004</v>
-      </c>
-      <c r="I1052" t="s">
-        <v>1147</v>
-      </c>
-      <c r="J1052" t="s">
-        <v>1160</v>
-      </c>
-      <c r="K1052" t="s">
-        <v>1149</v>
-      </c>
-      <c r="L1052" t="str">
-        <f t="shared" si="134"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0080_stX_D.19_01.png &lt;sup&gt;(D.19)&lt;/sup&gt;</v>
+        <v>107</v>
+      </c>
+      <c r="L1052" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="1053" spans="1:12" x14ac:dyDescent="0.2">
@@ -33480,89 +33411,10 @@
         <v>60</v>
       </c>
       <c r="B1053" s="27">
-        <v>410</v>
+        <v>400</v>
       </c>
       <c r="C1053" t="s">
-        <v>105</v>
-      </c>
-      <c r="E1053" t="s">
-        <v>1214</v>
-      </c>
-      <c r="G1053" t="s">
-        <v>1005</v>
-      </c>
-      <c r="I1053" t="s">
-        <v>1147</v>
-      </c>
-      <c r="J1053" t="s">
-        <v>1160</v>
-      </c>
-      <c r="K1053" t="s">
-        <v>1149</v>
-      </c>
-      <c r="L1053" t="str">
-        <f t="shared" si="134"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0090_stX_D.19_02.png &lt;sup&gt;(D.19)&lt;/sup&gt;</v>
-      </c>
-    </row>
-    <row r="1054" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1054" t="s">
-        <v>60</v>
-      </c>
-      <c r="B1054" s="27">
-        <v>410</v>
-      </c>
-      <c r="C1054" t="s">
-        <v>105</v>
-      </c>
-      <c r="E1054" t="s">
-        <v>1214</v>
-      </c>
-      <c r="G1054" t="s">
-        <v>1006</v>
-      </c>
-      <c r="I1054" t="s">
-        <v>1147</v>
-      </c>
-      <c r="J1054" t="s">
-        <v>1150</v>
-      </c>
-      <c r="K1054" t="s">
-        <v>1149</v>
-      </c>
-      <c r="L1054" t="str">
-        <f t="shared" si="134"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0100_stX_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
-      </c>
-    </row>
-    <row r="1055" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1055" t="s">
-        <v>60</v>
-      </c>
-      <c r="B1055" s="27">
-        <v>410</v>
-      </c>
-      <c r="C1055" t="s">
-        <v>105</v>
-      </c>
-      <c r="E1055" t="s">
-        <v>1214</v>
-      </c>
-      <c r="G1055" t="s">
-        <v>995</v>
-      </c>
-      <c r="I1055" t="s">
-        <v>1147</v>
-      </c>
-      <c r="J1055" t="s">
-        <v>1150</v>
-      </c>
-      <c r="K1055" t="s">
-        <v>1149</v>
-      </c>
-      <c r="L1055" t="str">
-        <f t="shared" si="134"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0110_stX_GR_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
+        <v>108</v>
       </c>
     </row>
     <row r="1056" spans="1:12" x14ac:dyDescent="0.2">
@@ -33573,20 +33425,10 @@
         <v>410</v>
       </c>
       <c r="C1056" t="s">
-        <v>106</v>
-      </c>
-      <c r="E1056" t="s">
-        <v>1214</v>
-      </c>
-      <c r="F1056" t="s">
-        <v>110</v>
-      </c>
-      <c r="G1056" t="s">
-        <v>1007</v>
-      </c>
-      <c r="L1056" t="str">
-        <f t="shared" si="133"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/det/0001_stX_det_01.png</v>
+        <v>39</v>
+      </c>
+      <c r="L1056" t="s">
+        <v>682</v>
       </c>
     </row>
     <row r="1057" spans="1:12" x14ac:dyDescent="0.2">
@@ -33597,20 +33439,17 @@
         <v>410</v>
       </c>
       <c r="C1057" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E1057" t="s">
         <v>1214</v>
       </c>
-      <c r="F1057" t="s">
-        <v>110</v>
-      </c>
       <c r="G1057" t="s">
-        <v>1008</v>
+        <v>996</v>
       </c>
       <c r="L1057" t="str">
-        <f t="shared" si="133"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/det/0010_stX_det_02.png</v>
+        <f t="shared" ref="L1057:L1070" si="136">_xlfn.TEXTJOIN("", TRUE, D1057:J1057)</f>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0001_stX_01.png</v>
       </c>
     </row>
     <row r="1058" spans="1:12" x14ac:dyDescent="0.2">
@@ -33621,29 +33460,26 @@
         <v>410</v>
       </c>
       <c r="C1058" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E1058" t="s">
         <v>1214</v>
       </c>
-      <c r="F1058" t="s">
-        <v>110</v>
-      </c>
       <c r="G1058" t="s">
-        <v>1009</v>
+        <v>997</v>
       </c>
       <c r="I1058" t="s">
         <v>1147</v>
       </c>
       <c r="J1058" t="s">
-        <v>1151</v>
+        <v>1148</v>
       </c>
       <c r="K1058" t="s">
         <v>1149</v>
       </c>
       <c r="L1058" t="str">
-        <f>_xlfn.TEXTJOIN("", TRUE, D1058:K1058)</f>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/det/0020_stX_det_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
+        <f t="shared" ref="L1058:L1068" si="137">_xlfn.TEXTJOIN("", TRUE, D1058:K1058)</f>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0010_stX_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1059" spans="1:12" x14ac:dyDescent="0.2">
@@ -33654,10 +33490,26 @@
         <v>410</v>
       </c>
       <c r="C1059" t="s">
-        <v>107</v>
-      </c>
-      <c r="L1059" t="s">
-        <v>165</v>
+        <v>105</v>
+      </c>
+      <c r="E1059" t="s">
+        <v>1214</v>
+      </c>
+      <c r="G1059" t="s">
+        <v>998</v>
+      </c>
+      <c r="I1059" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1059" t="s">
+        <v>1151</v>
+      </c>
+      <c r="K1059" t="s">
+        <v>1149</v>
+      </c>
+      <c r="L1059" t="str">
+        <f t="shared" si="137"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0020_stX_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1060" spans="1:12" x14ac:dyDescent="0.2">
@@ -33668,7 +33520,86 @@
         <v>410</v>
       </c>
       <c r="C1060" t="s">
-        <v>108</v>
+        <v>105</v>
+      </c>
+      <c r="E1060" t="s">
+        <v>1214</v>
+      </c>
+      <c r="G1060" t="s">
+        <v>999</v>
+      </c>
+      <c r="I1060" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1060" t="s">
+        <v>1165</v>
+      </c>
+      <c r="K1060" t="s">
+        <v>1149</v>
+      </c>
+      <c r="L1060" t="str">
+        <f t="shared" si="137"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0030_stX_MR-SP_01.png &lt;sup&gt;(MR; Sp.)&lt;/sup&gt;</v>
+      </c>
+    </row>
+    <row r="1061" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1061" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1061" s="27">
+        <v>410</v>
+      </c>
+      <c r="C1061" t="s">
+        <v>105</v>
+      </c>
+      <c r="E1061" t="s">
+        <v>1214</v>
+      </c>
+      <c r="G1061" t="s">
+        <v>1000</v>
+      </c>
+      <c r="I1061" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1061" t="s">
+        <v>1103</v>
+      </c>
+      <c r="K1061" t="s">
+        <v>1149</v>
+      </c>
+      <c r="L1061" t="str">
+        <f t="shared" si="137"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0040_stX_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
+      </c>
+    </row>
+    <row r="1062" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1062" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1062" s="27">
+        <v>410</v>
+      </c>
+      <c r="C1062" t="s">
+        <v>105</v>
+      </c>
+      <c r="E1062" t="s">
+        <v>1214</v>
+      </c>
+      <c r="G1062" t="s">
+        <v>1001</v>
+      </c>
+      <c r="I1062" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1062" t="s">
+        <v>1155</v>
+      </c>
+      <c r="K1062" t="s">
+        <v>1149</v>
+      </c>
+      <c r="L1062" t="str">
+        <f t="shared" si="137"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0050_stX_D.18_01.png &lt;sup&gt;(D.18)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1063" spans="1:12" x14ac:dyDescent="0.2">
@@ -33676,13 +33607,29 @@
         <v>60</v>
       </c>
       <c r="B1063" s="27">
-        <v>420</v>
+        <v>410</v>
       </c>
       <c r="C1063" t="s">
-        <v>39</v>
-      </c>
-      <c r="L1063" t="s">
-        <v>683</v>
+        <v>105</v>
+      </c>
+      <c r="E1063" t="s">
+        <v>1214</v>
+      </c>
+      <c r="G1063" t="s">
+        <v>1002</v>
+      </c>
+      <c r="I1063" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1063" t="s">
+        <v>1155</v>
+      </c>
+      <c r="K1063" t="s">
+        <v>1149</v>
+      </c>
+      <c r="L1063" t="str">
+        <f t="shared" si="137"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0060_stX_D.18_02.png &lt;sup&gt;(D.18)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1064" spans="1:12" x14ac:dyDescent="0.2">
@@ -33690,20 +33637,29 @@
         <v>60</v>
       </c>
       <c r="B1064" s="27">
-        <v>420</v>
+        <v>410</v>
       </c>
       <c r="C1064" t="s">
         <v>105</v>
       </c>
       <c r="E1064" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="G1064" t="s">
-        <v>1010</v>
+        <v>1003</v>
+      </c>
+      <c r="I1064" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1064" t="s">
+        <v>1155</v>
+      </c>
+      <c r="K1064" t="s">
+        <v>1149</v>
       </c>
       <c r="L1064" t="str">
-        <f t="shared" ref="L1064:L1069" si="135">_xlfn.TEXTJOIN("", TRUE, D1064:J1064)</f>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0420_Schu/0001_Sw_01.png</v>
+        <f t="shared" si="137"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0070_stX_D.18_03.png &lt;sup&gt;(D.18)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1065" spans="1:12" x14ac:dyDescent="0.2">
@@ -33711,29 +33667,29 @@
         <v>60</v>
       </c>
       <c r="B1065" s="27">
-        <v>420</v>
+        <v>410</v>
       </c>
       <c r="C1065" t="s">
         <v>105</v>
       </c>
       <c r="E1065" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="G1065" t="s">
-        <v>1011</v>
+        <v>1004</v>
       </c>
       <c r="I1065" t="s">
         <v>1147</v>
       </c>
       <c r="J1065" t="s">
-        <v>1148</v>
+        <v>1160</v>
       </c>
       <c r="K1065" t="s">
         <v>1149</v>
       </c>
       <c r="L1065" t="str">
-        <f t="shared" ref="L1065:L1068" si="136">_xlfn.TEXTJOIN("", TRUE, D1065:K1065)</f>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0420_Schu/0010_Sw_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
+        <f t="shared" si="137"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0080_stX_D.19_01.png &lt;sup&gt;(D.19)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1066" spans="1:12" x14ac:dyDescent="0.2">
@@ -33741,29 +33697,29 @@
         <v>60</v>
       </c>
       <c r="B1066" s="27">
-        <v>420</v>
+        <v>410</v>
       </c>
       <c r="C1066" t="s">
         <v>105</v>
       </c>
       <c r="E1066" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="G1066" t="s">
-        <v>1012</v>
+        <v>1005</v>
       </c>
       <c r="I1066" t="s">
         <v>1147</v>
       </c>
       <c r="J1066" t="s">
-        <v>1151</v>
+        <v>1160</v>
       </c>
       <c r="K1066" t="s">
         <v>1149</v>
       </c>
       <c r="L1066" t="str">
-        <f t="shared" si="136"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0420_Schu/0020_Sw_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
+        <f t="shared" si="137"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0090_stX_D.19_02.png &lt;sup&gt;(D.19)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1067" spans="1:12" x14ac:dyDescent="0.2">
@@ -33771,29 +33727,29 @@
         <v>60</v>
       </c>
       <c r="B1067" s="27">
-        <v>420</v>
+        <v>410</v>
       </c>
       <c r="C1067" t="s">
         <v>105</v>
       </c>
       <c r="E1067" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="G1067" t="s">
-        <v>1013</v>
+        <v>1006</v>
       </c>
       <c r="I1067" t="s">
         <v>1147</v>
       </c>
       <c r="J1067" t="s">
-        <v>1103</v>
+        <v>1150</v>
       </c>
       <c r="K1067" t="s">
         <v>1149</v>
       </c>
       <c r="L1067" t="str">
-        <f t="shared" si="136"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0420_Schu/0030_Sw_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
+        <f t="shared" si="137"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0100_stX_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1068" spans="1:12" x14ac:dyDescent="0.2">
@@ -33801,16 +33757,16 @@
         <v>60</v>
       </c>
       <c r="B1068" s="27">
-        <v>420</v>
+        <v>410</v>
       </c>
       <c r="C1068" t="s">
         <v>105</v>
       </c>
       <c r="E1068" t="s">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="G1068" t="s">
-        <v>1014</v>
+        <v>995</v>
       </c>
       <c r="I1068" t="s">
         <v>1147</v>
@@ -33822,8 +33778,8 @@
         <v>1149</v>
       </c>
       <c r="L1068" t="str">
-        <f t="shared" si="136"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0420_Schu/0040_Sw_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
+        <f t="shared" si="137"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/0110_stX_GR_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1069" spans="1:12" x14ac:dyDescent="0.2">
@@ -33831,14 +33787,23 @@
         <v>60</v>
       </c>
       <c r="B1069" s="27">
-        <v>420</v>
+        <v>410</v>
       </c>
       <c r="C1069" t="s">
         <v>106</v>
       </c>
+      <c r="E1069" t="s">
+        <v>1214</v>
+      </c>
+      <c r="F1069" t="s">
+        <v>110</v>
+      </c>
+      <c r="G1069" t="s">
+        <v>1007</v>
+      </c>
       <c r="L1069" t="str">
-        <f t="shared" si="135"/>
-        <v/>
+        <f t="shared" si="136"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/det/0001_stX_det_01.png</v>
       </c>
     </row>
     <row r="1070" spans="1:12" x14ac:dyDescent="0.2">
@@ -33846,13 +33811,23 @@
         <v>60</v>
       </c>
       <c r="B1070" s="27">
-        <v>420</v>
+        <v>410</v>
       </c>
       <c r="C1070" t="s">
-        <v>107</v>
-      </c>
-      <c r="L1070" t="s">
-        <v>166</v>
+        <v>106</v>
+      </c>
+      <c r="E1070" t="s">
+        <v>1214</v>
+      </c>
+      <c r="F1070" t="s">
+        <v>110</v>
+      </c>
+      <c r="G1070" t="s">
+        <v>1008</v>
+      </c>
+      <c r="L1070" t="str">
+        <f t="shared" si="136"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/det/0010_stX_det_02.png</v>
       </c>
     </row>
     <row r="1071" spans="1:12" x14ac:dyDescent="0.2">
@@ -33860,45 +33835,57 @@
         <v>60</v>
       </c>
       <c r="B1071" s="27">
-        <v>420</v>
+        <v>410</v>
       </c>
       <c r="C1071" t="s">
+        <v>106</v>
+      </c>
+      <c r="E1071" t="s">
+        <v>1214</v>
+      </c>
+      <c r="F1071" t="s">
+        <v>110</v>
+      </c>
+      <c r="G1071" t="s">
+        <v>1009</v>
+      </c>
+      <c r="I1071" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1071" t="s">
+        <v>1151</v>
+      </c>
+      <c r="K1071" t="s">
+        <v>1149</v>
+      </c>
+      <c r="L1071" t="str">
+        <f>_xlfn.TEXTJOIN("", TRUE, D1071:K1071)</f>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0410_Seth/det/0020_stX_det_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
+      </c>
+    </row>
+    <row r="1072" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1072" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1072" s="27">
+        <v>410</v>
+      </c>
+      <c r="C1072" t="s">
+        <v>107</v>
+      </c>
+      <c r="L1072" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="1073" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1073" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1073" s="27">
+        <v>410</v>
+      </c>
+      <c r="C1073" t="s">
         <v>108</v>
-      </c>
-    </row>
-    <row r="1074" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1074" t="s">
-        <v>60</v>
-      </c>
-      <c r="B1074" s="27">
-        <v>430</v>
-      </c>
-      <c r="C1074" t="s">
-        <v>39</v>
-      </c>
-      <c r="L1074" t="s">
-        <v>684</v>
-      </c>
-    </row>
-    <row r="1075" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1075" t="s">
-        <v>60</v>
-      </c>
-      <c r="B1075" s="27">
-        <v>430</v>
-      </c>
-      <c r="C1075" t="s">
-        <v>105</v>
-      </c>
-      <c r="E1075" t="s">
-        <v>1216</v>
-      </c>
-      <c r="G1075" t="s">
-        <v>1016</v>
-      </c>
-      <c r="L1075" t="str">
-        <f t="shared" ref="L1075:L1077" si="137">_xlfn.TEXTJOIN("", TRUE, D1075:J1075)</f>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/0001_qbH-snw=f_01.png</v>
       </c>
     </row>
     <row r="1076" spans="1:12" x14ac:dyDescent="0.2">
@@ -33906,20 +33893,13 @@
         <v>60</v>
       </c>
       <c r="B1076" s="27">
-        <v>430</v>
+        <v>420</v>
       </c>
       <c r="C1076" t="s">
-        <v>105</v>
-      </c>
-      <c r="E1076" t="s">
-        <v>1216</v>
-      </c>
-      <c r="G1076" t="s">
-        <v>1017</v>
-      </c>
-      <c r="L1076" t="str">
-        <f t="shared" si="137"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/0010_qbH-snw=f_02.png</v>
+        <v>39</v>
+      </c>
+      <c r="L1076" t="s">
+        <v>683</v>
       </c>
     </row>
     <row r="1077" spans="1:12" x14ac:dyDescent="0.2">
@@ -33927,20 +33907,20 @@
         <v>60</v>
       </c>
       <c r="B1077" s="27">
-        <v>430</v>
+        <v>420</v>
       </c>
       <c r="C1077" t="s">
         <v>105</v>
       </c>
       <c r="E1077" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="G1077" t="s">
-        <v>1018</v>
+        <v>1010</v>
       </c>
       <c r="L1077" t="str">
-        <f t="shared" si="137"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/0020_qbH-snw=f_03.png</v>
+        <f t="shared" ref="L1077:L1082" si="138">_xlfn.TEXTJOIN("", TRUE, D1077:J1077)</f>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0420_Schu/0001_Sw_01.png</v>
       </c>
     </row>
     <row r="1078" spans="1:12" x14ac:dyDescent="0.2">
@@ -33948,29 +33928,29 @@
         <v>60</v>
       </c>
       <c r="B1078" s="27">
-        <v>430</v>
+        <v>420</v>
       </c>
       <c r="C1078" t="s">
         <v>105</v>
       </c>
       <c r="E1078" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="G1078" t="s">
-        <v>1019</v>
+        <v>1011</v>
       </c>
       <c r="I1078" t="s">
         <v>1147</v>
       </c>
       <c r="J1078" t="s">
-        <v>1151</v>
+        <v>1148</v>
       </c>
       <c r="K1078" t="s">
         <v>1149</v>
       </c>
       <c r="L1078" t="str">
-        <f t="shared" ref="L1078:L1085" si="138">_xlfn.TEXTJOIN("", TRUE, D1078:K1078)</f>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/0030_qbH-snw=f_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
+        <f t="shared" ref="L1078:L1081" si="139">_xlfn.TEXTJOIN("", TRUE, D1078:K1078)</f>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0420_Schu/0010_Sw_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1079" spans="1:12" x14ac:dyDescent="0.2">
@@ -33978,16 +33958,16 @@
         <v>60</v>
       </c>
       <c r="B1079" s="27">
-        <v>430</v>
+        <v>420</v>
       </c>
       <c r="C1079" t="s">
         <v>105</v>
       </c>
       <c r="E1079" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="G1079" t="s">
-        <v>1020</v>
+        <v>1012</v>
       </c>
       <c r="I1079" t="s">
         <v>1147</v>
@@ -33999,8 +33979,8 @@
         <v>1149</v>
       </c>
       <c r="L1079" t="str">
-        <f t="shared" si="138"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/0040_qbH-snw=f_MR_02.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
+        <f t="shared" si="139"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0420_Schu/0020_Sw_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1080" spans="1:12" x14ac:dyDescent="0.2">
@@ -34008,29 +33988,29 @@
         <v>60</v>
       </c>
       <c r="B1080" s="27">
-        <v>430</v>
+        <v>420</v>
       </c>
       <c r="C1080" t="s">
         <v>105</v>
       </c>
       <c r="E1080" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="G1080" t="s">
-        <v>1021</v>
+        <v>1013</v>
       </c>
       <c r="I1080" t="s">
         <v>1147</v>
       </c>
       <c r="J1080" t="s">
-        <v>1150</v>
+        <v>1103</v>
       </c>
       <c r="K1080" t="s">
         <v>1149</v>
       </c>
       <c r="L1080" t="str">
-        <f t="shared" si="138"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/0050_qbH-snw=f_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
+        <f t="shared" si="139"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0420_Schu/0030_Sw_NR_01.png &lt;sup&gt;(NR)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1081" spans="1:12" x14ac:dyDescent="0.2">
@@ -34038,16 +34018,16 @@
         <v>60</v>
       </c>
       <c r="B1081" s="27">
-        <v>430</v>
+        <v>420</v>
       </c>
       <c r="C1081" t="s">
         <v>105</v>
       </c>
       <c r="E1081" t="s">
-        <v>1216</v>
+        <v>1215</v>
       </c>
       <c r="G1081" t="s">
-        <v>1022</v>
+        <v>1014</v>
       </c>
       <c r="I1081" t="s">
         <v>1147</v>
@@ -34059,8 +34039,8 @@
         <v>1149</v>
       </c>
       <c r="L1081" t="str">
-        <f t="shared" si="138"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/0060_qbH-snw=f_GR_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
+        <f t="shared" si="139"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0420_Schu/0040_Sw_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1082" spans="1:12" x14ac:dyDescent="0.2">
@@ -34068,29 +34048,14 @@
         <v>60</v>
       </c>
       <c r="B1082" s="27">
-        <v>430</v>
+        <v>420</v>
       </c>
       <c r="C1082" t="s">
-        <v>105</v>
-      </c>
-      <c r="E1082" t="s">
-        <v>1216</v>
-      </c>
-      <c r="G1082" t="s">
-        <v>1023</v>
-      </c>
-      <c r="I1082" t="s">
-        <v>1147</v>
-      </c>
-      <c r="J1082" t="s">
-        <v>1150</v>
-      </c>
-      <c r="K1082" t="s">
-        <v>1149</v>
+        <v>106</v>
       </c>
       <c r="L1082" t="str">
         <f t="shared" si="138"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/0070_qbH-snw=f_GR_03.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
+        <v/>
       </c>
     </row>
     <row r="1083" spans="1:12" x14ac:dyDescent="0.2">
@@ -34098,29 +34063,13 @@
         <v>60</v>
       </c>
       <c r="B1083" s="27">
-        <v>430</v>
+        <v>420</v>
       </c>
       <c r="C1083" t="s">
-        <v>105</v>
-      </c>
-      <c r="E1083" t="s">
-        <v>1216</v>
-      </c>
-      <c r="G1083" t="s">
-        <v>1015</v>
-      </c>
-      <c r="I1083" t="s">
-        <v>1147</v>
-      </c>
-      <c r="J1083" t="s">
-        <v>1150</v>
-      </c>
-      <c r="K1083" t="s">
-        <v>1149</v>
-      </c>
-      <c r="L1083" t="str">
-        <f t="shared" si="138"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/0080_qbH-snw=f_GR_04.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
+        <v>107</v>
+      </c>
+      <c r="L1083" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="1084" spans="1:12" x14ac:dyDescent="0.2">
@@ -34128,79 +34077,10 @@
         <v>60</v>
       </c>
       <c r="B1084" s="27">
-        <v>430</v>
+        <v>420</v>
       </c>
       <c r="C1084" t="s">
-        <v>106</v>
-      </c>
-      <c r="E1084" t="s">
-        <v>1216</v>
-      </c>
-      <c r="F1084" t="s">
-        <v>110</v>
-      </c>
-      <c r="G1084" t="s">
-        <v>1024</v>
-      </c>
-      <c r="I1084" t="s">
-        <v>1147</v>
-      </c>
-      <c r="J1084" t="s">
-        <v>1150</v>
-      </c>
-      <c r="K1084" t="s">
-        <v>1149</v>
-      </c>
-      <c r="L1084" t="str">
-        <f t="shared" si="138"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/det/0001_qbH-snw=f_det_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
-      </c>
-    </row>
-    <row r="1085" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1085" t="s">
-        <v>60</v>
-      </c>
-      <c r="B1085" s="27">
-        <v>430</v>
-      </c>
-      <c r="C1085" t="s">
-        <v>106</v>
-      </c>
-      <c r="E1085" t="s">
-        <v>1216</v>
-      </c>
-      <c r="F1085" t="s">
-        <v>110</v>
-      </c>
-      <c r="G1085" t="s">
-        <v>1025</v>
-      </c>
-      <c r="I1085" t="s">
-        <v>1147</v>
-      </c>
-      <c r="J1085" t="s">
-        <v>1150</v>
-      </c>
-      <c r="K1085" t="s">
-        <v>1149</v>
-      </c>
-      <c r="L1085" t="str">
-        <f t="shared" si="138"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/det/0010_qbH-snw=f_det_GR_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
-      </c>
-    </row>
-    <row r="1086" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1086" t="s">
-        <v>60</v>
-      </c>
-      <c r="B1086" s="27">
-        <v>430</v>
-      </c>
-      <c r="C1086" t="s">
-        <v>107</v>
-      </c>
-      <c r="L1086" t="s">
-        <v>167</v>
+        <v>108</v>
       </c>
     </row>
     <row r="1087" spans="1:12" x14ac:dyDescent="0.2">
@@ -34211,7 +34091,52 @@
         <v>430</v>
       </c>
       <c r="C1087" t="s">
-        <v>108</v>
+        <v>39</v>
+      </c>
+      <c r="L1087" t="s">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="1088" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1088" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1088" s="27">
+        <v>430</v>
+      </c>
+      <c r="C1088" t="s">
+        <v>105</v>
+      </c>
+      <c r="E1088" t="s">
+        <v>1216</v>
+      </c>
+      <c r="G1088" t="s">
+        <v>1016</v>
+      </c>
+      <c r="L1088" t="str">
+        <f t="shared" ref="L1088:L1090" si="140">_xlfn.TEXTJOIN("", TRUE, D1088:J1088)</f>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/0001_qbH-snw=f_01.png</v>
+      </c>
+    </row>
+    <row r="1089" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1089" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1089" s="27">
+        <v>430</v>
+      </c>
+      <c r="C1089" t="s">
+        <v>105</v>
+      </c>
+      <c r="E1089" t="s">
+        <v>1216</v>
+      </c>
+      <c r="G1089" t="s">
+        <v>1017</v>
+      </c>
+      <c r="L1089" t="str">
+        <f t="shared" si="140"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/0010_qbH-snw=f_02.png</v>
       </c>
     </row>
     <row r="1090" spans="1:12" x14ac:dyDescent="0.2">
@@ -34219,13 +34144,20 @@
         <v>60</v>
       </c>
       <c r="B1090" s="27">
-        <v>440</v>
+        <v>430</v>
       </c>
       <c r="C1090" t="s">
-        <v>39</v>
-      </c>
-      <c r="L1090" t="s">
-        <v>685</v>
+        <v>105</v>
+      </c>
+      <c r="E1090" t="s">
+        <v>1216</v>
+      </c>
+      <c r="G1090" t="s">
+        <v>1018</v>
+      </c>
+      <c r="L1090" t="str">
+        <f t="shared" si="140"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/0020_qbH-snw=f_03.png</v>
       </c>
     </row>
     <row r="1091" spans="1:12" x14ac:dyDescent="0.2">
@@ -34233,29 +34165,29 @@
         <v>60</v>
       </c>
       <c r="B1091" s="27">
-        <v>440</v>
+        <v>430</v>
       </c>
       <c r="C1091" t="s">
         <v>105</v>
       </c>
       <c r="E1091" t="s">
-        <v>1217</v>
+        <v>1216</v>
       </c>
       <c r="G1091" t="s">
-        <v>1026</v>
+        <v>1019</v>
       </c>
       <c r="I1091" t="s">
         <v>1147</v>
       </c>
       <c r="J1091" t="s">
-        <v>1148</v>
+        <v>1151</v>
       </c>
       <c r="K1091" t="s">
         <v>1149</v>
       </c>
       <c r="L1091" t="str">
-        <f t="shared" ref="L1091:L1095" si="139">_xlfn.TEXTJOIN("", TRUE, D1091:K1091)</f>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0440_Duamutef/0001_dwA-mw.t=f_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
+        <f t="shared" ref="L1091:L1098" si="141">_xlfn.TEXTJOIN("", TRUE, D1091:K1091)</f>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/0030_qbH-snw=f_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1092" spans="1:12" x14ac:dyDescent="0.2">
@@ -34263,29 +34195,29 @@
         <v>60</v>
       </c>
       <c r="B1092" s="27">
-        <v>440</v>
+        <v>430</v>
       </c>
       <c r="C1092" t="s">
         <v>105</v>
       </c>
       <c r="E1092" t="s">
-        <v>1217</v>
+        <v>1216</v>
       </c>
       <c r="G1092" t="s">
-        <v>1027</v>
+        <v>1020</v>
       </c>
       <c r="I1092" t="s">
         <v>1147</v>
       </c>
       <c r="J1092" t="s">
-        <v>1148</v>
+        <v>1151</v>
       </c>
       <c r="K1092" t="s">
         <v>1149</v>
       </c>
       <c r="L1092" t="str">
-        <f t="shared" si="139"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0440_Duamutef/0010_dwA-mw.t=f_AR_02.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
+        <f t="shared" si="141"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/0040_qbH-snw=f_MR_02.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1093" spans="1:12" x14ac:dyDescent="0.2">
@@ -34293,29 +34225,29 @@
         <v>60</v>
       </c>
       <c r="B1093" s="27">
-        <v>440</v>
+        <v>430</v>
       </c>
       <c r="C1093" t="s">
         <v>105</v>
       </c>
       <c r="E1093" t="s">
-        <v>1217</v>
+        <v>1216</v>
       </c>
       <c r="G1093" t="s">
-        <v>1028</v>
+        <v>1021</v>
       </c>
       <c r="I1093" t="s">
         <v>1147</v>
       </c>
       <c r="J1093" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="K1093" t="s">
         <v>1149</v>
       </c>
       <c r="L1093" t="str">
-        <f t="shared" si="139"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0440_Duamutef/0020_dwA-mw.t=f_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
+        <f t="shared" si="141"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/0050_qbH-snw=f_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1094" spans="1:12" x14ac:dyDescent="0.2">
@@ -34323,29 +34255,29 @@
         <v>60</v>
       </c>
       <c r="B1094" s="27">
-        <v>440</v>
+        <v>430</v>
       </c>
       <c r="C1094" t="s">
         <v>105</v>
       </c>
       <c r="E1094" t="s">
-        <v>1217</v>
+        <v>1216</v>
       </c>
       <c r="G1094" t="s">
-        <v>1029</v>
+        <v>1022</v>
       </c>
       <c r="I1094" t="s">
         <v>1147</v>
       </c>
       <c r="J1094" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="K1094" t="s">
         <v>1149</v>
       </c>
       <c r="L1094" t="str">
-        <f t="shared" si="139"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0440_Duamutef/0030_dwA-mw.t=f_MR_02.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
+        <f t="shared" si="141"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/0060_qbH-snw=f_GR_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1095" spans="1:12" x14ac:dyDescent="0.2">
@@ -34353,29 +34285,29 @@
         <v>60</v>
       </c>
       <c r="B1095" s="27">
-        <v>440</v>
+        <v>430</v>
       </c>
       <c r="C1095" t="s">
         <v>105</v>
       </c>
       <c r="E1095" t="s">
-        <v>1217</v>
+        <v>1216</v>
       </c>
       <c r="G1095" t="s">
-        <v>1030</v>
+        <v>1023</v>
       </c>
       <c r="I1095" t="s">
         <v>1147</v>
       </c>
       <c r="J1095" t="s">
-        <v>1151</v>
+        <v>1150</v>
       </c>
       <c r="K1095" t="s">
         <v>1149</v>
       </c>
       <c r="L1095" t="str">
-        <f t="shared" si="139"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0440_Duamutef/0040_dwA-mw.t=f_MR_03.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
+        <f t="shared" si="141"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/0070_qbH-snw=f_GR_03.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1096" spans="1:12" x14ac:dyDescent="0.2">
@@ -34383,14 +34315,29 @@
         <v>60</v>
       </c>
       <c r="B1096" s="27">
-        <v>440</v>
+        <v>430</v>
       </c>
       <c r="C1096" t="s">
-        <v>106</v>
+        <v>105</v>
+      </c>
+      <c r="E1096" t="s">
+        <v>1216</v>
+      </c>
+      <c r="G1096" t="s">
+        <v>1015</v>
+      </c>
+      <c r="I1096" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1096" t="s">
+        <v>1150</v>
+      </c>
+      <c r="K1096" t="s">
+        <v>1149</v>
       </c>
       <c r="L1096" t="str">
-        <f t="shared" ref="L1096" si="140">_xlfn.TEXTJOIN("", TRUE, D1096:J1096)</f>
-        <v/>
+        <f t="shared" si="141"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/0080_qbH-snw=f_GR_04.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1097" spans="1:12" x14ac:dyDescent="0.2">
@@ -34398,13 +34345,32 @@
         <v>60</v>
       </c>
       <c r="B1097" s="27">
-        <v>440</v>
+        <v>430</v>
       </c>
       <c r="C1097" t="s">
-        <v>107</v>
-      </c>
-      <c r="L1097" t="s">
-        <v>168</v>
+        <v>106</v>
+      </c>
+      <c r="E1097" t="s">
+        <v>1216</v>
+      </c>
+      <c r="F1097" t="s">
+        <v>110</v>
+      </c>
+      <c r="G1097" t="s">
+        <v>1024</v>
+      </c>
+      <c r="I1097" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1097" t="s">
+        <v>1150</v>
+      </c>
+      <c r="K1097" t="s">
+        <v>1149</v>
+      </c>
+      <c r="L1097" t="str">
+        <f t="shared" si="141"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/det/0001_qbH-snw=f_det_GR_01.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1098" spans="1:12" x14ac:dyDescent="0.2">
@@ -34412,54 +34378,57 @@
         <v>60</v>
       </c>
       <c r="B1098" s="27">
-        <v>440</v>
+        <v>430</v>
       </c>
       <c r="C1098" t="s">
+        <v>106</v>
+      </c>
+      <c r="E1098" t="s">
+        <v>1216</v>
+      </c>
+      <c r="F1098" t="s">
+        <v>110</v>
+      </c>
+      <c r="G1098" t="s">
+        <v>1025</v>
+      </c>
+      <c r="I1098" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1098" t="s">
+        <v>1150</v>
+      </c>
+      <c r="K1098" t="s">
+        <v>1149</v>
+      </c>
+      <c r="L1098" t="str">
+        <f t="shared" si="141"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0430_Qebehsenuef/det/0010_qbH-snw=f_det_GR_02.png &lt;sup&gt;(Gr.)&lt;/sup&gt;</v>
+      </c>
+    </row>
+    <row r="1099" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1099" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1099" s="27">
+        <v>430</v>
+      </c>
+      <c r="C1099" t="s">
+        <v>107</v>
+      </c>
+      <c r="L1099" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="1100" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1100" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1100" s="27">
+        <v>430</v>
+      </c>
+      <c r="C1100" t="s">
         <v>108</v>
-      </c>
-    </row>
-    <row r="1101" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1101" t="s">
-        <v>60</v>
-      </c>
-      <c r="B1101" s="27">
-        <v>450</v>
-      </c>
-      <c r="C1101" t="s">
-        <v>39</v>
-      </c>
-      <c r="L1101" t="s">
-        <v>686</v>
-      </c>
-    </row>
-    <row r="1102" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1102" t="s">
-        <v>60</v>
-      </c>
-      <c r="B1102" s="27">
-        <v>450</v>
-      </c>
-      <c r="C1102" t="s">
-        <v>105</v>
-      </c>
-      <c r="E1102" t="s">
-        <v>1218</v>
-      </c>
-      <c r="G1102" t="s">
-        <v>1031</v>
-      </c>
-      <c r="I1102" t="s">
-        <v>1147</v>
-      </c>
-      <c r="J1102" t="s">
-        <v>1148</v>
-      </c>
-      <c r="K1102" t="s">
-        <v>1149</v>
-      </c>
-      <c r="L1102" t="str">
-        <f t="shared" ref="L1102:L1112" si="141">_xlfn.TEXTJOIN("", TRUE, D1102:K1102)</f>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0001_DHwtj_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1103" spans="1:12" x14ac:dyDescent="0.2">
@@ -34467,29 +34436,13 @@
         <v>60</v>
       </c>
       <c r="B1103" s="27">
-        <v>450</v>
+        <v>440</v>
       </c>
       <c r="C1103" t="s">
-        <v>105</v>
-      </c>
-      <c r="E1103" t="s">
-        <v>1218</v>
-      </c>
-      <c r="G1103" t="s">
-        <v>1032</v>
-      </c>
-      <c r="I1103" t="s">
-        <v>1147</v>
-      </c>
-      <c r="J1103" t="s">
-        <v>1151</v>
-      </c>
-      <c r="K1103" t="s">
-        <v>1149</v>
-      </c>
-      <c r="L1103" t="str">
-        <f t="shared" si="141"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0010_DHwtj_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
+        <v>39</v>
+      </c>
+      <c r="L1103" t="s">
+        <v>685</v>
       </c>
     </row>
     <row r="1104" spans="1:12" x14ac:dyDescent="0.2">
@@ -34497,29 +34450,29 @@
         <v>60</v>
       </c>
       <c r="B1104" s="27">
-        <v>450</v>
+        <v>440</v>
       </c>
       <c r="C1104" t="s">
         <v>105</v>
       </c>
       <c r="E1104" t="s">
-        <v>1218</v>
+        <v>1217</v>
       </c>
       <c r="G1104" t="s">
-        <v>1033</v>
+        <v>1026</v>
       </c>
       <c r="I1104" t="s">
         <v>1147</v>
       </c>
       <c r="J1104" t="s">
-        <v>1151</v>
+        <v>1148</v>
       </c>
       <c r="K1104" t="s">
         <v>1149</v>
       </c>
       <c r="L1104" t="str">
-        <f t="shared" si="141"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0020_DHwtj_MR_02.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
+        <f t="shared" ref="L1104:L1108" si="142">_xlfn.TEXTJOIN("", TRUE, D1104:K1104)</f>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0440_Duamutef/0001_dwA-mw.t=f_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1105" spans="1:12" x14ac:dyDescent="0.2">
@@ -34527,29 +34480,29 @@
         <v>60</v>
       </c>
       <c r="B1105" s="27">
-        <v>450</v>
+        <v>440</v>
       </c>
       <c r="C1105" t="s">
         <v>105</v>
       </c>
       <c r="E1105" t="s">
-        <v>1218</v>
+        <v>1217</v>
       </c>
       <c r="G1105" t="s">
-        <v>1034</v>
+        <v>1027</v>
       </c>
       <c r="I1105" t="s">
         <v>1147</v>
       </c>
       <c r="J1105" t="s">
-        <v>1151</v>
+        <v>1148</v>
       </c>
       <c r="K1105" t="s">
         <v>1149</v>
       </c>
       <c r="L1105" t="str">
-        <f t="shared" si="141"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0030_DHwtj_MR_03.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
+        <f t="shared" si="142"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0440_Duamutef/0010_dwA-mw.t=f_AR_02.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1106" spans="1:12" x14ac:dyDescent="0.2">
@@ -34557,16 +34510,16 @@
         <v>60</v>
       </c>
       <c r="B1106" s="27">
-        <v>450</v>
+        <v>440</v>
       </c>
       <c r="C1106" t="s">
         <v>105</v>
       </c>
       <c r="E1106" t="s">
-        <v>1218</v>
+        <v>1217</v>
       </c>
       <c r="G1106" t="s">
-        <v>1035</v>
+        <v>1028</v>
       </c>
       <c r="I1106" t="s">
         <v>1147</v>
@@ -34578,8 +34531,8 @@
         <v>1149</v>
       </c>
       <c r="L1106" t="str">
-        <f t="shared" si="141"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0040_DHwtj_MR_04.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
+        <f t="shared" si="142"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0440_Duamutef/0020_dwA-mw.t=f_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1107" spans="1:12" x14ac:dyDescent="0.2">
@@ -34587,16 +34540,16 @@
         <v>60</v>
       </c>
       <c r="B1107" s="27">
-        <v>450</v>
+        <v>440</v>
       </c>
       <c r="C1107" t="s">
         <v>105</v>
       </c>
       <c r="E1107" t="s">
-        <v>1218</v>
+        <v>1217</v>
       </c>
       <c r="G1107" t="s">
-        <v>1036</v>
+        <v>1029</v>
       </c>
       <c r="I1107" t="s">
         <v>1147</v>
@@ -34608,8 +34561,8 @@
         <v>1149</v>
       </c>
       <c r="L1107" t="str">
-        <f t="shared" si="141"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0050_DHwtj_MR_05.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
+        <f t="shared" si="142"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0440_Duamutef/0030_dwA-mw.t=f_MR_02.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1108" spans="1:12" x14ac:dyDescent="0.2">
@@ -34617,29 +34570,29 @@
         <v>60</v>
       </c>
       <c r="B1108" s="27">
-        <v>450</v>
+        <v>440</v>
       </c>
       <c r="C1108" t="s">
         <v>105</v>
       </c>
       <c r="E1108" t="s">
-        <v>1218</v>
+        <v>1217</v>
       </c>
       <c r="G1108" t="s">
-        <v>1037</v>
+        <v>1030</v>
       </c>
       <c r="I1108" t="s">
         <v>1147</v>
       </c>
       <c r="J1108" t="s">
-        <v>1156</v>
+        <v>1151</v>
       </c>
       <c r="K1108" t="s">
         <v>1149</v>
       </c>
       <c r="L1108" t="str">
-        <f t="shared" si="141"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0060_DHwtj_SP_01.png &lt;sup&gt;(Sp.)&lt;/sup&gt;</v>
+        <f t="shared" si="142"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0440_Duamutef/0040_dwA-mw.t=f_MR_03.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
       </c>
     </row>
     <row r="1109" spans="1:12" x14ac:dyDescent="0.2">
@@ -34647,29 +34600,14 @@
         <v>60</v>
       </c>
       <c r="B1109" s="27">
-        <v>450</v>
+        <v>440</v>
       </c>
       <c r="C1109" t="s">
-        <v>105</v>
-      </c>
-      <c r="E1109" t="s">
-        <v>1218</v>
-      </c>
-      <c r="G1109" t="s">
-        <v>1038</v>
-      </c>
-      <c r="I1109" t="s">
-        <v>1147</v>
-      </c>
-      <c r="J1109" t="s">
-        <v>1156</v>
-      </c>
-      <c r="K1109" t="s">
-        <v>1149</v>
+        <v>106</v>
       </c>
       <c r="L1109" t="str">
-        <f t="shared" si="141"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0070_DHwtj_SP_02.png &lt;sup&gt;(Sp.)&lt;/sup&gt;</v>
+        <f t="shared" ref="L1109" si="143">_xlfn.TEXTJOIN("", TRUE, D1109:J1109)</f>
+        <v/>
       </c>
     </row>
     <row r="1110" spans="1:12" x14ac:dyDescent="0.2">
@@ -34677,29 +34615,13 @@
         <v>60</v>
       </c>
       <c r="B1110" s="27">
-        <v>450</v>
+        <v>440</v>
       </c>
       <c r="C1110" t="s">
-        <v>105</v>
-      </c>
-      <c r="E1110" t="s">
-        <v>1218</v>
-      </c>
-      <c r="G1110" t="s">
-        <v>1039</v>
-      </c>
-      <c r="I1110" t="s">
-        <v>1147</v>
-      </c>
-      <c r="J1110" t="s">
-        <v>1166</v>
-      </c>
-      <c r="K1110" t="s">
-        <v>1149</v>
-      </c>
-      <c r="L1110" t="str">
-        <f t="shared" si="141"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0080_DHwtj_SP-GR_01.png &lt;sup&gt;(Sp.; Gr.)&lt;/sup&gt;</v>
+        <v>107</v>
+      </c>
+      <c r="L1110" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="1111" spans="1:12" x14ac:dyDescent="0.2">
@@ -34707,76 +34629,10 @@
         <v>60</v>
       </c>
       <c r="B1111" s="27">
-        <v>450</v>
+        <v>440</v>
       </c>
       <c r="C1111" t="s">
-        <v>105</v>
-      </c>
-      <c r="E1111" t="s">
-        <v>1218</v>
-      </c>
-      <c r="G1111" t="s">
-        <v>1040</v>
-      </c>
-      <c r="I1111" t="s">
-        <v>1147</v>
-      </c>
-      <c r="J1111" t="s">
-        <v>1166</v>
-      </c>
-      <c r="K1111" t="s">
-        <v>1149</v>
-      </c>
-      <c r="L1111" t="str">
-        <f t="shared" si="141"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0090_DHwtj_SP-GR_02.png &lt;sup&gt;(Sp.; Gr.)&lt;/sup&gt;</v>
-      </c>
-    </row>
-    <row r="1112" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1112" t="s">
-        <v>60</v>
-      </c>
-      <c r="B1112" s="27">
-        <v>450</v>
-      </c>
-      <c r="C1112" t="s">
-        <v>106</v>
-      </c>
-      <c r="E1112" t="s">
-        <v>1218</v>
-      </c>
-      <c r="F1112" t="s">
-        <v>110</v>
-      </c>
-      <c r="G1112" t="s">
-        <v>1041</v>
-      </c>
-      <c r="I1112" t="s">
-        <v>1147</v>
-      </c>
-      <c r="J1112" t="s">
-        <v>1156</v>
-      </c>
-      <c r="K1112" t="s">
-        <v>1149</v>
-      </c>
-      <c r="L1112" t="str">
-        <f t="shared" si="141"/>
-        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/det/0001_DHwtj_det_SP_01.png &lt;sup&gt;(Sp.)&lt;/sup&gt;</v>
-      </c>
-    </row>
-    <row r="1113" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1113" t="s">
-        <v>60</v>
-      </c>
-      <c r="B1113" s="27">
-        <v>450</v>
-      </c>
-      <c r="C1113" t="s">
-        <v>107</v>
-      </c>
-      <c r="L1113" t="s">
-        <v>169</v>
+        <v>108</v>
       </c>
     </row>
     <row r="1114" spans="1:12" x14ac:dyDescent="0.2">
@@ -34787,211 +34643,572 @@
         <v>450</v>
       </c>
       <c r="C1114" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1114" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="1115" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1115" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1115" s="27">
+        <v>450</v>
+      </c>
+      <c r="C1115" t="s">
+        <v>105</v>
+      </c>
+      <c r="E1115" t="s">
+        <v>1218</v>
+      </c>
+      <c r="G1115" t="s">
+        <v>1031</v>
+      </c>
+      <c r="I1115" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1115" t="s">
+        <v>1148</v>
+      </c>
+      <c r="K1115" t="s">
+        <v>1149</v>
+      </c>
+      <c r="L1115" t="str">
+        <f t="shared" ref="L1115:L1125" si="144">_xlfn.TEXTJOIN("", TRUE, D1115:K1115)</f>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0001_DHwtj_AR_01.png &lt;sup&gt;(AR)&lt;/sup&gt;</v>
+      </c>
+    </row>
+    <row r="1116" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1116" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1116" s="27">
+        <v>450</v>
+      </c>
+      <c r="C1116" t="s">
+        <v>105</v>
+      </c>
+      <c r="E1116" t="s">
+        <v>1218</v>
+      </c>
+      <c r="G1116" t="s">
+        <v>1032</v>
+      </c>
+      <c r="I1116" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1116" t="s">
+        <v>1151</v>
+      </c>
+      <c r="K1116" t="s">
+        <v>1149</v>
+      </c>
+      <c r="L1116" t="str">
+        <f t="shared" si="144"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0010_DHwtj_MR_01.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
+      </c>
+    </row>
+    <row r="1117" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1117" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1117" s="27">
+        <v>450</v>
+      </c>
+      <c r="C1117" t="s">
+        <v>105</v>
+      </c>
+      <c r="E1117" t="s">
+        <v>1218</v>
+      </c>
+      <c r="G1117" t="s">
+        <v>1033</v>
+      </c>
+      <c r="I1117" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1117" t="s">
+        <v>1151</v>
+      </c>
+      <c r="K1117" t="s">
+        <v>1149</v>
+      </c>
+      <c r="L1117" t="str">
+        <f t="shared" si="144"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0020_DHwtj_MR_02.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
+      </c>
+    </row>
+    <row r="1118" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1118" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1118" s="27">
+        <v>450</v>
+      </c>
+      <c r="C1118" t="s">
+        <v>105</v>
+      </c>
+      <c r="E1118" t="s">
+        <v>1218</v>
+      </c>
+      <c r="G1118" t="s">
+        <v>1034</v>
+      </c>
+      <c r="I1118" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1118" t="s">
+        <v>1151</v>
+      </c>
+      <c r="K1118" t="s">
+        <v>1149</v>
+      </c>
+      <c r="L1118" t="str">
+        <f t="shared" si="144"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0030_DHwtj_MR_03.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
+      </c>
+    </row>
+    <row r="1119" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1119" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1119" s="27">
+        <v>450</v>
+      </c>
+      <c r="C1119" t="s">
+        <v>105</v>
+      </c>
+      <c r="E1119" t="s">
+        <v>1218</v>
+      </c>
+      <c r="G1119" t="s">
+        <v>1035</v>
+      </c>
+      <c r="I1119" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1119" t="s">
+        <v>1151</v>
+      </c>
+      <c r="K1119" t="s">
+        <v>1149</v>
+      </c>
+      <c r="L1119" t="str">
+        <f t="shared" si="144"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0040_DHwtj_MR_04.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
+      </c>
+    </row>
+    <row r="1120" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1120" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1120" s="27">
+        <v>450</v>
+      </c>
+      <c r="C1120" t="s">
+        <v>105</v>
+      </c>
+      <c r="E1120" t="s">
+        <v>1218</v>
+      </c>
+      <c r="G1120" t="s">
+        <v>1036</v>
+      </c>
+      <c r="I1120" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1120" t="s">
+        <v>1151</v>
+      </c>
+      <c r="K1120" t="s">
+        <v>1149</v>
+      </c>
+      <c r="L1120" t="str">
+        <f t="shared" si="144"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0050_DHwtj_MR_05.png &lt;sup&gt;(MR)&lt;/sup&gt;</v>
+      </c>
+    </row>
+    <row r="1121" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1121" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1121" s="27">
+        <v>450</v>
+      </c>
+      <c r="C1121" t="s">
+        <v>105</v>
+      </c>
+      <c r="E1121" t="s">
+        <v>1218</v>
+      </c>
+      <c r="G1121" t="s">
+        <v>1037</v>
+      </c>
+      <c r="I1121" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1121" t="s">
+        <v>1156</v>
+      </c>
+      <c r="K1121" t="s">
+        <v>1149</v>
+      </c>
+      <c r="L1121" t="str">
+        <f t="shared" si="144"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0060_DHwtj_SP_01.png &lt;sup&gt;(Sp.)&lt;/sup&gt;</v>
+      </c>
+    </row>
+    <row r="1122" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1122" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1122" s="27">
+        <v>450</v>
+      </c>
+      <c r="C1122" t="s">
+        <v>105</v>
+      </c>
+      <c r="E1122" t="s">
+        <v>1218</v>
+      </c>
+      <c r="G1122" t="s">
+        <v>1038</v>
+      </c>
+      <c r="I1122" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1122" t="s">
+        <v>1156</v>
+      </c>
+      <c r="K1122" t="s">
+        <v>1149</v>
+      </c>
+      <c r="L1122" t="str">
+        <f t="shared" si="144"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0070_DHwtj_SP_02.png &lt;sup&gt;(Sp.)&lt;/sup&gt;</v>
+      </c>
+    </row>
+    <row r="1123" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1123" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1123" s="27">
+        <v>450</v>
+      </c>
+      <c r="C1123" t="s">
+        <v>105</v>
+      </c>
+      <c r="E1123" t="s">
+        <v>1218</v>
+      </c>
+      <c r="G1123" t="s">
+        <v>1039</v>
+      </c>
+      <c r="I1123" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1123" t="s">
+        <v>1166</v>
+      </c>
+      <c r="K1123" t="s">
+        <v>1149</v>
+      </c>
+      <c r="L1123" t="str">
+        <f t="shared" si="144"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0080_DHwtj_SP-GR_01.png &lt;sup&gt;(Sp.; Gr.)&lt;/sup&gt;</v>
+      </c>
+    </row>
+    <row r="1124" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1124" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1124" s="27">
+        <v>450</v>
+      </c>
+      <c r="C1124" t="s">
+        <v>105</v>
+      </c>
+      <c r="E1124" t="s">
+        <v>1218</v>
+      </c>
+      <c r="G1124" t="s">
+        <v>1040</v>
+      </c>
+      <c r="I1124" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1124" t="s">
+        <v>1166</v>
+      </c>
+      <c r="K1124" t="s">
+        <v>1149</v>
+      </c>
+      <c r="L1124" t="str">
+        <f t="shared" si="144"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/0090_DHwtj_SP-GR_02.png &lt;sup&gt;(Sp.; Gr.)&lt;/sup&gt;</v>
+      </c>
+    </row>
+    <row r="1125" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1125" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1125" s="27">
+        <v>450</v>
+      </c>
+      <c r="C1125" t="s">
+        <v>106</v>
+      </c>
+      <c r="E1125" t="s">
+        <v>1218</v>
+      </c>
+      <c r="F1125" t="s">
+        <v>110</v>
+      </c>
+      <c r="G1125" t="s">
+        <v>1041</v>
+      </c>
+      <c r="I1125" t="s">
+        <v>1147</v>
+      </c>
+      <c r="J1125" t="s">
+        <v>1156</v>
+      </c>
+      <c r="K1125" t="s">
+        <v>1149</v>
+      </c>
+      <c r="L1125" t="str">
+        <f t="shared" si="144"/>
+        <v>02_Slots/Gottheit/Goetter-mit-Epitheta/0450_Thot/det/0001_DHwtj_det_SP_01.png &lt;sup&gt;(Sp.)&lt;/sup&gt;</v>
+      </c>
+    </row>
+    <row r="1126" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1126" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1126" s="27">
+        <v>450</v>
+      </c>
+      <c r="C1126" t="s">
+        <v>107</v>
+      </c>
+      <c r="L1126" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="1127" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1127" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1127" s="27">
+        <v>450</v>
+      </c>
+      <c r="C1127" t="s">
         <v>108</v>
-      </c>
-    </row>
-    <row r="1120" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1120" s="4" t="s">
-        <v>1236</v>
-      </c>
-      <c r="B1120" s="27">
-        <v>1</v>
-      </c>
-      <c r="C1120" t="s">
-        <v>1292</v>
-      </c>
-      <c r="L1120" t="s">
-        <v>1293</v>
-      </c>
-    </row>
-    <row r="1121" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1121" s="4" t="s">
-        <v>1236</v>
-      </c>
-      <c r="B1121" s="27">
-        <v>1</v>
-      </c>
-      <c r="C1121" t="s">
-        <v>1235</v>
-      </c>
-      <c r="E1121" t="s">
-        <v>1289</v>
-      </c>
-      <c r="G1121" t="s">
-        <v>1288</v>
-      </c>
-      <c r="H1121" t="s">
-        <v>112</v>
-      </c>
-      <c r="L1121" t="str">
-        <f t="shared" ref="L1121" si="142">_xlfn.TEXTJOIN("", TRUE, D1121:K1121)</f>
-        <v>03_Hieroglyphen-selten/F63_xnty_01.png</v>
-      </c>
-    </row>
-    <row r="1122" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1122" s="4" t="s">
-        <v>1236</v>
-      </c>
-      <c r="B1122" s="27">
-        <v>1</v>
-      </c>
-      <c r="C1122" t="s">
-        <v>39</v>
-      </c>
-      <c r="L1122" t="s">
-        <v>1290</v>
-      </c>
-    </row>
-    <row r="1123" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1123" s="4" t="s">
-        <v>1236</v>
-      </c>
-      <c r="B1123" s="27">
-        <v>1</v>
-      </c>
-      <c r="C1123" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1123" t="s">
-        <v>1291</v>
-      </c>
-    </row>
-    <row r="1128" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1128" s="4" t="s">
-        <v>1274</v>
-      </c>
-      <c r="B1128" s="27">
-        <v>1</v>
-      </c>
-      <c r="C1128" t="s">
-        <v>1292</v>
-      </c>
-      <c r="L1128" t="s">
-        <v>1294</v>
-      </c>
-    </row>
-    <row r="1129" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1129" s="4" t="s">
-        <v>1274</v>
-      </c>
-      <c r="B1129" s="27">
-        <v>1</v>
-      </c>
-      <c r="C1129" t="s">
-        <v>1235</v>
-      </c>
-      <c r="E1129" t="s">
-        <v>1289</v>
-      </c>
-      <c r="G1129" t="s">
-        <v>1295</v>
-      </c>
-      <c r="H1129" t="s">
-        <v>112</v>
-      </c>
-      <c r="L1129" t="str">
-        <f t="shared" ref="L1129" si="143">_xlfn.TEXTJOIN("", TRUE, D1129:K1129)</f>
-        <v>03_Hieroglyphen-selten/N6B_nsw-bjt_01.png</v>
-      </c>
-    </row>
-    <row r="1130" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1130" s="4" t="s">
-        <v>1274</v>
-      </c>
-      <c r="B1130" s="27">
-        <v>1</v>
-      </c>
-      <c r="C1130" t="s">
-        <v>39</v>
-      </c>
-      <c r="L1130" t="s">
-        <v>517</v>
-      </c>
-    </row>
-    <row r="1131" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1131" s="4" t="s">
-        <v>1274</v>
-      </c>
-      <c r="B1131" s="27">
-        <v>1</v>
-      </c>
-      <c r="C1131" t="s">
-        <v>27</v>
-      </c>
-      <c r="L1131" t="s">
-        <v>1296</v>
-      </c>
-    </row>
-    <row r="1132" spans="1:12" x14ac:dyDescent="0.2">
-      <c r="A1132" s="4" t="s">
-        <v>1274</v>
-      </c>
-      <c r="B1132" s="27">
-        <v>2</v>
-      </c>
-      <c r="C1132" t="s">
-        <v>1292</v>
-      </c>
-      <c r="L1132" t="s">
-        <v>1298</v>
       </c>
     </row>
     <row r="1133" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1133" s="4" t="s">
-        <v>1274</v>
+        <v>1236</v>
       </c>
       <c r="B1133" s="27">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C1133" t="s">
-        <v>1235</v>
-      </c>
-      <c r="E1133" t="s">
-        <v>1289</v>
-      </c>
-      <c r="G1133" t="s">
-        <v>1297</v>
-      </c>
-      <c r="H1133" t="s">
-        <v>112</v>
-      </c>
-      <c r="L1133" t="str">
-        <f t="shared" ref="L1133" si="144">_xlfn.TEXTJOIN("", TRUE, D1133:K1133)</f>
-        <v>03_Hieroglyphen-selten/N102_jmn_01.png</v>
+        <v>1292</v>
+      </c>
+      <c r="L1133" t="s">
+        <v>1293</v>
       </c>
     </row>
     <row r="1134" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1134" s="4" t="s">
-        <v>1274</v>
+        <v>1236</v>
       </c>
       <c r="B1134" s="27">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C1134" t="s">
-        <v>39</v>
-      </c>
-      <c r="L1134" t="s">
-        <v>175</v>
+        <v>1235</v>
+      </c>
+      <c r="E1134" t="s">
+        <v>1289</v>
+      </c>
+      <c r="G1134" t="s">
+        <v>1288</v>
+      </c>
+      <c r="H1134" t="s">
+        <v>112</v>
+      </c>
+      <c r="L1134" t="str">
+        <f t="shared" ref="L1134" si="145">_xlfn.TEXTJOIN("", TRUE, D1134:K1134)</f>
+        <v>03_Hieroglyphen-selten/F63_xnty_01.png</v>
       </c>
     </row>
     <row r="1135" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A1135" s="4" t="s">
+        <v>1236</v>
+      </c>
+      <c r="B1135" s="27">
+        <v>1</v>
+      </c>
+      <c r="C1135" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1135" t="s">
+        <v>1290</v>
+      </c>
+    </row>
+    <row r="1136" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1136" s="4" t="s">
+        <v>1236</v>
+      </c>
+      <c r="B1136" s="27">
+        <v>1</v>
+      </c>
+      <c r="C1136" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1136" t="s">
+        <v>1291</v>
+      </c>
+    </row>
+    <row r="1141" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1141" s="4" t="s">
         <v>1274</v>
       </c>
-      <c r="B1135" s="27">
+      <c r="B1141" s="27">
+        <v>1</v>
+      </c>
+      <c r="C1141" t="s">
+        <v>1292</v>
+      </c>
+      <c r="L1141" t="s">
+        <v>1294</v>
+      </c>
+    </row>
+    <row r="1142" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1142" s="4" t="s">
+        <v>1274</v>
+      </c>
+      <c r="B1142" s="27">
+        <v>1</v>
+      </c>
+      <c r="C1142" t="s">
+        <v>1235</v>
+      </c>
+      <c r="E1142" t="s">
+        <v>1289</v>
+      </c>
+      <c r="G1142" t="s">
+        <v>1295</v>
+      </c>
+      <c r="H1142" t="s">
+        <v>112</v>
+      </c>
+      <c r="L1142" t="str">
+        <f t="shared" ref="L1142" si="146">_xlfn.TEXTJOIN("", TRUE, D1142:K1142)</f>
+        <v>03_Hieroglyphen-selten/N6B_nsw-bjt_01.png</v>
+      </c>
+    </row>
+    <row r="1143" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1143" s="4" t="s">
+        <v>1274</v>
+      </c>
+      <c r="B1143" s="27">
+        <v>1</v>
+      </c>
+      <c r="C1143" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1143" t="s">
+        <v>517</v>
+      </c>
+    </row>
+    <row r="1144" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1144" s="4" t="s">
+        <v>1274</v>
+      </c>
+      <c r="B1144" s="27">
+        <v>1</v>
+      </c>
+      <c r="C1144" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1144" t="s">
+        <v>1296</v>
+      </c>
+    </row>
+    <row r="1145" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1145" s="4" t="s">
+        <v>1274</v>
+      </c>
+      <c r="B1145" s="27">
         <v>2</v>
       </c>
-      <c r="C1135" t="s">
+      <c r="C1145" t="s">
+        <v>1292</v>
+      </c>
+      <c r="L1145" t="s">
+        <v>1298</v>
+      </c>
+    </row>
+    <row r="1146" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1146" s="4" t="s">
+        <v>1274</v>
+      </c>
+      <c r="B1146" s="27">
+        <v>2</v>
+      </c>
+      <c r="C1146" t="s">
+        <v>1235</v>
+      </c>
+      <c r="E1146" t="s">
+        <v>1289</v>
+      </c>
+      <c r="G1146" t="s">
+        <v>1297</v>
+      </c>
+      <c r="H1146" t="s">
+        <v>112</v>
+      </c>
+      <c r="L1146" t="str">
+        <f t="shared" ref="L1146" si="147">_xlfn.TEXTJOIN("", TRUE, D1146:K1146)</f>
+        <v>03_Hieroglyphen-selten/N102_jmn_01.png</v>
+      </c>
+    </row>
+    <row r="1147" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1147" s="4" t="s">
+        <v>1274</v>
+      </c>
+      <c r="B1147" s="27">
+        <v>2</v>
+      </c>
+      <c r="C1147" t="s">
+        <v>39</v>
+      </c>
+      <c r="L1147" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="1148" spans="1:12" x14ac:dyDescent="0.2">
+      <c r="A1148" s="4" t="s">
+        <v>1274</v>
+      </c>
+      <c r="B1148" s="27">
+        <v>2</v>
+      </c>
+      <c r="C1148" t="s">
         <v>27</v>
       </c>
-      <c r="L1135" t="s">
+      <c r="L1148" t="s">
         <v>111</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="L37 L994 L1004" formula="1"/>
+    <ignoredError sqref="L37 L1017 L971" formula="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
updated header order and appearance
</commit_message>
<xml_diff>
--- a/data/content.xlsx
+++ b/data/content.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Markus/Documents/Arbeit/Inschriftenschluessel/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{698C15F0-969D-BA40-9A5F-36B05D42CFAA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F041A75D-8A37-1C4F-9330-B224F2AD60D2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4880" yWindow="500" windowWidth="20220" windowHeight="16120" xr2:uid="{F025A444-F8B0-5C41-A37E-BEE791B22240}"/>
   </bookViews>
@@ -4880,7 +4880,7 @@
     <t>- Meulenaere, H. J. A. de 1997–2000. Sculptures mendésiennes de Basse Époque. Jaarbericht van het Vooraziatisch-Egyptisch Genootschap Ex Oriente Lux 35–36, 33–39: F. 81</t>
   </si>
   <si>
-    <t>"&amp;#32;"</t>
+    <t>Inschriftenschlüssel</t>
   </si>
 </sst>
 </file>

</xml_diff>